<commit_message>
Aggiunge 13 nuove agenzie immobiliari (Costa Smeralda, Cagliari, Sassari) e corregge bug foglio Riepilogo in genera_ref.py
- Lista_Contatti_Rilievo_Contract.xlsx: 42 architetti + 32 agenzie (19 esistenti + 13 nuove), ref verificati senza collisioni
- genera_ref.py: il giro CSV/XLSX -> XLSX faceva sparire il foglio Riepilogo (letto ma mai riscritto in output) — ora viene sempre rigenerato con i conteggi aggiornati
</commit_message>
<xml_diff>
--- a/Lista_Contatti_Rilievo_Contract.xlsx
+++ b/Lista_Contatti_Rilievo_Contract.xlsx
@@ -13,7 +13,7 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Architetti'!$A$1:$G$43</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Agenzie immobiliari'!$A$1:$G$20</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Agenzie immobiliari'!$A$1:$G$33</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -22,36 +22,13 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="9">
+  <fonts count="7">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
       <color theme="1"/>
       <sz val="11"/>
       <scheme val="minor"/>
-    </font>
-    <font>
-      <name val="Arial"/>
-      <b val="1"/>
-      <color rgb="00F8F5EF"/>
-      <sz val="11"/>
-    </font>
-    <font>
-      <name val="Arial"/>
-      <color rgb="001C1C1A"/>
-      <sz val="10"/>
-    </font>
-    <font>
-      <name val="Arial"/>
-      <color rgb="000563C1"/>
-      <sz val="10"/>
-      <u val="single"/>
-    </font>
-    <font>
-      <name val="Arial"/>
-      <b val="1"/>
-      <color rgb="008A4B00"/>
-      <sz val="10"/>
     </font>
     <font>
       <name val="Arial"/>
@@ -68,17 +45,28 @@
     <font>
       <name val="Arial"/>
       <b val="1"/>
+      <color rgb="00F8F5EF"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <name val="Arial"/>
       <color rgb="001C1C1A"/>
       <sz val="10"/>
     </font>
     <font>
       <name val="Arial"/>
-      <i val="1"/>
-      <color rgb="007A7A75"/>
-      <sz val="9"/>
+      <b val="1"/>
+      <color rgb="001C1C1A"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <color rgb="000563C1"/>
+      <sz val="10"/>
+      <u val="single"/>
     </font>
   </fonts>
-  <fills count="5">
+  <fills count="4">
     <fill>
       <patternFill/>
     </fill>
@@ -95,12 +83,6 @@
       <patternFill patternType="solid">
         <fgColor rgb="00F8F5EF"/>
         <bgColor rgb="00F8F5EF"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00FCE8D6"/>
-        <bgColor rgb="00FCE8D6"/>
       </patternFill>
     </fill>
   </fills>
@@ -130,38 +112,23 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="15">
+  <cellXfs count="10">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
   </cellXfs>
@@ -238,21 +205,6 @@
     </indexedColors>
   </colors>
 </styleSheet>
-</file>
-
-<file path=xl/comments/comment1.xml><?xml version="1.0" encoding="utf-8"?>
-<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <authors>
-    <author>Rilievo Contract</author>
-  </authors>
-  <commentList>
-    <comment ref="B25" authorId="0" shapeId="0">
-      <text>
-        <t>CONFERMATO 20/07/2026: l'email con ref e7f0f e' stata spedita per errore sia ad Ark.e Studio sia a Studio Figus. I dati GA4 per e7f0f nel periodo di sovrapposizione sono contaminati e non recuperabili. Nuovo ref casuale assegnato per l'uso futuro: consigliato reinvio a gianluca@studiofigus.it con il link corretto.</t>
-      </text>
-    </comment>
-  </commentList>
-</comments>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -544,7 +496,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B10"/>
+  <dimension ref="A1:B7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="34" customWidth="1" min="1" max="1"/>
@@ -594,7 +546,7 @@
         </is>
       </c>
       <c r="B6" s="4" t="n">
-        <v>19</v>
+        <v>32</v>
       </c>
     </row>
     <row r="7">
@@ -604,20 +556,12 @@
         </is>
       </c>
       <c r="B7" s="5" t="n">
-        <v>61</v>
-      </c>
-    </row>
-    <row r="10" ht="90" customHeight="1">
-      <c r="A10" s="6" t="inlineStr">
-        <is>
-          <t>Nota metodo: 22 architetti sui 42 hanno il ref gia' confermato dal generatore email attivo (intoccati). 19 architetti nuovi hanno ref deterministico md5(email)[:5], verificato senza collisioni. 1 riga (Studio Figus, evidenziata in arancione nella tab Architetti) aveva un ref duplicato di Ark.e Studio nella lista originale: le e' stato assegnato un ref provvisorio, da confermare se non e' gia' stato spedito via email con il codice errato. Le 19 agenzie immobiliari hanno ref nuovi, verificati contro tutti i 42 ref architetti: nessuna collisione.</t>
-        </is>
+        <v>74</v>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="3">
+  <mergeCells count="2">
     <mergeCell ref="A2:B2"/>
-    <mergeCell ref="A10:B10"/>
     <mergeCell ref="A1:B1"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -633,1527 +577,1527 @@
   <dimension ref="A1:G43"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="8" customWidth="1" min="1" max="1"/>
-    <col width="34" customWidth="1" min="2" max="2"/>
-    <col width="24" customWidth="1" min="3" max="3"/>
-    <col width="32" customWidth="1" min="4" max="4"/>
-    <col width="26" customWidth="1" min="5" max="5"/>
-    <col width="10" customWidth="1" min="6" max="6"/>
+    <col width="30" customWidth="1" min="1" max="1"/>
+    <col width="30" customWidth="1" min="2" max="2"/>
+    <col width="30" customWidth="1" min="3" max="3"/>
+    <col width="30" customWidth="1" min="4" max="4"/>
+    <col width="30" customWidth="1" min="5" max="5"/>
+    <col width="30" customWidth="1" min="6" max="6"/>
     <col width="52" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
-    <row r="1" ht="20" customHeight="1">
-      <c r="A1" s="7" t="inlineStr">
-        <is>
-          <t>ID</t>
-        </is>
-      </c>
-      <c r="B1" s="7" t="inlineStr">
+    <row r="1">
+      <c r="A1" s="3" t="inlineStr">
+        <is>
+          <t>Id</t>
+        </is>
+      </c>
+      <c r="B1" s="3" t="inlineStr">
         <is>
           <t>Nome</t>
         </is>
       </c>
-      <c r="C1" s="7" t="inlineStr">
-        <is>
-          <t>Città</t>
-        </is>
-      </c>
-      <c r="D1" s="7" t="inlineStr">
+      <c r="C1" s="3" t="inlineStr">
+        <is>
+          <t>Citta</t>
+        </is>
+      </c>
+      <c r="D1" s="3" t="inlineStr">
         <is>
           <t>Email</t>
         </is>
       </c>
-      <c r="E1" s="7" t="inlineStr">
+      <c r="E1" s="3" t="inlineStr">
         <is>
           <t>Categoria</t>
         </is>
       </c>
-      <c r="F1" s="7" t="inlineStr">
+      <c r="F1" s="3" t="inlineStr">
         <is>
           <t>Ref</t>
         </is>
       </c>
-      <c r="G1" s="7" t="inlineStr">
-        <is>
-          <t>Link presentazione</t>
+      <c r="G1" s="3" t="inlineStr">
+        <is>
+          <t>Link</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="8" t="inlineStr">
+      <c r="A2" s="6" t="inlineStr">
         <is>
           <t>1</t>
         </is>
       </c>
-      <c r="B2" s="8" t="inlineStr">
+      <c r="B2" s="6" t="inlineStr">
         <is>
           <t>C+C04 Architetti</t>
         </is>
       </c>
-      <c r="C2" s="8" t="inlineStr">
+      <c r="C2" s="6" t="inlineStr">
         <is>
           <t>Cagliari</t>
         </is>
       </c>
-      <c r="D2" s="8" t="inlineStr">
+      <c r="D2" s="6" t="inlineStr">
         <is>
           <t>info@cc04.net</t>
         </is>
       </c>
-      <c r="E2" s="8" t="inlineStr">
+      <c r="E2" s="6" t="inlineStr">
         <is>
           <t>Hotel, Ristoranti, Retail</t>
         </is>
       </c>
-      <c r="F2" s="8" t="inlineStr">
+      <c r="F2" s="6" t="inlineStr">
         <is>
           <t>8fa8d</t>
         </is>
       </c>
-      <c r="G2" s="9" t="inlineStr">
+      <c r="G2" s="7" t="inlineStr">
         <is>
           <t>https://presentazione.rilievocontract.it/?ref=8fa8d</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="10" t="inlineStr">
+      <c r="A3" s="8" t="inlineStr">
         <is>
           <t>2</t>
         </is>
       </c>
-      <c r="B3" s="10" t="inlineStr">
+      <c r="B3" s="8" t="inlineStr">
         <is>
           <t>ALO Architettura</t>
         </is>
       </c>
-      <c r="C3" s="10" t="inlineStr">
+      <c r="C3" s="8" t="inlineStr">
         <is>
           <t>Cagliari</t>
         </is>
       </c>
-      <c r="D3" s="10" t="inlineStr">
+      <c r="D3" s="8" t="inlineStr">
         <is>
           <t>info@alo-architettura.com</t>
         </is>
       </c>
-      <c r="E3" s="10" t="inlineStr">
+      <c r="E3" s="8" t="inlineStr">
         <is>
           <t>Ricettivo, Retail, Ville</t>
         </is>
       </c>
-      <c r="F3" s="10" t="inlineStr">
+      <c r="F3" s="8" t="inlineStr">
         <is>
           <t>cf458</t>
         </is>
       </c>
-      <c r="G3" s="11" t="inlineStr">
+      <c r="G3" s="9" t="inlineStr">
         <is>
           <t>https://presentazione.rilievocontract.it/?ref=cf458</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="8" t="inlineStr">
+      <c r="A4" s="6" t="inlineStr">
         <is>
           <t>3</t>
         </is>
       </c>
-      <c r="B4" s="8" t="inlineStr">
+      <c r="B4" s="6" t="inlineStr">
         <is>
           <t>Studio Tramas</t>
         </is>
       </c>
-      <c r="C4" s="8" t="inlineStr">
+      <c r="C4" s="6" t="inlineStr">
         <is>
           <t>Cagliari</t>
         </is>
       </c>
-      <c r="D4" s="8" t="inlineStr">
+      <c r="D4" s="6" t="inlineStr">
         <is>
           <t>info@studiotramas.com</t>
         </is>
       </c>
-      <c r="E4" s="8" t="inlineStr">
+      <c r="E4" s="6" t="inlineStr">
         <is>
           <t>Ricettivo, Retail, Interior</t>
         </is>
       </c>
-      <c r="F4" s="8" t="inlineStr">
+      <c r="F4" s="6" t="inlineStr">
         <is>
           <t>04cb2</t>
         </is>
       </c>
-      <c r="G4" s="9" t="inlineStr">
+      <c r="G4" s="7" t="inlineStr">
         <is>
           <t>https://presentazione.rilievocontract.it/?ref=04cb2</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="10" t="inlineStr">
+      <c r="A5" s="8" t="inlineStr">
         <is>
           <t>4</t>
         </is>
       </c>
-      <c r="B5" s="10" t="inlineStr">
+      <c r="B5" s="8" t="inlineStr">
         <is>
           <t>MUCA Architettura</t>
         </is>
       </c>
-      <c r="C5" s="10" t="inlineStr">
+      <c r="C5" s="8" t="inlineStr">
         <is>
           <t>Cagliari</t>
         </is>
       </c>
-      <c r="D5" s="10" t="inlineStr">
+      <c r="D5" s="8" t="inlineStr">
         <is>
           <t>info@mucaarchitettura.com</t>
         </is>
       </c>
-      <c r="E5" s="10" t="inlineStr">
+      <c r="E5" s="8" t="inlineStr">
         <is>
           <t>Retail, Exhibit</t>
         </is>
       </c>
-      <c r="F5" s="10" t="inlineStr">
+      <c r="F5" s="8" t="inlineStr">
         <is>
           <t>e28a2</t>
         </is>
       </c>
-      <c r="G5" s="11" t="inlineStr">
+      <c r="G5" s="9" t="inlineStr">
         <is>
           <t>https://presentazione.rilievocontract.it/?ref=e28a2</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="8" t="inlineStr">
+      <c r="A6" s="6" t="inlineStr">
         <is>
           <t>5</t>
         </is>
       </c>
-      <c r="B6" s="8" t="inlineStr">
+      <c r="B6" s="6" t="inlineStr">
         <is>
           <t>essequadro|p</t>
         </is>
       </c>
-      <c r="C6" s="8" t="inlineStr">
+      <c r="C6" s="6" t="inlineStr">
         <is>
           <t>Cagliari</t>
         </is>
       </c>
-      <c r="D6" s="8" t="inlineStr">
+      <c r="D6" s="6" t="inlineStr">
         <is>
           <t>info@essequadrop.com</t>
         </is>
       </c>
-      <c r="E6" s="8" t="inlineStr">
+      <c r="E6" s="6" t="inlineStr">
         <is>
           <t>Hospitality, Lighting</t>
         </is>
       </c>
-      <c r="F6" s="8" t="inlineStr">
+      <c r="F6" s="6" t="inlineStr">
         <is>
           <t>0a85e</t>
         </is>
       </c>
-      <c r="G6" s="9" t="inlineStr">
+      <c r="G6" s="7" t="inlineStr">
         <is>
           <t>https://presentazione.rilievocontract.it/?ref=0a85e</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="10" t="inlineStr">
+      <c r="A7" s="8" t="inlineStr">
         <is>
           <t>6</t>
         </is>
       </c>
-      <c r="B7" s="10" t="inlineStr">
+      <c r="B7" s="8" t="inlineStr">
         <is>
           <t>Formaa Studio</t>
         </is>
       </c>
-      <c r="C7" s="10" t="inlineStr">
+      <c r="C7" s="8" t="inlineStr">
         <is>
           <t>Cagliari</t>
         </is>
       </c>
-      <c r="D7" s="10" t="inlineStr">
+      <c r="D7" s="8" t="inlineStr">
         <is>
           <t>info@formaa.it</t>
         </is>
       </c>
-      <c r="E7" s="10" t="inlineStr">
+      <c r="E7" s="8" t="inlineStr">
         <is>
           <t>Ricettivo, Locali</t>
         </is>
       </c>
-      <c r="F7" s="10" t="inlineStr">
+      <c r="F7" s="8" t="inlineStr">
         <is>
           <t>f815c</t>
         </is>
       </c>
-      <c r="G7" s="11" t="inlineStr">
+      <c r="G7" s="9" t="inlineStr">
         <is>
           <t>https://presentazione.rilievocontract.it/?ref=f815c</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="8" t="inlineStr">
+      <c r="A8" s="6" t="inlineStr">
         <is>
           <t>7</t>
         </is>
       </c>
-      <c r="B8" s="8" t="inlineStr">
+      <c r="B8" s="6" t="inlineStr">
         <is>
           <t>Orma Studio</t>
         </is>
       </c>
-      <c r="C8" s="8" t="inlineStr">
+      <c r="C8" s="6" t="inlineStr">
         <is>
           <t>Cagliari</t>
         </is>
       </c>
-      <c r="D8" s="8" t="inlineStr">
+      <c r="D8" s="6" t="inlineStr">
         <is>
           <t>info@ormastudio.it</t>
         </is>
       </c>
-      <c r="E8" s="8" t="inlineStr">
+      <c r="E8" s="6" t="inlineStr">
         <is>
           <t>Commerciale, Interior</t>
         </is>
       </c>
-      <c r="F8" s="8" t="inlineStr">
+      <c r="F8" s="6" t="inlineStr">
         <is>
           <t>4d5d7</t>
         </is>
       </c>
-      <c r="G8" s="9" t="inlineStr">
+      <c r="G8" s="7" t="inlineStr">
         <is>
           <t>https://presentazione.rilievocontract.it/?ref=4d5d7</t>
         </is>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="10" t="inlineStr">
+      <c r="A9" s="8" t="inlineStr">
         <is>
           <t>9</t>
         </is>
       </c>
-      <c r="B9" s="10" t="inlineStr">
+      <c r="B9" s="8" t="inlineStr">
         <is>
           <t>Studio Rifinito — Lara Serra</t>
         </is>
       </c>
-      <c r="C9" s="10" t="inlineStr">
+      <c r="C9" s="8" t="inlineStr">
         <is>
           <t>Cagliari</t>
         </is>
       </c>
-      <c r="D9" s="10" t="inlineStr">
+      <c r="D9" s="8" t="inlineStr">
         <is>
           <t>info@studiorifinito.it</t>
         </is>
       </c>
-      <c r="E9" s="10" t="inlineStr">
+      <c r="E9" s="8" t="inlineStr">
         <is>
           <t>Interior, Residenziale</t>
         </is>
       </c>
-      <c r="F9" s="10" t="inlineStr">
+      <c r="F9" s="8" t="inlineStr">
         <is>
           <t>dc232</t>
         </is>
       </c>
-      <c r="G9" s="11" t="inlineStr">
+      <c r="G9" s="9" t="inlineStr">
         <is>
           <t>https://presentazione.rilievocontract.it/?ref=dc232</t>
         </is>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="8" t="inlineStr">
+      <c r="A10" s="6" t="inlineStr">
         <is>
           <t>10</t>
         </is>
       </c>
-      <c r="B10" s="8" t="inlineStr">
+      <c r="B10" s="6" t="inlineStr">
         <is>
           <t>domECO Studio</t>
         </is>
       </c>
-      <c r="C10" s="8" t="inlineStr">
+      <c r="C10" s="6" t="inlineStr">
         <is>
           <t>Cagliari / Sassari</t>
         </is>
       </c>
-      <c r="D10" s="8" t="inlineStr">
+      <c r="D10" s="6" t="inlineStr">
         <is>
           <t>info@domecostudio.it</t>
         </is>
       </c>
-      <c r="E10" s="8" t="inlineStr">
+      <c r="E10" s="6" t="inlineStr">
         <is>
           <t>Residenziale, Interior</t>
         </is>
       </c>
-      <c r="F10" s="8" t="inlineStr">
+      <c r="F10" s="6" t="inlineStr">
         <is>
           <t>53775</t>
         </is>
       </c>
-      <c r="G10" s="9" t="inlineStr">
+      <c r="G10" s="7" t="inlineStr">
         <is>
           <t>https://presentazione.rilievocontract.it/?ref=53775</t>
         </is>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="10" t="inlineStr">
+      <c r="A11" s="8" t="inlineStr">
         <is>
           <t>21</t>
         </is>
       </c>
-      <c r="B11" s="10" t="inlineStr">
+      <c r="B11" s="8" t="inlineStr">
         <is>
           <t>Studio Careddu</t>
         </is>
       </c>
-      <c r="C11" s="10" t="inlineStr">
+      <c r="C11" s="8" t="inlineStr">
         <is>
           <t>Olbia / Costa Smeralda</t>
         </is>
       </c>
-      <c r="D11" s="10" t="inlineStr">
+      <c r="D11" s="8" t="inlineStr">
         <is>
           <t>info@architettocareddu.it</t>
         </is>
       </c>
-      <c r="E11" s="10" t="inlineStr">
+      <c r="E11" s="8" t="inlineStr">
         <is>
           <t>Ville pregio, Ricettivo</t>
         </is>
       </c>
-      <c r="F11" s="10" t="inlineStr">
+      <c r="F11" s="8" t="inlineStr">
         <is>
           <t>7c83b</t>
         </is>
       </c>
-      <c r="G11" s="11" t="inlineStr">
+      <c r="G11" s="9" t="inlineStr">
         <is>
           <t>https://presentazione.rilievocontract.it/?ref=7c83b</t>
         </is>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="8" t="inlineStr">
+      <c r="A12" s="6" t="inlineStr">
         <is>
           <t>22</t>
         </is>
       </c>
-      <c r="B12" s="8" t="inlineStr">
+      <c r="B12" s="6" t="inlineStr">
         <is>
           <t>Marcello Scano Interior Design</t>
         </is>
       </c>
-      <c r="C12" s="8" t="inlineStr">
+      <c r="C12" s="6" t="inlineStr">
         <is>
           <t>Olbia</t>
         </is>
       </c>
-      <c r="D12" s="8" t="inlineStr">
+      <c r="D12" s="6" t="inlineStr">
         <is>
           <t>info@marcelloscano.it</t>
         </is>
       </c>
-      <c r="E12" s="8" t="inlineStr">
+      <c r="E12" s="6" t="inlineStr">
         <is>
           <t>Hospitality, Ville</t>
         </is>
       </c>
-      <c r="F12" s="8" t="inlineStr">
+      <c r="F12" s="6" t="inlineStr">
         <is>
           <t>90a53</t>
         </is>
       </c>
-      <c r="G12" s="9" t="inlineStr">
+      <c r="G12" s="7" t="inlineStr">
         <is>
           <t>https://presentazione.rilievocontract.it/?ref=90a53</t>
         </is>
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="10" t="inlineStr">
+      <c r="A13" s="8" t="inlineStr">
         <is>
           <t>23</t>
         </is>
       </c>
-      <c r="B13" s="10" t="inlineStr">
+      <c r="B13" s="8" t="inlineStr">
         <is>
           <t>Antonello Carta Interior Design</t>
         </is>
       </c>
-      <c r="C13" s="10" t="inlineStr">
+      <c r="C13" s="8" t="inlineStr">
         <is>
           <t>Olbia</t>
         </is>
       </c>
-      <c r="D13" s="10" t="inlineStr">
+      <c r="D13" s="8" t="inlineStr">
         <is>
           <t>info@antonellocarta.com</t>
         </is>
       </c>
-      <c r="E13" s="10" t="inlineStr">
+      <c r="E13" s="8" t="inlineStr">
         <is>
           <t>Ristoranti, Retail</t>
         </is>
       </c>
-      <c r="F13" s="10" t="inlineStr">
+      <c r="F13" s="8" t="inlineStr">
         <is>
           <t>aa5ba</t>
         </is>
       </c>
-      <c r="G13" s="11" t="inlineStr">
+      <c r="G13" s="9" t="inlineStr">
         <is>
           <t>https://presentazione.rilievocontract.it/?ref=aa5ba</t>
         </is>
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="8" t="inlineStr">
+      <c r="A14" s="6" t="inlineStr">
         <is>
           <t>24</t>
         </is>
       </c>
-      <c r="B14" s="8" t="inlineStr">
+      <c r="B14" s="6" t="inlineStr">
         <is>
           <t>Studio Miniaci e Associati</t>
         </is>
       </c>
-      <c r="C14" s="8" t="inlineStr">
+      <c r="C14" s="6" t="inlineStr">
         <is>
           <t>Olbia / Costa Smeralda</t>
         </is>
       </c>
-      <c r="D14" s="8" t="inlineStr">
+      <c r="D14" s="6" t="inlineStr">
         <is>
           <t>info@architettimea.it</t>
         </is>
       </c>
-      <c r="E14" s="8" t="inlineStr">
+      <c r="E14" s="6" t="inlineStr">
         <is>
           <t>Hospitality, Residenziale</t>
         </is>
       </c>
-      <c r="F14" s="8" t="inlineStr">
+      <c r="F14" s="6" t="inlineStr">
         <is>
           <t>7b647</t>
         </is>
       </c>
-      <c r="G14" s="9" t="inlineStr">
+      <c r="G14" s="7" t="inlineStr">
         <is>
           <t>https://presentazione.rilievocontract.it/?ref=7b647</t>
         </is>
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="10" t="inlineStr">
+      <c r="A15" s="8" t="inlineStr">
         <is>
           <t>25</t>
         </is>
       </c>
-      <c r="B15" s="10" t="inlineStr">
+      <c r="B15" s="8" t="inlineStr">
         <is>
           <t>FabDesign Interiors</t>
         </is>
       </c>
-      <c r="C15" s="10" t="inlineStr">
+      <c r="C15" s="8" t="inlineStr">
         <is>
           <t>Olbia</t>
         </is>
       </c>
-      <c r="D15" s="10" t="inlineStr">
+      <c r="D15" s="8" t="inlineStr">
         <is>
           <t>info@fabdesigninteriors.com</t>
         </is>
       </c>
-      <c r="E15" s="10" t="inlineStr">
+      <c r="E15" s="8" t="inlineStr">
         <is>
           <t>Bar/Ristoranti, Retail</t>
         </is>
       </c>
-      <c r="F15" s="10" t="inlineStr">
+      <c r="F15" s="8" t="inlineStr">
         <is>
           <t>7b3cb</t>
         </is>
       </c>
-      <c r="G15" s="11" t="inlineStr">
+      <c r="G15" s="9" t="inlineStr">
         <is>
           <t>https://presentazione.rilievocontract.it/?ref=7b3cb</t>
         </is>
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="8" t="inlineStr">
+      <c r="A16" s="6" t="inlineStr">
         <is>
           <t>26</t>
         </is>
       </c>
-      <c r="B16" s="8" t="inlineStr">
+      <c r="B16" s="6" t="inlineStr">
         <is>
           <t>Studio Olivieri Architetti</t>
         </is>
       </c>
-      <c r="C16" s="8" t="inlineStr">
+      <c r="C16" s="6" t="inlineStr">
         <is>
           <t>Arzachena / Costa Smeralda</t>
         </is>
       </c>
-      <c r="D16" s="8" t="inlineStr">
+      <c r="D16" s="6" t="inlineStr">
         <is>
           <t>info@olivieriarchitetti.it</t>
         </is>
       </c>
-      <c r="E16" s="8" t="inlineStr">
+      <c r="E16" s="6" t="inlineStr">
         <is>
           <t>Ville lusso, Ricettivo</t>
         </is>
       </c>
-      <c r="F16" s="8" t="inlineStr">
+      <c r="F16" s="6" t="inlineStr">
         <is>
           <t>99814</t>
         </is>
       </c>
-      <c r="G16" s="9" t="inlineStr">
+      <c r="G16" s="7" t="inlineStr">
         <is>
           <t>https://presentazione.rilievocontract.it/?ref=99814</t>
         </is>
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="10" t="inlineStr">
+      <c r="A17" s="8" t="inlineStr">
         <is>
           <t>28</t>
         </is>
       </c>
-      <c r="B17" s="10" t="inlineStr">
+      <c r="B17" s="8" t="inlineStr">
         <is>
           <t>Pitzus Group</t>
         </is>
       </c>
-      <c r="C17" s="10" t="inlineStr">
+      <c r="C17" s="8" t="inlineStr">
         <is>
           <t>Costa Smeralda</t>
         </is>
       </c>
-      <c r="D17" s="10" t="inlineStr">
+      <c r="D17" s="8" t="inlineStr">
         <is>
           <t>info@pitzusgroup.com</t>
         </is>
       </c>
-      <c r="E17" s="10" t="inlineStr">
+      <c r="E17" s="8" t="inlineStr">
         <is>
           <t>Ville lusso</t>
         </is>
       </c>
-      <c r="F17" s="10" t="inlineStr">
+      <c r="F17" s="8" t="inlineStr">
         <is>
           <t>3b50d</t>
         </is>
       </c>
-      <c r="G17" s="11" t="inlineStr">
+      <c r="G17" s="9" t="inlineStr">
         <is>
           <t>https://presentazione.rilievocontract.it/?ref=3b50d</t>
         </is>
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="8" t="inlineStr">
+      <c r="A18" s="6" t="inlineStr">
         <is>
           <t>29</t>
         </is>
       </c>
-      <c r="B18" s="8" t="inlineStr">
+      <c r="B18" s="6" t="inlineStr">
         <is>
           <t>Architettare &amp; Design Srl</t>
         </is>
       </c>
-      <c r="C18" s="8" t="inlineStr">
+      <c r="C18" s="6" t="inlineStr">
         <is>
           <t>Olbia</t>
         </is>
       </c>
-      <c r="D18" s="8" t="inlineStr">
+      <c r="D18" s="6" t="inlineStr">
         <is>
           <t>info@architettaredesignsrl.it</t>
         </is>
       </c>
-      <c r="E18" s="8" t="inlineStr">
+      <c r="E18" s="6" t="inlineStr">
         <is>
           <t>Costa Smeralda, Ville</t>
         </is>
       </c>
-      <c r="F18" s="8" t="inlineStr">
+      <c r="F18" s="6" t="inlineStr">
         <is>
           <t>60531</t>
         </is>
       </c>
-      <c r="G18" s="9" t="inlineStr">
+      <c r="G18" s="7" t="inlineStr">
         <is>
           <t>https://presentazione.rilievocontract.it/?ref=60531</t>
         </is>
       </c>
     </row>
     <row r="19">
-      <c r="A19" s="10" t="inlineStr">
+      <c r="A19" s="8" t="inlineStr">
         <is>
           <t>31</t>
         </is>
       </c>
-      <c r="B19" s="10" t="inlineStr">
+      <c r="B19" s="8" t="inlineStr">
         <is>
           <t>Studio Arch. Pietro Giordo</t>
         </is>
       </c>
-      <c r="C19" s="10" t="inlineStr">
+      <c r="C19" s="8" t="inlineStr">
         <is>
           <t>Arzachena / Porto Cervo</t>
         </is>
       </c>
-      <c r="D19" s="10" t="inlineStr">
+      <c r="D19" s="8" t="inlineStr">
         <is>
           <t>info@pietrogiordo.it</t>
         </is>
       </c>
-      <c r="E19" s="10" t="inlineStr">
+      <c r="E19" s="8" t="inlineStr">
         <is>
           <t>Ville storiche, Ricettivo</t>
         </is>
       </c>
-      <c r="F19" s="10" t="inlineStr">
+      <c r="F19" s="8" t="inlineStr">
         <is>
           <t>8a2a4</t>
         </is>
       </c>
-      <c r="G19" s="11" t="inlineStr">
+      <c r="G19" s="9" t="inlineStr">
         <is>
           <t>https://presentazione.rilievocontract.it/?ref=8a2a4</t>
         </is>
       </c>
     </row>
     <row r="20">
-      <c r="A20" s="8" t="inlineStr">
+      <c r="A20" s="6" t="inlineStr">
         <is>
           <t>34</t>
         </is>
       </c>
-      <c r="B20" s="8" t="inlineStr">
+      <c r="B20" s="6" t="inlineStr">
         <is>
           <t>Officina29 Architetti</t>
         </is>
       </c>
-      <c r="C20" s="8" t="inlineStr">
+      <c r="C20" s="6" t="inlineStr">
         <is>
           <t>Sassari / Olbia</t>
         </is>
       </c>
-      <c r="D20" s="8" t="inlineStr">
+      <c r="D20" s="6" t="inlineStr">
         <is>
           <t>info@officina29architetti.it</t>
         </is>
       </c>
-      <c r="E20" s="8" t="inlineStr">
+      <c r="E20" s="6" t="inlineStr">
         <is>
           <t>Interior, Residenziale</t>
         </is>
       </c>
-      <c r="F20" s="8" t="inlineStr">
+      <c r="F20" s="6" t="inlineStr">
         <is>
           <t>82701</t>
         </is>
       </c>
-      <c r="G20" s="9" t="inlineStr">
+      <c r="G20" s="7" t="inlineStr">
         <is>
           <t>https://presentazione.rilievocontract.it/?ref=82701</t>
         </is>
       </c>
     </row>
     <row r="21">
-      <c r="A21" s="10" t="inlineStr">
+      <c r="A21" s="8" t="inlineStr">
         <is>
           <t>37</t>
         </is>
       </c>
-      <c r="B21" s="10" t="inlineStr">
+      <c r="B21" s="8" t="inlineStr">
         <is>
           <t>ADM Progetti</t>
         </is>
       </c>
-      <c r="C21" s="10" t="inlineStr">
+      <c r="C21" s="8" t="inlineStr">
         <is>
           <t>Sassari</t>
         </is>
       </c>
-      <c r="D21" s="10" t="inlineStr">
+      <c r="D21" s="8" t="inlineStr">
         <is>
           <t>info@admprogetti.it</t>
         </is>
       </c>
-      <c r="E21" s="10" t="inlineStr">
+      <c r="E21" s="8" t="inlineStr">
         <is>
           <t>Residenziale, Commerciale</t>
         </is>
       </c>
-      <c r="F21" s="10" t="inlineStr">
+      <c r="F21" s="8" t="inlineStr">
         <is>
           <t>4959f</t>
         </is>
       </c>
-      <c r="G21" s="11" t="inlineStr">
+      <c r="G21" s="9" t="inlineStr">
         <is>
           <t>https://presentazione.rilievocontract.it/?ref=4959f</t>
         </is>
       </c>
     </row>
     <row r="22">
-      <c r="A22" s="8" t="inlineStr">
+      <c r="A22" s="6" t="inlineStr">
         <is>
           <t>38</t>
         </is>
       </c>
-      <c r="B22" s="8" t="inlineStr">
+      <c r="B22" s="6" t="inlineStr">
         <is>
           <t>Studio Cartamantiglia</t>
         </is>
       </c>
-      <c r="C22" s="8" t="inlineStr">
+      <c r="C22" s="6" t="inlineStr">
         <is>
           <t>Alghero</t>
         </is>
       </c>
-      <c r="D22" s="8" t="inlineStr">
+      <c r="D22" s="6" t="inlineStr">
         <is>
           <t>info@federicocartamantiglia.com</t>
         </is>
       </c>
-      <c r="E22" s="8" t="inlineStr">
+      <c r="E22" s="6" t="inlineStr">
         <is>
           <t>Hotel, Beach bar, Retail</t>
         </is>
       </c>
-      <c r="F22" s="8" t="inlineStr">
+      <c r="F22" s="6" t="inlineStr">
         <is>
           <t>80ed1</t>
         </is>
       </c>
-      <c r="G22" s="9" t="inlineStr">
+      <c r="G22" s="7" t="inlineStr">
         <is>
           <t>https://presentazione.rilievocontract.it/?ref=80ed1</t>
         </is>
       </c>
     </row>
     <row r="23">
-      <c r="A23" s="10" t="inlineStr">
+      <c r="A23" s="8" t="inlineStr">
         <is>
           <t>39</t>
         </is>
       </c>
-      <c r="B23" s="10" t="inlineStr">
+      <c r="B23" s="8" t="inlineStr">
         <is>
           <t>DESINNU Studio</t>
         </is>
       </c>
-      <c r="C23" s="10" t="inlineStr">
+      <c r="C23" s="8" t="inlineStr">
         <is>
           <t>Alghero</t>
         </is>
       </c>
-      <c r="D23" s="10" t="inlineStr">
+      <c r="D23" s="8" t="inlineStr">
         <is>
           <t>info@architettura-alghero.it</t>
         </is>
       </c>
-      <c r="E23" s="10" t="inlineStr">
+      <c r="E23" s="8" t="inlineStr">
         <is>
           <t>Commerciale, Residenziale</t>
         </is>
       </c>
-      <c r="F23" s="10" t="inlineStr">
+      <c r="F23" s="8" t="inlineStr">
         <is>
           <t>0b9cc</t>
         </is>
       </c>
-      <c r="G23" s="11" t="inlineStr">
+      <c r="G23" s="9" t="inlineStr">
         <is>
           <t>https://presentazione.rilievocontract.it/?ref=0b9cc</t>
         </is>
       </c>
     </row>
     <row r="24">
-      <c r="A24" s="8" t="inlineStr">
+      <c r="A24" s="6" t="inlineStr">
         <is>
           <t>40</t>
         </is>
       </c>
-      <c r="B24" s="8" t="inlineStr">
+      <c r="B24" s="6" t="inlineStr">
         <is>
           <t>Ark.e Studio</t>
         </is>
       </c>
-      <c r="C24" s="8" t="inlineStr">
+      <c r="C24" s="6" t="inlineStr">
         <is>
           <t>Alghero</t>
         </is>
       </c>
-      <c r="D24" s="8" t="inlineStr">
+      <c r="D24" s="6" t="inlineStr">
         <is>
           <t>info@arkestudio.eu</t>
         </is>
       </c>
-      <c r="E24" s="8" t="inlineStr">
+      <c r="E24" s="6" t="inlineStr">
         <is>
           <t>Residenziale, Ricettivo</t>
         </is>
       </c>
-      <c r="F24" s="8" t="inlineStr">
+      <c r="F24" s="6" t="inlineStr">
         <is>
           <t>e7f0f</t>
         </is>
       </c>
-      <c r="G24" s="9" t="inlineStr">
+      <c r="G24" s="7" t="inlineStr">
         <is>
           <t>https://presentazione.rilievocontract.it/?ref=e7f0f</t>
         </is>
       </c>
     </row>
     <row r="25">
-      <c r="A25" s="12" t="inlineStr">
+      <c r="A25" s="8" t="inlineStr">
         <is>
           <t>100</t>
         </is>
       </c>
-      <c r="B25" s="12" t="inlineStr">
+      <c r="B25" s="8" t="inlineStr">
         <is>
           <t>Studio Figus</t>
         </is>
       </c>
-      <c r="C25" s="12" t="inlineStr"/>
-      <c r="D25" s="12" t="inlineStr">
+      <c r="C25" s="8" t="inlineStr"/>
+      <c r="D25" s="8" t="inlineStr">
         <is>
           <t>gianluca@studiofigus.it</t>
         </is>
       </c>
-      <c r="E25" s="12" t="inlineStr">
+      <c r="E25" s="8" t="inlineStr">
         <is>
           <t>Architetto</t>
         </is>
       </c>
-      <c r="F25" s="13" t="inlineStr">
+      <c r="F25" s="8" t="inlineStr">
         <is>
           <t>4e268</t>
         </is>
       </c>
-      <c r="G25" s="14" t="inlineStr">
-        <is>
-          <t>https://collaboratori.rilievocontract.it/?ref=4e268</t>
+      <c r="G25" s="9" t="inlineStr">
+        <is>
+          <t>https://presentazione.rilievocontract.it/?ref=4e268</t>
         </is>
       </c>
     </row>
     <row r="26">
-      <c r="A26" s="8" t="inlineStr">
+      <c r="A26" s="6" t="inlineStr">
         <is>
           <t>101</t>
         </is>
       </c>
-      <c r="B26" s="8" t="inlineStr">
+      <c r="B26" s="6" t="inlineStr">
         <is>
           <t>Arch. Davide Fancello</t>
         </is>
       </c>
-      <c r="C26" s="8" t="inlineStr"/>
-      <c r="D26" s="8" t="inlineStr">
+      <c r="C26" s="6" t="inlineStr"/>
+      <c r="D26" s="6" t="inlineStr">
         <is>
           <t>info@davidefancello.it</t>
         </is>
       </c>
-      <c r="E26" s="8" t="inlineStr">
+      <c r="E26" s="6" t="inlineStr">
         <is>
           <t>Architetto</t>
         </is>
       </c>
-      <c r="F26" s="8" t="inlineStr">
+      <c r="F26" s="6" t="inlineStr">
         <is>
           <t>d59d8</t>
         </is>
       </c>
-      <c r="G26" s="9" t="inlineStr">
-        <is>
-          <t>https://collaboratori.rilievocontract.it/?ref=d59d8</t>
+      <c r="G26" s="7" t="inlineStr">
+        <is>
+          <t>https://presentazione.rilievocontract.it/?ref=d59d8</t>
         </is>
       </c>
     </row>
     <row r="27">
-      <c r="A27" s="10" t="inlineStr">
+      <c r="A27" s="8" t="inlineStr">
         <is>
           <t>102</t>
         </is>
       </c>
-      <c r="B27" s="10" t="inlineStr">
+      <c r="B27" s="8" t="inlineStr">
         <is>
           <t>Studio Arch. Colomo</t>
         </is>
       </c>
-      <c r="C27" s="10" t="inlineStr"/>
-      <c r="D27" s="10" t="inlineStr">
+      <c r="C27" s="8" t="inlineStr"/>
+      <c r="D27" s="8" t="inlineStr">
         <is>
           <t>virgilio.colomo@gmail.com</t>
         </is>
       </c>
-      <c r="E27" s="10" t="inlineStr">
+      <c r="E27" s="8" t="inlineStr">
         <is>
           <t>Architetto</t>
         </is>
       </c>
-      <c r="F27" s="10" t="inlineStr">
+      <c r="F27" s="8" t="inlineStr">
         <is>
           <t>c25f9</t>
         </is>
       </c>
-      <c r="G27" s="11" t="inlineStr">
-        <is>
-          <t>https://collaboratori.rilievocontract.it/?ref=c25f9</t>
+      <c r="G27" s="9" t="inlineStr">
+        <is>
+          <t>https://presentazione.rilievocontract.it/?ref=c25f9</t>
         </is>
       </c>
     </row>
     <row r="28">
-      <c r="A28" s="8" t="inlineStr">
+      <c r="A28" s="6" t="inlineStr">
         <is>
           <t>103</t>
         </is>
       </c>
-      <c r="B28" s="8" t="inlineStr">
+      <c r="B28" s="6" t="inlineStr">
         <is>
           <t>Studio Ing. Floridu Stefano</t>
         </is>
       </c>
-      <c r="C28" s="8" t="inlineStr"/>
-      <c r="D28" s="8" t="inlineStr">
+      <c r="C28" s="6" t="inlineStr"/>
+      <c r="D28" s="6" t="inlineStr">
         <is>
           <t>info@floridiastudio.com</t>
         </is>
       </c>
-      <c r="E28" s="8" t="inlineStr">
+      <c r="E28" s="6" t="inlineStr">
         <is>
           <t>Architetto</t>
         </is>
       </c>
-      <c r="F28" s="8" t="inlineStr">
+      <c r="F28" s="6" t="inlineStr">
         <is>
           <t>cd24d</t>
         </is>
       </c>
-      <c r="G28" s="9" t="inlineStr">
-        <is>
-          <t>https://collaboratori.rilievocontract.it/?ref=cd24d</t>
+      <c r="G28" s="7" t="inlineStr">
+        <is>
+          <t>https://presentazione.rilievocontract.it/?ref=cd24d</t>
         </is>
       </c>
     </row>
     <row r="29">
-      <c r="A29" s="10" t="inlineStr">
+      <c r="A29" s="8" t="inlineStr">
         <is>
           <t>104</t>
         </is>
       </c>
-      <c r="B29" s="10" t="inlineStr">
+      <c r="B29" s="8" t="inlineStr">
         <is>
           <t>Studio Arch. Soru Giovanni</t>
         </is>
       </c>
-      <c r="C29" s="10" t="inlineStr"/>
-      <c r="D29" s="10" t="inlineStr">
+      <c r="C29" s="8" t="inlineStr"/>
+      <c r="D29" s="8" t="inlineStr">
         <is>
           <t>archsoru@gmail.com</t>
         </is>
       </c>
-      <c r="E29" s="10" t="inlineStr">
+      <c r="E29" s="8" t="inlineStr">
         <is>
           <t>Architetto</t>
         </is>
       </c>
-      <c r="F29" s="10" t="inlineStr">
+      <c r="F29" s="8" t="inlineStr">
         <is>
           <t>62279</t>
         </is>
       </c>
-      <c r="G29" s="11" t="inlineStr">
-        <is>
-          <t>https://collaboratori.rilievocontract.it/?ref=62279</t>
+      <c r="G29" s="9" t="inlineStr">
+        <is>
+          <t>https://presentazione.rilievocontract.it/?ref=62279</t>
         </is>
       </c>
     </row>
     <row r="30">
-      <c r="A30" s="8" t="inlineStr">
+      <c r="A30" s="6" t="inlineStr">
         <is>
           <t>105</t>
         </is>
       </c>
-      <c r="B30" s="8" t="inlineStr">
+      <c r="B30" s="6" t="inlineStr">
         <is>
           <t>FASE Architettura</t>
         </is>
       </c>
-      <c r="C30" s="8" t="inlineStr"/>
-      <c r="D30" s="8" t="inlineStr">
+      <c r="C30" s="6" t="inlineStr"/>
+      <c r="D30" s="6" t="inlineStr">
         <is>
           <t>fasearchitettura@gmail.com</t>
         </is>
       </c>
-      <c r="E30" s="8" t="inlineStr">
+      <c r="E30" s="6" t="inlineStr">
         <is>
           <t>Architetto</t>
         </is>
       </c>
-      <c r="F30" s="8" t="inlineStr">
+      <c r="F30" s="6" t="inlineStr">
         <is>
           <t>4cde0</t>
         </is>
       </c>
-      <c r="G30" s="9" t="inlineStr">
-        <is>
-          <t>https://collaboratori.rilievocontract.it/?ref=4cde0</t>
+      <c r="G30" s="7" t="inlineStr">
+        <is>
+          <t>https://presentazione.rilievocontract.it/?ref=4cde0</t>
         </is>
       </c>
     </row>
     <row r="31">
-      <c r="A31" s="10" t="inlineStr">
+      <c r="A31" s="8" t="inlineStr">
         <is>
           <t>106</t>
         </is>
       </c>
-      <c r="B31" s="10" t="inlineStr">
+      <c r="B31" s="8" t="inlineStr">
         <is>
           <t>De signIS Studio</t>
         </is>
       </c>
-      <c r="C31" s="10" t="inlineStr"/>
-      <c r="D31" s="10" t="inlineStr">
+      <c r="C31" s="8" t="inlineStr"/>
+      <c r="D31" s="8" t="inlineStr">
         <is>
           <t>laura.designis@gmail.com</t>
         </is>
       </c>
-      <c r="E31" s="10" t="inlineStr">
+      <c r="E31" s="8" t="inlineStr">
         <is>
           <t>Architetto</t>
         </is>
       </c>
-      <c r="F31" s="10" t="inlineStr">
+      <c r="F31" s="8" t="inlineStr">
         <is>
           <t>0ccea</t>
         </is>
       </c>
-      <c r="G31" s="11" t="inlineStr">
-        <is>
-          <t>https://collaboratori.rilievocontract.it/?ref=0ccea</t>
+      <c r="G31" s="9" t="inlineStr">
+        <is>
+          <t>https://presentazione.rilievocontract.it/?ref=0ccea</t>
         </is>
       </c>
     </row>
     <row r="32">
-      <c r="A32" s="8" t="inlineStr">
+      <c r="A32" s="6" t="inlineStr">
         <is>
           <t>107</t>
         </is>
       </c>
-      <c r="B32" s="8" t="inlineStr">
+      <c r="B32" s="6" t="inlineStr">
         <is>
           <t>Studio Arch. Lubiani</t>
         </is>
       </c>
-      <c r="C32" s="8" t="inlineStr"/>
-      <c r="D32" s="8" t="inlineStr">
+      <c r="C32" s="6" t="inlineStr"/>
+      <c r="D32" s="6" t="inlineStr">
         <is>
           <t>marcello.lubiani@gmail.com</t>
         </is>
       </c>
-      <c r="E32" s="8" t="inlineStr">
+      <c r="E32" s="6" t="inlineStr">
         <is>
           <t>Architetto</t>
         </is>
       </c>
-      <c r="F32" s="8" t="inlineStr">
+      <c r="F32" s="6" t="inlineStr">
         <is>
           <t>59352</t>
         </is>
       </c>
-      <c r="G32" s="9" t="inlineStr">
-        <is>
-          <t>https://collaboratori.rilievocontract.it/?ref=59352</t>
+      <c r="G32" s="7" t="inlineStr">
+        <is>
+          <t>https://presentazione.rilievocontract.it/?ref=59352</t>
         </is>
       </c>
     </row>
     <row r="33">
-      <c r="A33" s="10" t="inlineStr">
+      <c r="A33" s="8" t="inlineStr">
         <is>
           <t>108</t>
         </is>
       </c>
-      <c r="B33" s="10" t="inlineStr">
+      <c r="B33" s="8" t="inlineStr">
         <is>
           <t>PIXEL Architecture Studio</t>
         </is>
       </c>
-      <c r="C33" s="10" t="inlineStr"/>
-      <c r="D33" s="10" t="inlineStr">
+      <c r="C33" s="8" t="inlineStr"/>
+      <c r="D33" s="8" t="inlineStr">
         <is>
           <t>archstefanogovoni@gmail.com</t>
         </is>
       </c>
-      <c r="E33" s="10" t="inlineStr">
+      <c r="E33" s="8" t="inlineStr">
         <is>
           <t>Architetto</t>
         </is>
       </c>
-      <c r="F33" s="10" t="inlineStr">
+      <c r="F33" s="8" t="inlineStr">
         <is>
           <t>1828a</t>
         </is>
       </c>
-      <c r="G33" s="11" t="inlineStr">
-        <is>
-          <t>https://collaboratori.rilievocontract.it/?ref=1828a</t>
+      <c r="G33" s="9" t="inlineStr">
+        <is>
+          <t>https://presentazione.rilievocontract.it/?ref=1828a</t>
         </is>
       </c>
     </row>
     <row r="34">
-      <c r="A34" s="8" t="inlineStr">
+      <c r="A34" s="6" t="inlineStr">
         <is>
           <t>109</t>
         </is>
       </c>
-      <c r="B34" s="8" t="inlineStr">
+      <c r="B34" s="6" t="inlineStr">
         <is>
           <t>Arch. Tedde</t>
         </is>
       </c>
-      <c r="C34" s="8" t="inlineStr"/>
-      <c r="D34" s="8" t="inlineStr">
+      <c r="C34" s="6" t="inlineStr"/>
+      <c r="D34" s="6" t="inlineStr">
         <is>
           <t>info@sandrotedde.com</t>
         </is>
       </c>
-      <c r="E34" s="8" t="inlineStr">
+      <c r="E34" s="6" t="inlineStr">
         <is>
           <t>Architetto</t>
         </is>
       </c>
-      <c r="F34" s="8" t="inlineStr">
+      <c r="F34" s="6" t="inlineStr">
         <is>
           <t>995bd</t>
         </is>
       </c>
-      <c r="G34" s="9" t="inlineStr">
-        <is>
-          <t>https://collaboratori.rilievocontract.it/?ref=995bd</t>
+      <c r="G34" s="7" t="inlineStr">
+        <is>
+          <t>https://presentazione.rilievocontract.it/?ref=995bd</t>
         </is>
       </c>
     </row>
     <row r="35">
-      <c r="A35" s="10" t="inlineStr">
+      <c r="A35" s="8" t="inlineStr">
         <is>
           <t>110</t>
         </is>
       </c>
-      <c r="B35" s="10" t="inlineStr">
+      <c r="B35" s="8" t="inlineStr">
         <is>
           <t>GAAP Studio</t>
         </is>
       </c>
-      <c r="C35" s="10" t="inlineStr"/>
-      <c r="D35" s="10" t="inlineStr">
+      <c r="C35" s="8" t="inlineStr"/>
+      <c r="D35" s="8" t="inlineStr">
         <is>
           <t>giorgio.asciutti@gmail.com</t>
         </is>
       </c>
-      <c r="E35" s="10" t="inlineStr">
+      <c r="E35" s="8" t="inlineStr">
         <is>
           <t>Architetto</t>
         </is>
       </c>
-      <c r="F35" s="10" t="inlineStr">
+      <c r="F35" s="8" t="inlineStr">
         <is>
           <t>929ef</t>
         </is>
       </c>
-      <c r="G35" s="11" t="inlineStr">
-        <is>
-          <t>https://collaboratori.rilievocontract.it/?ref=929ef</t>
+      <c r="G35" s="9" t="inlineStr">
+        <is>
+          <t>https://presentazione.rilievocontract.it/?ref=929ef</t>
         </is>
       </c>
     </row>
     <row r="36">
-      <c r="A36" s="8" t="inlineStr">
+      <c r="A36" s="6" t="inlineStr">
         <is>
           <t>111</t>
         </is>
       </c>
-      <c r="B36" s="8" t="inlineStr">
+      <c r="B36" s="6" t="inlineStr">
         <is>
           <t>Studio Lesuisse</t>
         </is>
       </c>
-      <c r="C36" s="8" t="inlineStr"/>
-      <c r="D36" s="8" t="inlineStr">
+      <c r="C36" s="6" t="inlineStr"/>
+      <c r="D36" s="6" t="inlineStr">
         <is>
           <t>studio@studiolesuisse.com</t>
         </is>
       </c>
-      <c r="E36" s="8" t="inlineStr">
+      <c r="E36" s="6" t="inlineStr">
         <is>
           <t>Architetto</t>
         </is>
       </c>
-      <c r="F36" s="8" t="inlineStr">
+      <c r="F36" s="6" t="inlineStr">
         <is>
           <t>d6f13</t>
         </is>
       </c>
-      <c r="G36" s="9" t="inlineStr">
-        <is>
-          <t>https://collaboratori.rilievocontract.it/?ref=d6f13</t>
+      <c r="G36" s="7" t="inlineStr">
+        <is>
+          <t>https://presentazione.rilievocontract.it/?ref=d6f13</t>
         </is>
       </c>
     </row>
     <row r="37">
-      <c r="A37" s="10" t="inlineStr">
+      <c r="A37" s="8" t="inlineStr">
         <is>
           <t>112</t>
         </is>
       </c>
-      <c r="B37" s="10" t="inlineStr">
+      <c r="B37" s="8" t="inlineStr">
         <is>
           <t>SP Interior Design</t>
         </is>
       </c>
-      <c r="C37" s="10" t="inlineStr"/>
-      <c r="D37" s="10" t="inlineStr">
+      <c r="C37" s="8" t="inlineStr"/>
+      <c r="D37" s="8" t="inlineStr">
         <is>
           <t>info@annalisazini.it</t>
         </is>
       </c>
-      <c r="E37" s="10" t="inlineStr">
+      <c r="E37" s="8" t="inlineStr">
         <is>
           <t>Architetto</t>
         </is>
       </c>
-      <c r="F37" s="10" t="inlineStr">
+      <c r="F37" s="8" t="inlineStr">
         <is>
           <t>8d0aa</t>
         </is>
       </c>
-      <c r="G37" s="11" t="inlineStr">
-        <is>
-          <t>https://collaboratori.rilievocontract.it/?ref=8d0aa</t>
+      <c r="G37" s="9" t="inlineStr">
+        <is>
+          <t>https://presentazione.rilievocontract.it/?ref=8d0aa</t>
         </is>
       </c>
     </row>
     <row r="38">
-      <c r="A38" s="8" t="inlineStr">
+      <c r="A38" s="6" t="inlineStr">
         <is>
           <t>113</t>
         </is>
       </c>
-      <c r="B38" s="8" t="inlineStr">
+      <c r="B38" s="6" t="inlineStr">
         <is>
           <t>Cozy Design</t>
         </is>
       </c>
-      <c r="C38" s="8" t="inlineStr"/>
-      <c r="D38" s="8" t="inlineStr">
+      <c r="C38" s="6" t="inlineStr"/>
+      <c r="D38" s="6" t="inlineStr">
         <is>
           <t>sonia@cozydesign.it</t>
         </is>
       </c>
-      <c r="E38" s="8" t="inlineStr">
+      <c r="E38" s="6" t="inlineStr">
         <is>
           <t>Architetto</t>
         </is>
       </c>
-      <c r="F38" s="8" t="inlineStr">
+      <c r="F38" s="6" t="inlineStr">
         <is>
           <t>56ef3</t>
         </is>
       </c>
-      <c r="G38" s="9" t="inlineStr">
-        <is>
-          <t>https://collaboratori.rilievocontract.it/?ref=56ef3</t>
+      <c r="G38" s="7" t="inlineStr">
+        <is>
+          <t>https://presentazione.rilievocontract.it/?ref=56ef3</t>
         </is>
       </c>
     </row>
     <row r="39">
-      <c r="A39" s="10" t="inlineStr">
+      <c r="A39" s="8" t="inlineStr">
         <is>
           <t>114</t>
         </is>
       </c>
-      <c r="B39" s="10" t="inlineStr">
+      <c r="B39" s="8" t="inlineStr">
         <is>
           <t>Studio LineArch</t>
         </is>
       </c>
-      <c r="C39" s="10" t="inlineStr"/>
-      <c r="D39" s="10" t="inlineStr">
+      <c r="C39" s="8" t="inlineStr"/>
+      <c r="D39" s="8" t="inlineStr">
         <is>
           <t>info@linearch.it</t>
         </is>
       </c>
-      <c r="E39" s="10" t="inlineStr">
+      <c r="E39" s="8" t="inlineStr">
         <is>
           <t>Architetto</t>
         </is>
       </c>
-      <c r="F39" s="10" t="inlineStr">
+      <c r="F39" s="8" t="inlineStr">
         <is>
           <t>bbd89</t>
         </is>
       </c>
-      <c r="G39" s="11" t="inlineStr">
-        <is>
-          <t>https://collaboratori.rilievocontract.it/?ref=bbd89</t>
+      <c r="G39" s="9" t="inlineStr">
+        <is>
+          <t>https://presentazione.rilievocontract.it/?ref=bbd89</t>
         </is>
       </c>
     </row>
     <row r="40">
-      <c r="A40" s="8" t="inlineStr">
+      <c r="A40" s="6" t="inlineStr">
         <is>
           <t>115</t>
         </is>
       </c>
-      <c r="B40" s="8" t="inlineStr">
+      <c r="B40" s="6" t="inlineStr">
         <is>
           <t>Arch. Danila Lampis</t>
         </is>
       </c>
-      <c r="C40" s="8" t="inlineStr"/>
-      <c r="D40" s="8" t="inlineStr">
+      <c r="C40" s="6" t="inlineStr"/>
+      <c r="D40" s="6" t="inlineStr">
         <is>
           <t>lampis.danila@gmail.com</t>
         </is>
       </c>
-      <c r="E40" s="8" t="inlineStr">
+      <c r="E40" s="6" t="inlineStr">
         <is>
           <t>Architetto</t>
         </is>
       </c>
-      <c r="F40" s="8" t="inlineStr">
+      <c r="F40" s="6" t="inlineStr">
         <is>
           <t>6897e</t>
         </is>
       </c>
-      <c r="G40" s="9" t="inlineStr">
-        <is>
-          <t>https://collaboratori.rilievocontract.it/?ref=6897e</t>
+      <c r="G40" s="7" t="inlineStr">
+        <is>
+          <t>https://presentazione.rilievocontract.it/?ref=6897e</t>
         </is>
       </c>
     </row>
     <row r="41">
-      <c r="A41" s="10" t="inlineStr">
+      <c r="A41" s="8" t="inlineStr">
         <is>
           <t>116</t>
         </is>
       </c>
-      <c r="B41" s="10" t="inlineStr">
+      <c r="B41" s="8" t="inlineStr">
         <is>
           <t>Arch. Alessandro Cardellini</t>
         </is>
       </c>
-      <c r="C41" s="10" t="inlineStr"/>
-      <c r="D41" s="10" t="inlineStr">
+      <c r="C41" s="8" t="inlineStr"/>
+      <c r="D41" s="8" t="inlineStr">
         <is>
           <t>alessandro@ac-architetto.com</t>
         </is>
       </c>
-      <c r="E41" s="10" t="inlineStr">
+      <c r="E41" s="8" t="inlineStr">
         <is>
           <t>Architetto</t>
         </is>
       </c>
-      <c r="F41" s="10" t="inlineStr">
+      <c r="F41" s="8" t="inlineStr">
         <is>
           <t>8d589</t>
         </is>
       </c>
-      <c r="G41" s="11" t="inlineStr">
-        <is>
-          <t>https://collaboratori.rilievocontract.it/?ref=8d589</t>
+      <c r="G41" s="9" t="inlineStr">
+        <is>
+          <t>https://presentazione.rilievocontract.it/?ref=8d589</t>
         </is>
       </c>
     </row>
     <row r="42">
-      <c r="A42" s="8" t="inlineStr">
+      <c r="A42" s="6" t="inlineStr">
         <is>
           <t>117</t>
         </is>
       </c>
-      <c r="B42" s="8" t="inlineStr">
+      <c r="B42" s="6" t="inlineStr">
         <is>
           <t>Arch. Stefania Negrini</t>
         </is>
       </c>
-      <c r="C42" s="8" t="inlineStr"/>
-      <c r="D42" s="8" t="inlineStr">
+      <c r="C42" s="6" t="inlineStr"/>
+      <c r="D42" s="6" t="inlineStr">
         <is>
           <t>info@negriniinteriors.com</t>
         </is>
       </c>
-      <c r="E42" s="8" t="inlineStr">
+      <c r="E42" s="6" t="inlineStr">
         <is>
           <t>Architetto</t>
         </is>
       </c>
-      <c r="F42" s="8" t="inlineStr">
+      <c r="F42" s="6" t="inlineStr">
         <is>
           <t>3322a</t>
         </is>
       </c>
-      <c r="G42" s="9" t="inlineStr">
-        <is>
-          <t>https://collaboratori.rilievocontract.it/?ref=3322a</t>
+      <c r="G42" s="7" t="inlineStr">
+        <is>
+          <t>https://presentazione.rilievocontract.it/?ref=3322a</t>
         </is>
       </c>
     </row>
     <row r="43">
-      <c r="A43" s="10" t="inlineStr">
+      <c r="A43" s="8" t="inlineStr">
         <is>
           <t>118</t>
         </is>
       </c>
-      <c r="B43" s="10" t="inlineStr">
+      <c r="B43" s="8" t="inlineStr">
         <is>
           <t>HZ Studio Architettura</t>
         </is>
       </c>
-      <c r="C43" s="10" t="inlineStr"/>
-      <c r="D43" s="10" t="inlineStr">
+      <c r="C43" s="8" t="inlineStr"/>
+      <c r="D43" s="8" t="inlineStr">
         <is>
           <t>studio@hzstudio.it</t>
         </is>
       </c>
-      <c r="E43" s="10" t="inlineStr">
+      <c r="E43" s="8" t="inlineStr">
         <is>
           <t>Architetto</t>
         </is>
       </c>
-      <c r="F43" s="10" t="inlineStr">
+      <c r="F43" s="8" t="inlineStr">
         <is>
           <t>f2d0e</t>
         </is>
       </c>
-      <c r="G43" s="11" t="inlineStr">
-        <is>
-          <t>https://collaboratori.rilievocontract.it/?ref=f2d0e</t>
+      <c r="G43" s="9" t="inlineStr">
+        <is>
+          <t>https://presentazione.rilievocontract.it/?ref=f2d0e</t>
         </is>
       </c>
     </row>
@@ -2204,7 +2148,6 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G43" r:id="rId42"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-  <legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="anysvml"/>
 </worksheet>
 </file>
 
@@ -2214,684 +2157,1165 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G20"/>
+  <dimension ref="A1:G33"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="8" customWidth="1" min="1" max="1"/>
-    <col width="34" customWidth="1" min="2" max="2"/>
-    <col width="24" customWidth="1" min="3" max="3"/>
-    <col width="32" customWidth="1" min="4" max="4"/>
-    <col width="26" customWidth="1" min="5" max="5"/>
-    <col width="10" customWidth="1" min="6" max="6"/>
+    <col width="30" customWidth="1" min="1" max="1"/>
+    <col width="30" customWidth="1" min="2" max="2"/>
+    <col width="30" customWidth="1" min="3" max="3"/>
+    <col width="30" customWidth="1" min="4" max="4"/>
+    <col width="30" customWidth="1" min="5" max="5"/>
+    <col width="30" customWidth="1" min="6" max="6"/>
     <col width="52" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
-    <row r="1" ht="20" customHeight="1">
-      <c r="A1" s="7" t="inlineStr">
-        <is>
-          <t>ID</t>
-        </is>
-      </c>
-      <c r="B1" s="7" t="inlineStr">
+    <row r="1">
+      <c r="A1" s="3" t="inlineStr">
+        <is>
+          <t>Id</t>
+        </is>
+      </c>
+      <c r="B1" s="3" t="inlineStr">
         <is>
           <t>Nome</t>
         </is>
       </c>
-      <c r="C1" s="7" t="inlineStr">
-        <is>
-          <t>Città</t>
-        </is>
-      </c>
-      <c r="D1" s="7" t="inlineStr">
+      <c r="C1" s="3" t="inlineStr">
+        <is>
+          <t>Citta</t>
+        </is>
+      </c>
+      <c r="D1" s="3" t="inlineStr">
         <is>
           <t>Email</t>
         </is>
       </c>
-      <c r="E1" s="7" t="inlineStr">
+      <c r="E1" s="3" t="inlineStr">
         <is>
           <t>Categoria</t>
         </is>
       </c>
-      <c r="F1" s="7" t="inlineStr">
+      <c r="F1" s="3" t="inlineStr">
         <is>
           <t>Ref</t>
         </is>
       </c>
-      <c r="G1" s="7" t="inlineStr">
-        <is>
-          <t>Link presentazione</t>
+      <c r="G1" s="3" t="inlineStr">
+        <is>
+          <t>Link</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="8" t="inlineStr">
+      <c r="A2" s="6" t="inlineStr">
         <is>
           <t>A1</t>
         </is>
       </c>
-      <c r="B2" s="8" t="inlineStr">
+      <c r="B2" s="6" t="inlineStr">
         <is>
           <t>Centocase Sardegna</t>
         </is>
       </c>
-      <c r="C2" s="8" t="inlineStr"/>
-      <c r="D2" s="8" t="inlineStr">
+      <c r="C2" s="6" t="inlineStr"/>
+      <c r="D2" s="6" t="inlineStr">
         <is>
           <t>info@centocasesardegna.it</t>
         </is>
       </c>
-      <c r="E2" s="8" t="inlineStr">
+      <c r="E2" s="6" t="inlineStr">
         <is>
           <t>Agenzia immobiliare</t>
         </is>
       </c>
-      <c r="F2" s="8" t="inlineStr">
+      <c r="F2" s="6" t="inlineStr">
         <is>
           <t>a1f1c</t>
         </is>
       </c>
-      <c r="G2" s="9" t="inlineStr">
+      <c r="G2" s="7" t="inlineStr">
         <is>
           <t>https://agenzie-immobiliari.rilievocontract.it/?ref=a1f1c</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="10" t="inlineStr">
+      <c r="A3" s="8" t="inlineStr">
         <is>
           <t>A2</t>
         </is>
       </c>
-      <c r="B3" s="10" t="inlineStr">
+      <c r="B3" s="8" t="inlineStr">
         <is>
           <t>Smeraldina Immobiliare</t>
         </is>
       </c>
-      <c r="C3" s="10" t="inlineStr"/>
-      <c r="D3" s="10" t="inlineStr">
+      <c r="C3" s="8" t="inlineStr"/>
+      <c r="D3" s="8" t="inlineStr">
         <is>
           <t>smeraldinaimmobiliare@gmail.com</t>
         </is>
       </c>
-      <c r="E3" s="10" t="inlineStr">
+      <c r="E3" s="8" t="inlineStr">
         <is>
           <t>Agenzia immobiliare</t>
         </is>
       </c>
-      <c r="F3" s="10" t="inlineStr">
+      <c r="F3" s="8" t="inlineStr">
         <is>
           <t>77a3d</t>
         </is>
       </c>
-      <c r="G3" s="11" t="inlineStr">
+      <c r="G3" s="9" t="inlineStr">
         <is>
           <t>https://agenzie-immobiliari.rilievocontract.it/?ref=77a3d</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="8" t="inlineStr">
+      <c r="A4" s="6" t="inlineStr">
         <is>
           <t>A3</t>
         </is>
       </c>
-      <c r="B4" s="8" t="inlineStr">
+      <c r="B4" s="6" t="inlineStr">
         <is>
           <t>Immobiliare La Maddalena</t>
         </is>
       </c>
-      <c r="C4" s="8" t="inlineStr"/>
-      <c r="D4" s="8" t="inlineStr">
+      <c r="C4" s="6" t="inlineStr"/>
+      <c r="D4" s="6" t="inlineStr">
         <is>
           <t>immlamaddalena@gmail.com</t>
         </is>
       </c>
-      <c r="E4" s="8" t="inlineStr">
+      <c r="E4" s="6" t="inlineStr">
         <is>
           <t>Agenzia immobiliare</t>
         </is>
       </c>
-      <c r="F4" s="8" t="inlineStr">
+      <c r="F4" s="6" t="inlineStr">
         <is>
           <t>18fd2</t>
         </is>
       </c>
-      <c r="G4" s="9" t="inlineStr">
+      <c r="G4" s="7" t="inlineStr">
         <is>
           <t>https://agenzie-immobiliari.rilievocontract.it/?ref=18fd2</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="10" t="inlineStr">
+      <c r="A5" s="8" t="inlineStr">
         <is>
           <t>A4</t>
         </is>
       </c>
-      <c r="B5" s="10" t="inlineStr">
+      <c r="B5" s="8" t="inlineStr">
         <is>
           <t>Realia Brokers</t>
         </is>
       </c>
-      <c r="C5" s="10" t="inlineStr"/>
-      <c r="D5" s="10" t="inlineStr">
+      <c r="C5" s="8" t="inlineStr"/>
+      <c r="D5" s="8" t="inlineStr">
         <is>
           <t>info@realiabrokers.com</t>
         </is>
       </c>
-      <c r="E5" s="10" t="inlineStr">
+      <c r="E5" s="8" t="inlineStr">
         <is>
           <t>Agenzia immobiliare</t>
         </is>
       </c>
-      <c r="F5" s="10" t="inlineStr">
+      <c r="F5" s="8" t="inlineStr">
         <is>
           <t>70df9</t>
         </is>
       </c>
-      <c r="G5" s="11" t="inlineStr">
+      <c r="G5" s="9" t="inlineStr">
         <is>
           <t>https://agenzie-immobiliari.rilievocontract.it/?ref=70df9</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="8" t="inlineStr">
+      <c r="A6" s="6" t="inlineStr">
         <is>
           <t>A5</t>
         </is>
       </c>
-      <c r="B6" s="8" t="inlineStr">
+      <c r="B6" s="6" t="inlineStr">
         <is>
           <t>Phoenix Real Estate</t>
         </is>
       </c>
-      <c r="C6" s="8" t="inlineStr"/>
-      <c r="D6" s="8" t="inlineStr">
+      <c r="C6" s="6" t="inlineStr"/>
+      <c r="D6" s="6" t="inlineStr">
         <is>
           <t>phoenixrealestatesrls@gmail.com</t>
         </is>
       </c>
-      <c r="E6" s="8" t="inlineStr">
+      <c r="E6" s="6" t="inlineStr">
         <is>
           <t>Agenzia immobiliare</t>
         </is>
       </c>
-      <c r="F6" s="8" t="inlineStr">
+      <c r="F6" s="6" t="inlineStr">
         <is>
           <t>67910</t>
         </is>
       </c>
-      <c r="G6" s="9" t="inlineStr">
+      <c r="G6" s="7" t="inlineStr">
         <is>
           <t>https://agenzie-immobiliari.rilievocontract.it/?ref=67910</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="10" t="inlineStr">
+      <c r="A7" s="8" t="inlineStr">
         <is>
           <t>A6</t>
         </is>
       </c>
-      <c r="B7" s="10" t="inlineStr">
+      <c r="B7" s="8" t="inlineStr">
         <is>
           <t>Maior Capital | Forbes Global Properties</t>
         </is>
       </c>
-      <c r="C7" s="10" t="inlineStr"/>
-      <c r="D7" s="10" t="inlineStr">
+      <c r="C7" s="8" t="inlineStr"/>
+      <c r="D7" s="8" t="inlineStr">
         <is>
           <t>sardinia@maiorcapital.com</t>
         </is>
       </c>
-      <c r="E7" s="10" t="inlineStr">
+      <c r="E7" s="8" t="inlineStr">
         <is>
           <t>Agenzia immobiliare</t>
         </is>
       </c>
-      <c r="F7" s="10" t="inlineStr">
+      <c r="F7" s="8" t="inlineStr">
         <is>
           <t>11f28</t>
         </is>
       </c>
-      <c r="G7" s="11" t="inlineStr">
+      <c r="G7" s="9" t="inlineStr">
         <is>
           <t>https://agenzie-immobiliari.rilievocontract.it/?ref=11f28</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="8" t="inlineStr">
+      <c r="A8" s="6" t="inlineStr">
         <is>
           <t>A7</t>
         </is>
       </c>
-      <c r="B8" s="8" t="inlineStr">
+      <c r="B8" s="6" t="inlineStr">
         <is>
           <t>Gallura Immobiliare</t>
         </is>
       </c>
-      <c r="C8" s="8" t="inlineStr"/>
-      <c r="D8" s="8" t="inlineStr">
+      <c r="C8" s="6" t="inlineStr"/>
+      <c r="D8" s="6" t="inlineStr">
         <is>
           <t>galluraimmobiliare@virgilio.it</t>
         </is>
       </c>
-      <c r="E8" s="8" t="inlineStr">
+      <c r="E8" s="6" t="inlineStr">
         <is>
           <t>Agenzia immobiliare</t>
         </is>
       </c>
-      <c r="F8" s="8" t="inlineStr">
+      <c r="F8" s="6" t="inlineStr">
         <is>
           <t>15eb0</t>
         </is>
       </c>
-      <c r="G8" s="9" t="inlineStr">
+      <c r="G8" s="7" t="inlineStr">
         <is>
           <t>https://agenzie-immobiliari.rilievocontract.it/?ref=15eb0</t>
         </is>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="10" t="inlineStr">
+      <c r="A9" s="8" t="inlineStr">
         <is>
           <t>A8</t>
         </is>
       </c>
-      <c r="B9" s="10" t="inlineStr">
+      <c r="B9" s="8" t="inlineStr">
         <is>
           <t>House &amp; Domos Immobiliare</t>
         </is>
       </c>
-      <c r="C9" s="10" t="inlineStr"/>
-      <c r="D9" s="10" t="inlineStr">
+      <c r="C9" s="8" t="inlineStr"/>
+      <c r="D9" s="8" t="inlineStr">
         <is>
           <t>info@housedomos.com</t>
         </is>
       </c>
-      <c r="E9" s="10" t="inlineStr">
+      <c r="E9" s="8" t="inlineStr">
         <is>
           <t>Agenzia immobiliare</t>
         </is>
       </c>
-      <c r="F9" s="10" t="inlineStr">
+      <c r="F9" s="8" t="inlineStr">
         <is>
           <t>61b12</t>
         </is>
       </c>
-      <c r="G9" s="11" t="inlineStr">
+      <c r="G9" s="9" t="inlineStr">
         <is>
           <t>https://agenzie-immobiliari.rilievocontract.it/?ref=61b12</t>
         </is>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="8" t="inlineStr">
+      <c r="A10" s="6" t="inlineStr">
         <is>
           <t>A9</t>
         </is>
       </c>
-      <c r="B10" s="8" t="inlineStr">
+      <c r="B10" s="6" t="inlineStr">
         <is>
           <t>Il Faro Immobiliare</t>
         </is>
       </c>
-      <c r="C10" s="8" t="inlineStr"/>
-      <c r="D10" s="8" t="inlineStr">
+      <c r="C10" s="6" t="inlineStr"/>
+      <c r="D10" s="6" t="inlineStr">
         <is>
           <t>info@agenziailfaro.it</t>
         </is>
       </c>
-      <c r="E10" s="8" t="inlineStr">
+      <c r="E10" s="6" t="inlineStr">
         <is>
           <t>Agenzia immobiliare</t>
         </is>
       </c>
-      <c r="F10" s="8" t="inlineStr">
+      <c r="F10" s="6" t="inlineStr">
         <is>
           <t>66476</t>
         </is>
       </c>
-      <c r="G10" s="9" t="inlineStr">
+      <c r="G10" s="7" t="inlineStr">
         <is>
           <t>https://agenzie-immobiliari.rilievocontract.it/?ref=66476</t>
         </is>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="10" t="inlineStr">
+      <c r="A11" s="8" t="inlineStr">
         <is>
           <t>A10</t>
         </is>
       </c>
-      <c r="B11" s="10" t="inlineStr">
+      <c r="B11" s="8" t="inlineStr">
         <is>
           <t>Simius Immobiliare</t>
         </is>
       </c>
-      <c r="C11" s="10" t="inlineStr"/>
-      <c r="D11" s="10" t="inlineStr">
+      <c r="C11" s="8" t="inlineStr"/>
+      <c r="D11" s="8" t="inlineStr">
         <is>
           <t>info@simiusimmobiliare.com</t>
         </is>
       </c>
-      <c r="E11" s="10" t="inlineStr">
+      <c r="E11" s="8" t="inlineStr">
         <is>
           <t>Agenzia immobiliare</t>
         </is>
       </c>
-      <c r="F11" s="10" t="inlineStr">
+      <c r="F11" s="8" t="inlineStr">
         <is>
           <t>2c1c5</t>
         </is>
       </c>
-      <c r="G11" s="11" t="inlineStr">
+      <c r="G11" s="9" t="inlineStr">
         <is>
           <t>https://agenzie-immobiliari.rilievocontract.it/?ref=2c1c5</t>
         </is>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="8" t="inlineStr">
+      <c r="A12" s="6" t="inlineStr">
         <is>
           <t>A11</t>
         </is>
       </c>
-      <c r="B12" s="8" t="inlineStr">
+      <c r="B12" s="6" t="inlineStr">
         <is>
           <t>FrauMare Immobiliare</t>
         </is>
       </c>
-      <c r="C12" s="8" t="inlineStr"/>
-      <c r="D12" s="8" t="inlineStr">
+      <c r="C12" s="6" t="inlineStr"/>
+      <c r="D12" s="6" t="inlineStr">
         <is>
           <t>agenzia@fraumare.com</t>
         </is>
       </c>
-      <c r="E12" s="8" t="inlineStr">
+      <c r="E12" s="6" t="inlineStr">
         <is>
           <t>Agenzia immobiliare</t>
         </is>
       </c>
-      <c r="F12" s="8" t="inlineStr">
+      <c r="F12" s="6" t="inlineStr">
         <is>
           <t>f0e2b</t>
         </is>
       </c>
-      <c r="G12" s="9" t="inlineStr">
+      <c r="G12" s="7" t="inlineStr">
         <is>
           <t>https://agenzie-immobiliari.rilievocontract.it/?ref=f0e2b</t>
         </is>
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="10" t="inlineStr">
+      <c r="A13" s="8" t="inlineStr">
         <is>
           <t>A12</t>
         </is>
       </c>
-      <c r="B13" s="10" t="inlineStr">
+      <c r="B13" s="8" t="inlineStr">
         <is>
           <t>Casula Immobiliare</t>
         </is>
       </c>
-      <c r="C13" s="10" t="inlineStr"/>
-      <c r="D13" s="10" t="inlineStr">
+      <c r="C13" s="8" t="inlineStr"/>
+      <c r="D13" s="8" t="inlineStr">
         <is>
           <t>info@casulaimmobiliare.com</t>
         </is>
       </c>
-      <c r="E13" s="10" t="inlineStr">
+      <c r="E13" s="8" t="inlineStr">
         <is>
           <t>Agenzia immobiliare</t>
         </is>
       </c>
-      <c r="F13" s="10" t="inlineStr">
+      <c r="F13" s="8" t="inlineStr">
         <is>
           <t>2d044</t>
         </is>
       </c>
-      <c r="G13" s="11" t="inlineStr">
+      <c r="G13" s="9" t="inlineStr">
         <is>
           <t>https://agenzie-immobiliari.rilievocontract.it/?ref=2d044</t>
         </is>
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="8" t="inlineStr">
+      <c r="A14" s="6" t="inlineStr">
         <is>
           <t>A13</t>
         </is>
       </c>
-      <c r="B14" s="8" t="inlineStr">
+      <c r="B14" s="6" t="inlineStr">
         <is>
           <t>Ital Home Costa Rei/Villasimius</t>
         </is>
       </c>
-      <c r="C14" s="8" t="inlineStr"/>
-      <c r="D14" s="8" t="inlineStr">
+      <c r="C14" s="6" t="inlineStr"/>
+      <c r="D14" s="6" t="inlineStr">
         <is>
           <t>villasimius@ital-home.it</t>
         </is>
       </c>
-      <c r="E14" s="8" t="inlineStr">
+      <c r="E14" s="6" t="inlineStr">
         <is>
           <t>Agenzia immobiliare</t>
         </is>
       </c>
-      <c r="F14" s="8" t="inlineStr">
+      <c r="F14" s="6" t="inlineStr">
         <is>
           <t>0d759</t>
         </is>
       </c>
-      <c r="G14" s="9" t="inlineStr">
+      <c r="G14" s="7" t="inlineStr">
         <is>
           <t>https://agenzie-immobiliari.rilievocontract.it/?ref=0d759</t>
         </is>
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="10" t="inlineStr">
+      <c r="A15" s="8" t="inlineStr">
         <is>
           <t>A14</t>
         </is>
       </c>
-      <c r="B15" s="10" t="inlineStr">
+      <c r="B15" s="8" t="inlineStr">
         <is>
           <t>IMMOVA</t>
         </is>
       </c>
-      <c r="C15" s="10" t="inlineStr"/>
-      <c r="D15" s="10" t="inlineStr">
+      <c r="C15" s="8" t="inlineStr"/>
+      <c r="D15" s="8" t="inlineStr">
         <is>
           <t>immova2021@gmail.com</t>
         </is>
       </c>
-      <c r="E15" s="10" t="inlineStr">
+      <c r="E15" s="8" t="inlineStr">
         <is>
           <t>Agenzia immobiliare</t>
         </is>
       </c>
-      <c r="F15" s="10" t="inlineStr">
+      <c r="F15" s="8" t="inlineStr">
         <is>
           <t>baa1e</t>
         </is>
       </c>
-      <c r="G15" s="11" t="inlineStr">
+      <c r="G15" s="9" t="inlineStr">
         <is>
           <t>https://agenzie-immobiliari.rilievocontract.it/?ref=baa1e</t>
         </is>
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="8" t="inlineStr">
+      <c r="A16" s="6" t="inlineStr">
         <is>
           <t>A15</t>
         </is>
       </c>
-      <c r="B16" s="8" t="inlineStr">
+      <c r="B16" s="6" t="inlineStr">
         <is>
           <t>Minvicase</t>
         </is>
       </c>
-      <c r="C16" s="8" t="inlineStr"/>
-      <c r="D16" s="8" t="inlineStr">
+      <c r="C16" s="6" t="inlineStr"/>
+      <c r="D16" s="6" t="inlineStr">
         <is>
           <t>info@minvicase.it</t>
         </is>
       </c>
-      <c r="E16" s="8" t="inlineStr">
+      <c r="E16" s="6" t="inlineStr">
         <is>
           <t>Agenzia immobiliare</t>
         </is>
       </c>
-      <c r="F16" s="8" t="inlineStr">
+      <c r="F16" s="6" t="inlineStr">
         <is>
           <t>24ebd</t>
         </is>
       </c>
-      <c r="G16" s="9" t="inlineStr">
+      <c r="G16" s="7" t="inlineStr">
         <is>
           <t>https://agenzie-immobiliari.rilievocontract.it/?ref=24ebd</t>
         </is>
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="10" t="inlineStr">
+      <c r="A17" s="8" t="inlineStr">
         <is>
           <t>A16</t>
         </is>
       </c>
-      <c r="B17" s="10" t="inlineStr">
+      <c r="B17" s="8" t="inlineStr">
         <is>
           <t>La Tua Casa al Mare</t>
         </is>
       </c>
-      <c r="C17" s="10" t="inlineStr"/>
-      <c r="D17" s="10" t="inlineStr">
+      <c r="C17" s="8" t="inlineStr"/>
+      <c r="D17" s="8" t="inlineStr">
         <is>
           <t>info@latuacasaalmare.it</t>
         </is>
       </c>
-      <c r="E17" s="10" t="inlineStr">
+      <c r="E17" s="8" t="inlineStr">
         <is>
           <t>Agenzia immobiliare</t>
         </is>
       </c>
-      <c r="F17" s="10" t="inlineStr">
+      <c r="F17" s="8" t="inlineStr">
         <is>
           <t>8583b</t>
         </is>
       </c>
-      <c r="G17" s="11" t="inlineStr">
+      <c r="G17" s="9" t="inlineStr">
         <is>
           <t>https://agenzie-immobiliari.rilievocontract.it/?ref=8583b</t>
         </is>
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="8" t="inlineStr">
+      <c r="A18" s="6" t="inlineStr">
         <is>
           <t>A17</t>
         </is>
       </c>
-      <c r="B18" s="8" t="inlineStr">
+      <c r="B18" s="6" t="inlineStr">
         <is>
           <t>Alghero Ital Home</t>
         </is>
       </c>
-      <c r="C18" s="8" t="inlineStr"/>
-      <c r="D18" s="8" t="inlineStr">
+      <c r="C18" s="6" t="inlineStr"/>
+      <c r="D18" s="6" t="inlineStr">
         <is>
           <t>alghero@ital-home.it</t>
         </is>
       </c>
-      <c r="E18" s="8" t="inlineStr">
+      <c r="E18" s="6" t="inlineStr">
         <is>
           <t>Agenzia immobiliare</t>
         </is>
       </c>
-      <c r="F18" s="8" t="inlineStr">
+      <c r="F18" s="6" t="inlineStr">
         <is>
           <t>3dfa7</t>
         </is>
       </c>
-      <c r="G18" s="9" t="inlineStr">
+      <c r="G18" s="7" t="inlineStr">
         <is>
           <t>https://agenzie-immobiliari.rilievocontract.it/?ref=3dfa7</t>
         </is>
       </c>
     </row>
     <row r="19">
-      <c r="A19" s="10" t="inlineStr">
+      <c r="A19" s="8" t="inlineStr">
         <is>
           <t>A18</t>
         </is>
       </c>
-      <c r="B19" s="10" t="inlineStr">
+      <c r="B19" s="8" t="inlineStr">
         <is>
           <t>Agenzia Capo Falcone</t>
         </is>
       </c>
-      <c r="C19" s="10" t="inlineStr"/>
-      <c r="D19" s="10" t="inlineStr">
+      <c r="C19" s="8" t="inlineStr"/>
+      <c r="D19" s="8" t="inlineStr">
         <is>
           <t>stintino@email.it</t>
         </is>
       </c>
-      <c r="E19" s="10" t="inlineStr">
+      <c r="E19" s="8" t="inlineStr">
         <is>
           <t>Agenzia immobiliare</t>
         </is>
       </c>
-      <c r="F19" s="10" t="inlineStr">
+      <c r="F19" s="8" t="inlineStr">
         <is>
           <t>4c4fd</t>
         </is>
       </c>
-      <c r="G19" s="11" t="inlineStr">
+      <c r="G19" s="9" t="inlineStr">
         <is>
           <t>https://agenzie-immobiliari.rilievocontract.it/?ref=4c4fd</t>
         </is>
       </c>
     </row>
     <row r="20">
-      <c r="A20" s="8" t="inlineStr">
+      <c r="A20" s="6" t="inlineStr">
         <is>
           <t>A19</t>
         </is>
       </c>
-      <c r="B20" s="8" t="inlineStr">
+      <c r="B20" s="6" t="inlineStr">
         <is>
           <t>Ajò Immobiliare</t>
         </is>
       </c>
-      <c r="C20" s="8" t="inlineStr"/>
-      <c r="D20" s="8" t="inlineStr">
+      <c r="C20" s="6" t="inlineStr"/>
+      <c r="D20" s="6" t="inlineStr">
         <is>
           <t>info@ajo.casa</t>
         </is>
       </c>
-      <c r="E20" s="8" t="inlineStr">
+      <c r="E20" s="6" t="inlineStr">
         <is>
           <t>Agenzia immobiliare</t>
         </is>
       </c>
-      <c r="F20" s="8" t="inlineStr">
+      <c r="F20" s="6" t="inlineStr">
         <is>
           <t>e3d9a</t>
         </is>
       </c>
-      <c r="G20" s="9" t="inlineStr">
+      <c r="G20" s="7" t="inlineStr">
         <is>
           <t>https://agenzie-immobiliari.rilievocontract.it/?ref=e3d9a</t>
         </is>
       </c>
     </row>
+    <row r="21">
+      <c r="A21" s="8" t="inlineStr">
+        <is>
+          <t>A20</t>
+        </is>
+      </c>
+      <c r="B21" s="8" t="inlineStr">
+        <is>
+          <t>Coldwell Banker Global Luxury</t>
+        </is>
+      </c>
+      <c r="C21" s="8" t="inlineStr">
+        <is>
+          <t>Porto Cervo — Arzachena (SS)</t>
+        </is>
+      </c>
+      <c r="D21" s="8" t="inlineStr">
+        <is>
+          <t>portocervo@cbitaly.it</t>
+        </is>
+      </c>
+      <c r="E21" s="8" t="inlineStr">
+        <is>
+          <t>Agenzia immobiliare</t>
+        </is>
+      </c>
+      <c r="F21" s="8" t="inlineStr">
+        <is>
+          <t>f169a</t>
+        </is>
+      </c>
+      <c r="G21" s="8" t="inlineStr">
+        <is>
+          <t>https://agenzie-immobiliari.rilievocontract.it/?ref=f169a</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="6" t="inlineStr">
+        <is>
+          <t>A21</t>
+        </is>
+      </c>
+      <c r="B22" s="6" t="inlineStr">
+        <is>
+          <t>Luxury Esmeralda (Savills)</t>
+        </is>
+      </c>
+      <c r="C22" s="6" t="inlineStr">
+        <is>
+          <t>Porto Rotondo — Olbia (SS)</t>
+        </is>
+      </c>
+      <c r="D22" s="6" t="inlineStr">
+        <is>
+          <t>info@luxuryesmeralda.com</t>
+        </is>
+      </c>
+      <c r="E22" s="6" t="inlineStr">
+        <is>
+          <t>Agenzia immobiliare</t>
+        </is>
+      </c>
+      <c r="F22" s="6" t="inlineStr">
+        <is>
+          <t>88560</t>
+        </is>
+      </c>
+      <c r="G22" s="6" t="inlineStr">
+        <is>
+          <t>https://agenzie-immobiliari.rilievocontract.it/?ref=88560</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="8" t="inlineStr">
+        <is>
+          <t>A22</t>
+        </is>
+      </c>
+      <c r="B23" s="8" t="inlineStr">
+        <is>
+          <t>BARNES Sardegna</t>
+        </is>
+      </c>
+      <c r="C23" s="8" t="inlineStr">
+        <is>
+          <t>Porto Cervo — Arzachena (SS)</t>
+        </is>
+      </c>
+      <c r="D23" s="8" t="inlineStr">
+        <is>
+          <t>portocervo@barnes-international.com</t>
+        </is>
+      </c>
+      <c r="E23" s="8" t="inlineStr">
+        <is>
+          <t>Agenzia immobiliare</t>
+        </is>
+      </c>
+      <c r="F23" s="8" t="inlineStr">
+        <is>
+          <t>90eca</t>
+        </is>
+      </c>
+      <c r="G23" s="8" t="inlineStr">
+        <is>
+          <t>https://agenzie-immobiliari.rilievocontract.it/?ref=90eca</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="6" t="inlineStr">
+        <is>
+          <t>A23</t>
+        </is>
+      </c>
+      <c r="B24" s="6" t="inlineStr">
+        <is>
+          <t>Engel &amp; Völkers Costa Smeralda</t>
+        </is>
+      </c>
+      <c r="C24" s="6" t="inlineStr">
+        <is>
+          <t>Porto Cervo — Arzachena (SS)</t>
+        </is>
+      </c>
+      <c r="D24" s="6" t="inlineStr">
+        <is>
+          <t>portocervo@engelvoelkers.com</t>
+        </is>
+      </c>
+      <c r="E24" s="6" t="inlineStr">
+        <is>
+          <t>Agenzia immobiliare</t>
+        </is>
+      </c>
+      <c r="F24" s="6" t="inlineStr">
+        <is>
+          <t>d73db</t>
+        </is>
+      </c>
+      <c r="G24" s="6" t="inlineStr">
+        <is>
+          <t>https://agenzie-immobiliari.rilievocontract.it/?ref=d73db</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="8" t="inlineStr">
+        <is>
+          <t>A24</t>
+        </is>
+      </c>
+      <c r="B25" s="8" t="inlineStr">
+        <is>
+          <t>Italy Sotheby's International Realty</t>
+        </is>
+      </c>
+      <c r="C25" s="8" t="inlineStr">
+        <is>
+          <t>Porto Cervo (SS)</t>
+        </is>
+      </c>
+      <c r="D25" s="8" t="inlineStr">
+        <is>
+          <t>portocervo@sothebysrealty.it</t>
+        </is>
+      </c>
+      <c r="E25" s="8" t="inlineStr">
+        <is>
+          <t>Agenzia immobiliare</t>
+        </is>
+      </c>
+      <c r="F25" s="8" t="inlineStr">
+        <is>
+          <t>e6e4d</t>
+        </is>
+      </c>
+      <c r="G25" s="8" t="inlineStr">
+        <is>
+          <t>https://agenzie-immobiliari.rilievocontract.it/?ref=e6e4d</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="6" t="inlineStr">
+        <is>
+          <t>A25</t>
+        </is>
+      </c>
+      <c r="B26" s="6" t="inlineStr">
+        <is>
+          <t>ImmobilSarda Christie's International Real Estate</t>
+        </is>
+      </c>
+      <c r="C26" s="6" t="inlineStr">
+        <is>
+          <t>Porto Cervo (SS)</t>
+        </is>
+      </c>
+      <c r="D26" s="6" t="inlineStr">
+        <is>
+          <t>portocervo@immobilsarda.com</t>
+        </is>
+      </c>
+      <c r="E26" s="6" t="inlineStr">
+        <is>
+          <t>Agenzia immobiliare</t>
+        </is>
+      </c>
+      <c r="F26" s="6" t="inlineStr">
+        <is>
+          <t>f36e7</t>
+        </is>
+      </c>
+      <c r="G26" s="6" t="inlineStr">
+        <is>
+          <t>https://agenzie-immobiliari.rilievocontract.it/?ref=f36e7</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="8" t="inlineStr">
+        <is>
+          <t>A26</t>
+        </is>
+      </c>
+      <c r="B27" s="8" t="inlineStr">
+        <is>
+          <t>Capitta &amp; Partners</t>
+        </is>
+      </c>
+      <c r="C27" s="8" t="inlineStr">
+        <is>
+          <t>Cagliari</t>
+        </is>
+      </c>
+      <c r="D27" s="8" t="inlineStr">
+        <is>
+          <t>info@capittaepartners.it</t>
+        </is>
+      </c>
+      <c r="E27" s="8" t="inlineStr">
+        <is>
+          <t>Agenzia immobiliare</t>
+        </is>
+      </c>
+      <c r="F27" s="8" t="inlineStr">
+        <is>
+          <t>65a2a</t>
+        </is>
+      </c>
+      <c r="G27" s="8" t="inlineStr">
+        <is>
+          <t>https://agenzie-immobiliari.rilievocontract.it/?ref=65a2a</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="6" t="inlineStr">
+        <is>
+          <t>A27</t>
+        </is>
+      </c>
+      <c r="B28" s="6" t="inlineStr">
+        <is>
+          <t>Ladiri Immobiliare</t>
+        </is>
+      </c>
+      <c r="C28" s="6" t="inlineStr">
+        <is>
+          <t>Cagliari</t>
+        </is>
+      </c>
+      <c r="D28" s="6" t="inlineStr">
+        <is>
+          <t>info@ladiri.it</t>
+        </is>
+      </c>
+      <c r="E28" s="6" t="inlineStr">
+        <is>
+          <t>Agenzia immobiliare</t>
+        </is>
+      </c>
+      <c r="F28" s="6" t="inlineStr">
+        <is>
+          <t>00fb9</t>
+        </is>
+      </c>
+      <c r="G28" s="6" t="inlineStr">
+        <is>
+          <t>https://agenzie-immobiliari.rilievocontract.it/?ref=00fb9</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="8" t="inlineStr">
+        <is>
+          <t>A28</t>
+        </is>
+      </c>
+      <c r="B29" s="8" t="inlineStr">
+        <is>
+          <t>P&amp;S Property &amp; Sales</t>
+        </is>
+      </c>
+      <c r="C29" s="8" t="inlineStr">
+        <is>
+          <t>Cagliari</t>
+        </is>
+      </c>
+      <c r="D29" s="8" t="inlineStr">
+        <is>
+          <t>pes.intermediazioni@gmail.com</t>
+        </is>
+      </c>
+      <c r="E29" s="8" t="inlineStr">
+        <is>
+          <t>Agenzia immobiliare</t>
+        </is>
+      </c>
+      <c r="F29" s="8" t="inlineStr">
+        <is>
+          <t>06282</t>
+        </is>
+      </c>
+      <c r="G29" s="8" t="inlineStr">
+        <is>
+          <t>https://agenzie-immobiliari.rilievocontract.it/?ref=06282</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="6" t="inlineStr">
+        <is>
+          <t>A29</t>
+        </is>
+      </c>
+      <c r="B30" s="6" t="inlineStr">
+        <is>
+          <t>Sardinia Real Estate</t>
+        </is>
+      </c>
+      <c r="C30" s="6" t="inlineStr">
+        <is>
+          <t>Quartucciu (CA)</t>
+        </is>
+      </c>
+      <c r="D30" s="6" t="inlineStr">
+        <is>
+          <t>info.sardiniare@gmail.com</t>
+        </is>
+      </c>
+      <c r="E30" s="6" t="inlineStr">
+        <is>
+          <t>Agenzia immobiliare</t>
+        </is>
+      </c>
+      <c r="F30" s="6" t="inlineStr">
+        <is>
+          <t>b5bfb</t>
+        </is>
+      </c>
+      <c r="G30" s="6" t="inlineStr">
+        <is>
+          <t>https://agenzie-immobiliari.rilievocontract.it/?ref=b5bfb</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="8" t="inlineStr">
+        <is>
+          <t>A30</t>
+        </is>
+      </c>
+      <c r="B31" s="8" t="inlineStr">
+        <is>
+          <t>Galleria d'Autore Immobili di Lusso</t>
+        </is>
+      </c>
+      <c r="C31" s="8" t="inlineStr">
+        <is>
+          <t>Sassari</t>
+        </is>
+      </c>
+      <c r="D31" s="8" t="inlineStr">
+        <is>
+          <t>info@galleriadautore.it</t>
+        </is>
+      </c>
+      <c r="E31" s="8" t="inlineStr">
+        <is>
+          <t>Agenzia immobiliare</t>
+        </is>
+      </c>
+      <c r="F31" s="8" t="inlineStr">
+        <is>
+          <t>3d65f</t>
+        </is>
+      </c>
+      <c r="G31" s="8" t="inlineStr">
+        <is>
+          <t>https://agenzie-immobiliari.rilievocontract.it/?ref=3d65f</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="6" t="inlineStr">
+        <is>
+          <t>A31</t>
+        </is>
+      </c>
+      <c r="B32" s="6" t="inlineStr">
+        <is>
+          <t>Vallebona Immobiliare</t>
+        </is>
+      </c>
+      <c r="C32" s="6" t="inlineStr">
+        <is>
+          <t>Cagliari / Chia / Villasimius</t>
+        </is>
+      </c>
+      <c r="D32" s="6" t="inlineStr">
+        <is>
+          <t>info@vallebonarealestate.it</t>
+        </is>
+      </c>
+      <c r="E32" s="6" t="inlineStr">
+        <is>
+          <t>Agenzia immobiliare</t>
+        </is>
+      </c>
+      <c r="F32" s="6" t="inlineStr">
+        <is>
+          <t>6c731</t>
+        </is>
+      </c>
+      <c r="G32" s="6" t="inlineStr">
+        <is>
+          <t>https://agenzie-immobiliari.rilievocontract.it/?ref=6c731</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="8" t="inlineStr">
+        <is>
+          <t>A32</t>
+        </is>
+      </c>
+      <c r="B33" s="8" t="inlineStr">
+        <is>
+          <t>L'Immobiliare Sardegna</t>
+        </is>
+      </c>
+      <c r="C33" s="8" t="inlineStr">
+        <is>
+          <t>Alghero (SS)</t>
+        </is>
+      </c>
+      <c r="D33" s="8" t="inlineStr">
+        <is>
+          <t>info@immobiliaresardegna.eu</t>
+        </is>
+      </c>
+      <c r="E33" s="8" t="inlineStr">
+        <is>
+          <t>Agenzia immobiliare</t>
+        </is>
+      </c>
+      <c r="F33" s="8" t="inlineStr">
+        <is>
+          <t>95611</t>
+        </is>
+      </c>
+      <c r="G33" s="8" t="inlineStr">
+        <is>
+          <t>https://agenzie-immobiliari.rilievocontract.it/?ref=95611</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:G20"/>
+  <autoFilter ref="A1:G33"/>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G2" r:id="rId1"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G3" r:id="rId2"/>

</xml_diff>

<commit_message>
Sincronizza lista contatti (74) e generatore agenzie da collaboratori, corregge bug citta/categoria in genera_generatore.py
- Lista_Contatti_Rilievo_Contract.xlsx: allineata a collaboratori, 42 architetti + 32 agenzie (13 nuove: Costa Smeralda, Cagliari, Sassari)
- generatore_email.html: rigenerato con le 32 agenzie, link su agenzie-immobiliari.rilievocontract.it
- genera_ref.py: porta il fix del foglio Riepilogo (vedi commit su collaboratori)
- genera_generatore.py: citta/categoria ora prese dalla lista contatti quando presenti, non piu' sempre e solo dal generatore esistente (bug: la lista le aveva gia' compilate per le 13 agenzie nuove, il generatore le scriveva comunque vuote)
</commit_message>
<xml_diff>
--- a/Lista_Contatti_Rilievo_Contract.xlsx
+++ b/Lista_Contatti_Rilievo_Contract.xlsx
@@ -13,7 +13,7 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Architetti'!$A$1:$G$43</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Agenzie immobiliari'!$A$1:$G$20</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Agenzie immobiliari'!$A$1:$G$33</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -22,36 +22,13 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="9">
+  <fonts count="7">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
       <color theme="1"/>
       <sz val="11"/>
       <scheme val="minor"/>
-    </font>
-    <font>
-      <name val="Arial"/>
-      <b val="1"/>
-      <color rgb="00F8F5EF"/>
-      <sz val="11"/>
-    </font>
-    <font>
-      <name val="Arial"/>
-      <color rgb="001C1C1A"/>
-      <sz val="10"/>
-    </font>
-    <font>
-      <name val="Arial"/>
-      <color rgb="000563C1"/>
-      <sz val="10"/>
-      <u val="single"/>
-    </font>
-    <font>
-      <name val="Arial"/>
-      <b val="1"/>
-      <color rgb="008A4B00"/>
-      <sz val="10"/>
     </font>
     <font>
       <name val="Arial"/>
@@ -68,17 +45,28 @@
     <font>
       <name val="Arial"/>
       <b val="1"/>
+      <color rgb="00F8F5EF"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <name val="Arial"/>
       <color rgb="001C1C1A"/>
       <sz val="10"/>
     </font>
     <font>
       <name val="Arial"/>
-      <i val="1"/>
-      <color rgb="007A7A75"/>
-      <sz val="9"/>
+      <b val="1"/>
+      <color rgb="001C1C1A"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <color rgb="000563C1"/>
+      <sz val="10"/>
+      <u val="single"/>
     </font>
   </fonts>
-  <fills count="5">
+  <fills count="4">
     <fill>
       <patternFill/>
     </fill>
@@ -95,12 +83,6 @@
       <patternFill patternType="solid">
         <fgColor rgb="00F8F5EF"/>
         <bgColor rgb="00F8F5EF"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00FCE8D6"/>
-        <bgColor rgb="00FCE8D6"/>
       </patternFill>
     </fill>
   </fills>
@@ -130,38 +112,23 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="15">
+  <cellXfs count="10">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
   </cellXfs>
@@ -238,21 +205,6 @@
     </indexedColors>
   </colors>
 </styleSheet>
-</file>
-
-<file path=xl/comments/comment1.xml><?xml version="1.0" encoding="utf-8"?>
-<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <authors>
-    <author>Rilievo Contract</author>
-  </authors>
-  <commentList>
-    <comment ref="B25" authorId="0" shapeId="0">
-      <text>
-        <t>CONFERMATO 20/07/2026: l'email con ref e7f0f e' stata spedita per errore sia ad Ark.e Studio sia a Studio Figus. I dati GA4 per e7f0f nel periodo di sovrapposizione sono contaminati e non recuperabili. Nuovo ref casuale assegnato per l'uso futuro: consigliato reinvio a gianluca@studiofigus.it con il link corretto.</t>
-      </text>
-    </comment>
-  </commentList>
-</comments>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -544,7 +496,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B10"/>
+  <dimension ref="A1:B7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="34" customWidth="1" min="1" max="1"/>
@@ -594,7 +546,7 @@
         </is>
       </c>
       <c r="B6" s="4" t="n">
-        <v>19</v>
+        <v>32</v>
       </c>
     </row>
     <row r="7">
@@ -604,20 +556,12 @@
         </is>
       </c>
       <c r="B7" s="5" t="n">
-        <v>61</v>
-      </c>
-    </row>
-    <row r="10" ht="90" customHeight="1">
-      <c r="A10" s="6" t="inlineStr">
-        <is>
-          <t>Nota metodo: 22 architetti sui 42 hanno il ref gia' confermato dal generatore email attivo (intoccati). 19 architetti nuovi hanno ref deterministico md5(email)[:5], verificato senza collisioni. 1 riga (Studio Figus, evidenziata in arancione nella tab Architetti) aveva un ref duplicato di Ark.e Studio nella lista originale: le e' stato assegnato un ref provvisorio, da confermare se non e' gia' stato spedito via email con il codice errato. Le 19 agenzie immobiliari hanno ref nuovi, verificati contro tutti i 42 ref architetti: nessuna collisione.</t>
-        </is>
+        <v>74</v>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="3">
+  <mergeCells count="2">
     <mergeCell ref="A2:B2"/>
-    <mergeCell ref="A10:B10"/>
     <mergeCell ref="A1:B1"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -633,1527 +577,1527 @@
   <dimension ref="A1:G43"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="8" customWidth="1" min="1" max="1"/>
-    <col width="34" customWidth="1" min="2" max="2"/>
-    <col width="24" customWidth="1" min="3" max="3"/>
-    <col width="32" customWidth="1" min="4" max="4"/>
-    <col width="26" customWidth="1" min="5" max="5"/>
-    <col width="10" customWidth="1" min="6" max="6"/>
+    <col width="30" customWidth="1" min="1" max="1"/>
+    <col width="30" customWidth="1" min="2" max="2"/>
+    <col width="30" customWidth="1" min="3" max="3"/>
+    <col width="30" customWidth="1" min="4" max="4"/>
+    <col width="30" customWidth="1" min="5" max="5"/>
+    <col width="30" customWidth="1" min="6" max="6"/>
     <col width="52" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
-    <row r="1" ht="20" customHeight="1">
-      <c r="A1" s="7" t="inlineStr">
-        <is>
-          <t>ID</t>
-        </is>
-      </c>
-      <c r="B1" s="7" t="inlineStr">
+    <row r="1">
+      <c r="A1" s="3" t="inlineStr">
+        <is>
+          <t>Id</t>
+        </is>
+      </c>
+      <c r="B1" s="3" t="inlineStr">
         <is>
           <t>Nome</t>
         </is>
       </c>
-      <c r="C1" s="7" t="inlineStr">
-        <is>
-          <t>Città</t>
-        </is>
-      </c>
-      <c r="D1" s="7" t="inlineStr">
+      <c r="C1" s="3" t="inlineStr">
+        <is>
+          <t>Citta</t>
+        </is>
+      </c>
+      <c r="D1" s="3" t="inlineStr">
         <is>
           <t>Email</t>
         </is>
       </c>
-      <c r="E1" s="7" t="inlineStr">
+      <c r="E1" s="3" t="inlineStr">
         <is>
           <t>Categoria</t>
         </is>
       </c>
-      <c r="F1" s="7" t="inlineStr">
+      <c r="F1" s="3" t="inlineStr">
         <is>
           <t>Ref</t>
         </is>
       </c>
-      <c r="G1" s="7" t="inlineStr">
-        <is>
-          <t>Link presentazione</t>
+      <c r="G1" s="3" t="inlineStr">
+        <is>
+          <t>Link</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="8" t="inlineStr">
+      <c r="A2" s="6" t="inlineStr">
         <is>
           <t>1</t>
         </is>
       </c>
-      <c r="B2" s="8" t="inlineStr">
+      <c r="B2" s="6" t="inlineStr">
         <is>
           <t>C+C04 Architetti</t>
         </is>
       </c>
-      <c r="C2" s="8" t="inlineStr">
+      <c r="C2" s="6" t="inlineStr">
         <is>
           <t>Cagliari</t>
         </is>
       </c>
-      <c r="D2" s="8" t="inlineStr">
+      <c r="D2" s="6" t="inlineStr">
         <is>
           <t>info@cc04.net</t>
         </is>
       </c>
-      <c r="E2" s="8" t="inlineStr">
+      <c r="E2" s="6" t="inlineStr">
         <is>
           <t>Hotel, Ristoranti, Retail</t>
         </is>
       </c>
-      <c r="F2" s="8" t="inlineStr">
+      <c r="F2" s="6" t="inlineStr">
         <is>
           <t>8fa8d</t>
         </is>
       </c>
-      <c r="G2" s="9" t="inlineStr">
+      <c r="G2" s="7" t="inlineStr">
         <is>
           <t>https://presentazione.rilievocontract.it/?ref=8fa8d</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="10" t="inlineStr">
+      <c r="A3" s="8" t="inlineStr">
         <is>
           <t>2</t>
         </is>
       </c>
-      <c r="B3" s="10" t="inlineStr">
+      <c r="B3" s="8" t="inlineStr">
         <is>
           <t>ALO Architettura</t>
         </is>
       </c>
-      <c r="C3" s="10" t="inlineStr">
+      <c r="C3" s="8" t="inlineStr">
         <is>
           <t>Cagliari</t>
         </is>
       </c>
-      <c r="D3" s="10" t="inlineStr">
+      <c r="D3" s="8" t="inlineStr">
         <is>
           <t>info@alo-architettura.com</t>
         </is>
       </c>
-      <c r="E3" s="10" t="inlineStr">
+      <c r="E3" s="8" t="inlineStr">
         <is>
           <t>Ricettivo, Retail, Ville</t>
         </is>
       </c>
-      <c r="F3" s="10" t="inlineStr">
+      <c r="F3" s="8" t="inlineStr">
         <is>
           <t>cf458</t>
         </is>
       </c>
-      <c r="G3" s="11" t="inlineStr">
+      <c r="G3" s="9" t="inlineStr">
         <is>
           <t>https://presentazione.rilievocontract.it/?ref=cf458</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="8" t="inlineStr">
+      <c r="A4" s="6" t="inlineStr">
         <is>
           <t>3</t>
         </is>
       </c>
-      <c r="B4" s="8" t="inlineStr">
+      <c r="B4" s="6" t="inlineStr">
         <is>
           <t>Studio Tramas</t>
         </is>
       </c>
-      <c r="C4" s="8" t="inlineStr">
+      <c r="C4" s="6" t="inlineStr">
         <is>
           <t>Cagliari</t>
         </is>
       </c>
-      <c r="D4" s="8" t="inlineStr">
+      <c r="D4" s="6" t="inlineStr">
         <is>
           <t>info@studiotramas.com</t>
         </is>
       </c>
-      <c r="E4" s="8" t="inlineStr">
+      <c r="E4" s="6" t="inlineStr">
         <is>
           <t>Ricettivo, Retail, Interior</t>
         </is>
       </c>
-      <c r="F4" s="8" t="inlineStr">
+      <c r="F4" s="6" t="inlineStr">
         <is>
           <t>04cb2</t>
         </is>
       </c>
-      <c r="G4" s="9" t="inlineStr">
+      <c r="G4" s="7" t="inlineStr">
         <is>
           <t>https://presentazione.rilievocontract.it/?ref=04cb2</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="10" t="inlineStr">
+      <c r="A5" s="8" t="inlineStr">
         <is>
           <t>4</t>
         </is>
       </c>
-      <c r="B5" s="10" t="inlineStr">
+      <c r="B5" s="8" t="inlineStr">
         <is>
           <t>MUCA Architettura</t>
         </is>
       </c>
-      <c r="C5" s="10" t="inlineStr">
+      <c r="C5" s="8" t="inlineStr">
         <is>
           <t>Cagliari</t>
         </is>
       </c>
-      <c r="D5" s="10" t="inlineStr">
+      <c r="D5" s="8" t="inlineStr">
         <is>
           <t>info@mucaarchitettura.com</t>
         </is>
       </c>
-      <c r="E5" s="10" t="inlineStr">
+      <c r="E5" s="8" t="inlineStr">
         <is>
           <t>Retail, Exhibit</t>
         </is>
       </c>
-      <c r="F5" s="10" t="inlineStr">
+      <c r="F5" s="8" t="inlineStr">
         <is>
           <t>e28a2</t>
         </is>
       </c>
-      <c r="G5" s="11" t="inlineStr">
+      <c r="G5" s="9" t="inlineStr">
         <is>
           <t>https://presentazione.rilievocontract.it/?ref=e28a2</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="8" t="inlineStr">
+      <c r="A6" s="6" t="inlineStr">
         <is>
           <t>5</t>
         </is>
       </c>
-      <c r="B6" s="8" t="inlineStr">
+      <c r="B6" s="6" t="inlineStr">
         <is>
           <t>essequadro|p</t>
         </is>
       </c>
-      <c r="C6" s="8" t="inlineStr">
+      <c r="C6" s="6" t="inlineStr">
         <is>
           <t>Cagliari</t>
         </is>
       </c>
-      <c r="D6" s="8" t="inlineStr">
+      <c r="D6" s="6" t="inlineStr">
         <is>
           <t>info@essequadrop.com</t>
         </is>
       </c>
-      <c r="E6" s="8" t="inlineStr">
+      <c r="E6" s="6" t="inlineStr">
         <is>
           <t>Hospitality, Lighting</t>
         </is>
       </c>
-      <c r="F6" s="8" t="inlineStr">
+      <c r="F6" s="6" t="inlineStr">
         <is>
           <t>0a85e</t>
         </is>
       </c>
-      <c r="G6" s="9" t="inlineStr">
+      <c r="G6" s="7" t="inlineStr">
         <is>
           <t>https://presentazione.rilievocontract.it/?ref=0a85e</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="10" t="inlineStr">
+      <c r="A7" s="8" t="inlineStr">
         <is>
           <t>6</t>
         </is>
       </c>
-      <c r="B7" s="10" t="inlineStr">
+      <c r="B7" s="8" t="inlineStr">
         <is>
           <t>Formaa Studio</t>
         </is>
       </c>
-      <c r="C7" s="10" t="inlineStr">
+      <c r="C7" s="8" t="inlineStr">
         <is>
           <t>Cagliari</t>
         </is>
       </c>
-      <c r="D7" s="10" t="inlineStr">
+      <c r="D7" s="8" t="inlineStr">
         <is>
           <t>info@formaa.it</t>
         </is>
       </c>
-      <c r="E7" s="10" t="inlineStr">
+      <c r="E7" s="8" t="inlineStr">
         <is>
           <t>Ricettivo, Locali</t>
         </is>
       </c>
-      <c r="F7" s="10" t="inlineStr">
+      <c r="F7" s="8" t="inlineStr">
         <is>
           <t>f815c</t>
         </is>
       </c>
-      <c r="G7" s="11" t="inlineStr">
+      <c r="G7" s="9" t="inlineStr">
         <is>
           <t>https://presentazione.rilievocontract.it/?ref=f815c</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="8" t="inlineStr">
+      <c r="A8" s="6" t="inlineStr">
         <is>
           <t>7</t>
         </is>
       </c>
-      <c r="B8" s="8" t="inlineStr">
+      <c r="B8" s="6" t="inlineStr">
         <is>
           <t>Orma Studio</t>
         </is>
       </c>
-      <c r="C8" s="8" t="inlineStr">
+      <c r="C8" s="6" t="inlineStr">
         <is>
           <t>Cagliari</t>
         </is>
       </c>
-      <c r="D8" s="8" t="inlineStr">
+      <c r="D8" s="6" t="inlineStr">
         <is>
           <t>info@ormastudio.it</t>
         </is>
       </c>
-      <c r="E8" s="8" t="inlineStr">
+      <c r="E8" s="6" t="inlineStr">
         <is>
           <t>Commerciale, Interior</t>
         </is>
       </c>
-      <c r="F8" s="8" t="inlineStr">
+      <c r="F8" s="6" t="inlineStr">
         <is>
           <t>4d5d7</t>
         </is>
       </c>
-      <c r="G8" s="9" t="inlineStr">
+      <c r="G8" s="7" t="inlineStr">
         <is>
           <t>https://presentazione.rilievocontract.it/?ref=4d5d7</t>
         </is>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="10" t="inlineStr">
+      <c r="A9" s="8" t="inlineStr">
         <is>
           <t>9</t>
         </is>
       </c>
-      <c r="B9" s="10" t="inlineStr">
+      <c r="B9" s="8" t="inlineStr">
         <is>
           <t>Studio Rifinito — Lara Serra</t>
         </is>
       </c>
-      <c r="C9" s="10" t="inlineStr">
+      <c r="C9" s="8" t="inlineStr">
         <is>
           <t>Cagliari</t>
         </is>
       </c>
-      <c r="D9" s="10" t="inlineStr">
+      <c r="D9" s="8" t="inlineStr">
         <is>
           <t>info@studiorifinito.it</t>
         </is>
       </c>
-      <c r="E9" s="10" t="inlineStr">
+      <c r="E9" s="8" t="inlineStr">
         <is>
           <t>Interior, Residenziale</t>
         </is>
       </c>
-      <c r="F9" s="10" t="inlineStr">
+      <c r="F9" s="8" t="inlineStr">
         <is>
           <t>dc232</t>
         </is>
       </c>
-      <c r="G9" s="11" t="inlineStr">
+      <c r="G9" s="9" t="inlineStr">
         <is>
           <t>https://presentazione.rilievocontract.it/?ref=dc232</t>
         </is>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="8" t="inlineStr">
+      <c r="A10" s="6" t="inlineStr">
         <is>
           <t>10</t>
         </is>
       </c>
-      <c r="B10" s="8" t="inlineStr">
+      <c r="B10" s="6" t="inlineStr">
         <is>
           <t>domECO Studio</t>
         </is>
       </c>
-      <c r="C10" s="8" t="inlineStr">
+      <c r="C10" s="6" t="inlineStr">
         <is>
           <t>Cagliari / Sassari</t>
         </is>
       </c>
-      <c r="D10" s="8" t="inlineStr">
+      <c r="D10" s="6" t="inlineStr">
         <is>
           <t>info@domecostudio.it</t>
         </is>
       </c>
-      <c r="E10" s="8" t="inlineStr">
+      <c r="E10" s="6" t="inlineStr">
         <is>
           <t>Residenziale, Interior</t>
         </is>
       </c>
-      <c r="F10" s="8" t="inlineStr">
+      <c r="F10" s="6" t="inlineStr">
         <is>
           <t>53775</t>
         </is>
       </c>
-      <c r="G10" s="9" t="inlineStr">
+      <c r="G10" s="7" t="inlineStr">
         <is>
           <t>https://presentazione.rilievocontract.it/?ref=53775</t>
         </is>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="10" t="inlineStr">
+      <c r="A11" s="8" t="inlineStr">
         <is>
           <t>21</t>
         </is>
       </c>
-      <c r="B11" s="10" t="inlineStr">
+      <c r="B11" s="8" t="inlineStr">
         <is>
           <t>Studio Careddu</t>
         </is>
       </c>
-      <c r="C11" s="10" t="inlineStr">
+      <c r="C11" s="8" t="inlineStr">
         <is>
           <t>Olbia / Costa Smeralda</t>
         </is>
       </c>
-      <c r="D11" s="10" t="inlineStr">
+      <c r="D11" s="8" t="inlineStr">
         <is>
           <t>info@architettocareddu.it</t>
         </is>
       </c>
-      <c r="E11" s="10" t="inlineStr">
+      <c r="E11" s="8" t="inlineStr">
         <is>
           <t>Ville pregio, Ricettivo</t>
         </is>
       </c>
-      <c r="F11" s="10" t="inlineStr">
+      <c r="F11" s="8" t="inlineStr">
         <is>
           <t>7c83b</t>
         </is>
       </c>
-      <c r="G11" s="11" t="inlineStr">
+      <c r="G11" s="9" t="inlineStr">
         <is>
           <t>https://presentazione.rilievocontract.it/?ref=7c83b</t>
         </is>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="8" t="inlineStr">
+      <c r="A12" s="6" t="inlineStr">
         <is>
           <t>22</t>
         </is>
       </c>
-      <c r="B12" s="8" t="inlineStr">
+      <c r="B12" s="6" t="inlineStr">
         <is>
           <t>Marcello Scano Interior Design</t>
         </is>
       </c>
-      <c r="C12" s="8" t="inlineStr">
+      <c r="C12" s="6" t="inlineStr">
         <is>
           <t>Olbia</t>
         </is>
       </c>
-      <c r="D12" s="8" t="inlineStr">
+      <c r="D12" s="6" t="inlineStr">
         <is>
           <t>info@marcelloscano.it</t>
         </is>
       </c>
-      <c r="E12" s="8" t="inlineStr">
+      <c r="E12" s="6" t="inlineStr">
         <is>
           <t>Hospitality, Ville</t>
         </is>
       </c>
-      <c r="F12" s="8" t="inlineStr">
+      <c r="F12" s="6" t="inlineStr">
         <is>
           <t>90a53</t>
         </is>
       </c>
-      <c r="G12" s="9" t="inlineStr">
+      <c r="G12" s="7" t="inlineStr">
         <is>
           <t>https://presentazione.rilievocontract.it/?ref=90a53</t>
         </is>
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="10" t="inlineStr">
+      <c r="A13" s="8" t="inlineStr">
         <is>
           <t>23</t>
         </is>
       </c>
-      <c r="B13" s="10" t="inlineStr">
+      <c r="B13" s="8" t="inlineStr">
         <is>
           <t>Antonello Carta Interior Design</t>
         </is>
       </c>
-      <c r="C13" s="10" t="inlineStr">
+      <c r="C13" s="8" t="inlineStr">
         <is>
           <t>Olbia</t>
         </is>
       </c>
-      <c r="D13" s="10" t="inlineStr">
+      <c r="D13" s="8" t="inlineStr">
         <is>
           <t>info@antonellocarta.com</t>
         </is>
       </c>
-      <c r="E13" s="10" t="inlineStr">
+      <c r="E13" s="8" t="inlineStr">
         <is>
           <t>Ristoranti, Retail</t>
         </is>
       </c>
-      <c r="F13" s="10" t="inlineStr">
+      <c r="F13" s="8" t="inlineStr">
         <is>
           <t>aa5ba</t>
         </is>
       </c>
-      <c r="G13" s="11" t="inlineStr">
+      <c r="G13" s="9" t="inlineStr">
         <is>
           <t>https://presentazione.rilievocontract.it/?ref=aa5ba</t>
         </is>
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="8" t="inlineStr">
+      <c r="A14" s="6" t="inlineStr">
         <is>
           <t>24</t>
         </is>
       </c>
-      <c r="B14" s="8" t="inlineStr">
+      <c r="B14" s="6" t="inlineStr">
         <is>
           <t>Studio Miniaci e Associati</t>
         </is>
       </c>
-      <c r="C14" s="8" t="inlineStr">
+      <c r="C14" s="6" t="inlineStr">
         <is>
           <t>Olbia / Costa Smeralda</t>
         </is>
       </c>
-      <c r="D14" s="8" t="inlineStr">
+      <c r="D14" s="6" t="inlineStr">
         <is>
           <t>info@architettimea.it</t>
         </is>
       </c>
-      <c r="E14" s="8" t="inlineStr">
+      <c r="E14" s="6" t="inlineStr">
         <is>
           <t>Hospitality, Residenziale</t>
         </is>
       </c>
-      <c r="F14" s="8" t="inlineStr">
+      <c r="F14" s="6" t="inlineStr">
         <is>
           <t>7b647</t>
         </is>
       </c>
-      <c r="G14" s="9" t="inlineStr">
+      <c r="G14" s="7" t="inlineStr">
         <is>
           <t>https://presentazione.rilievocontract.it/?ref=7b647</t>
         </is>
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="10" t="inlineStr">
+      <c r="A15" s="8" t="inlineStr">
         <is>
           <t>25</t>
         </is>
       </c>
-      <c r="B15" s="10" t="inlineStr">
+      <c r="B15" s="8" t="inlineStr">
         <is>
           <t>FabDesign Interiors</t>
         </is>
       </c>
-      <c r="C15" s="10" t="inlineStr">
+      <c r="C15" s="8" t="inlineStr">
         <is>
           <t>Olbia</t>
         </is>
       </c>
-      <c r="D15" s="10" t="inlineStr">
+      <c r="D15" s="8" t="inlineStr">
         <is>
           <t>info@fabdesigninteriors.com</t>
         </is>
       </c>
-      <c r="E15" s="10" t="inlineStr">
+      <c r="E15" s="8" t="inlineStr">
         <is>
           <t>Bar/Ristoranti, Retail</t>
         </is>
       </c>
-      <c r="F15" s="10" t="inlineStr">
+      <c r="F15" s="8" t="inlineStr">
         <is>
           <t>7b3cb</t>
         </is>
       </c>
-      <c r="G15" s="11" t="inlineStr">
+      <c r="G15" s="9" t="inlineStr">
         <is>
           <t>https://presentazione.rilievocontract.it/?ref=7b3cb</t>
         </is>
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="8" t="inlineStr">
+      <c r="A16" s="6" t="inlineStr">
         <is>
           <t>26</t>
         </is>
       </c>
-      <c r="B16" s="8" t="inlineStr">
+      <c r="B16" s="6" t="inlineStr">
         <is>
           <t>Studio Olivieri Architetti</t>
         </is>
       </c>
-      <c r="C16" s="8" t="inlineStr">
+      <c r="C16" s="6" t="inlineStr">
         <is>
           <t>Arzachena / Costa Smeralda</t>
         </is>
       </c>
-      <c r="D16" s="8" t="inlineStr">
+      <c r="D16" s="6" t="inlineStr">
         <is>
           <t>info@olivieriarchitetti.it</t>
         </is>
       </c>
-      <c r="E16" s="8" t="inlineStr">
+      <c r="E16" s="6" t="inlineStr">
         <is>
           <t>Ville lusso, Ricettivo</t>
         </is>
       </c>
-      <c r="F16" s="8" t="inlineStr">
+      <c r="F16" s="6" t="inlineStr">
         <is>
           <t>99814</t>
         </is>
       </c>
-      <c r="G16" s="9" t="inlineStr">
+      <c r="G16" s="7" t="inlineStr">
         <is>
           <t>https://presentazione.rilievocontract.it/?ref=99814</t>
         </is>
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="10" t="inlineStr">
+      <c r="A17" s="8" t="inlineStr">
         <is>
           <t>28</t>
         </is>
       </c>
-      <c r="B17" s="10" t="inlineStr">
+      <c r="B17" s="8" t="inlineStr">
         <is>
           <t>Pitzus Group</t>
         </is>
       </c>
-      <c r="C17" s="10" t="inlineStr">
+      <c r="C17" s="8" t="inlineStr">
         <is>
           <t>Costa Smeralda</t>
         </is>
       </c>
-      <c r="D17" s="10" t="inlineStr">
+      <c r="D17" s="8" t="inlineStr">
         <is>
           <t>info@pitzusgroup.com</t>
         </is>
       </c>
-      <c r="E17" s="10" t="inlineStr">
+      <c r="E17" s="8" t="inlineStr">
         <is>
           <t>Ville lusso</t>
         </is>
       </c>
-      <c r="F17" s="10" t="inlineStr">
+      <c r="F17" s="8" t="inlineStr">
         <is>
           <t>3b50d</t>
         </is>
       </c>
-      <c r="G17" s="11" t="inlineStr">
+      <c r="G17" s="9" t="inlineStr">
         <is>
           <t>https://presentazione.rilievocontract.it/?ref=3b50d</t>
         </is>
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="8" t="inlineStr">
+      <c r="A18" s="6" t="inlineStr">
         <is>
           <t>29</t>
         </is>
       </c>
-      <c r="B18" s="8" t="inlineStr">
+      <c r="B18" s="6" t="inlineStr">
         <is>
           <t>Architettare &amp; Design Srl</t>
         </is>
       </c>
-      <c r="C18" s="8" t="inlineStr">
+      <c r="C18" s="6" t="inlineStr">
         <is>
           <t>Olbia</t>
         </is>
       </c>
-      <c r="D18" s="8" t="inlineStr">
+      <c r="D18" s="6" t="inlineStr">
         <is>
           <t>info@architettaredesignsrl.it</t>
         </is>
       </c>
-      <c r="E18" s="8" t="inlineStr">
+      <c r="E18" s="6" t="inlineStr">
         <is>
           <t>Costa Smeralda, Ville</t>
         </is>
       </c>
-      <c r="F18" s="8" t="inlineStr">
+      <c r="F18" s="6" t="inlineStr">
         <is>
           <t>60531</t>
         </is>
       </c>
-      <c r="G18" s="9" t="inlineStr">
+      <c r="G18" s="7" t="inlineStr">
         <is>
           <t>https://presentazione.rilievocontract.it/?ref=60531</t>
         </is>
       </c>
     </row>
     <row r="19">
-      <c r="A19" s="10" t="inlineStr">
+      <c r="A19" s="8" t="inlineStr">
         <is>
           <t>31</t>
         </is>
       </c>
-      <c r="B19" s="10" t="inlineStr">
+      <c r="B19" s="8" t="inlineStr">
         <is>
           <t>Studio Arch. Pietro Giordo</t>
         </is>
       </c>
-      <c r="C19" s="10" t="inlineStr">
+      <c r="C19" s="8" t="inlineStr">
         <is>
           <t>Arzachena / Porto Cervo</t>
         </is>
       </c>
-      <c r="D19" s="10" t="inlineStr">
+      <c r="D19" s="8" t="inlineStr">
         <is>
           <t>info@pietrogiordo.it</t>
         </is>
       </c>
-      <c r="E19" s="10" t="inlineStr">
+      <c r="E19" s="8" t="inlineStr">
         <is>
           <t>Ville storiche, Ricettivo</t>
         </is>
       </c>
-      <c r="F19" s="10" t="inlineStr">
+      <c r="F19" s="8" t="inlineStr">
         <is>
           <t>8a2a4</t>
         </is>
       </c>
-      <c r="G19" s="11" t="inlineStr">
+      <c r="G19" s="9" t="inlineStr">
         <is>
           <t>https://presentazione.rilievocontract.it/?ref=8a2a4</t>
         </is>
       </c>
     </row>
     <row r="20">
-      <c r="A20" s="8" t="inlineStr">
+      <c r="A20" s="6" t="inlineStr">
         <is>
           <t>34</t>
         </is>
       </c>
-      <c r="B20" s="8" t="inlineStr">
+      <c r="B20" s="6" t="inlineStr">
         <is>
           <t>Officina29 Architetti</t>
         </is>
       </c>
-      <c r="C20" s="8" t="inlineStr">
+      <c r="C20" s="6" t="inlineStr">
         <is>
           <t>Sassari / Olbia</t>
         </is>
       </c>
-      <c r="D20" s="8" t="inlineStr">
+      <c r="D20" s="6" t="inlineStr">
         <is>
           <t>info@officina29architetti.it</t>
         </is>
       </c>
-      <c r="E20" s="8" t="inlineStr">
+      <c r="E20" s="6" t="inlineStr">
         <is>
           <t>Interior, Residenziale</t>
         </is>
       </c>
-      <c r="F20" s="8" t="inlineStr">
+      <c r="F20" s="6" t="inlineStr">
         <is>
           <t>82701</t>
         </is>
       </c>
-      <c r="G20" s="9" t="inlineStr">
+      <c r="G20" s="7" t="inlineStr">
         <is>
           <t>https://presentazione.rilievocontract.it/?ref=82701</t>
         </is>
       </c>
     </row>
     <row r="21">
-      <c r="A21" s="10" t="inlineStr">
+      <c r="A21" s="8" t="inlineStr">
         <is>
           <t>37</t>
         </is>
       </c>
-      <c r="B21" s="10" t="inlineStr">
+      <c r="B21" s="8" t="inlineStr">
         <is>
           <t>ADM Progetti</t>
         </is>
       </c>
-      <c r="C21" s="10" t="inlineStr">
+      <c r="C21" s="8" t="inlineStr">
         <is>
           <t>Sassari</t>
         </is>
       </c>
-      <c r="D21" s="10" t="inlineStr">
+      <c r="D21" s="8" t="inlineStr">
         <is>
           <t>info@admprogetti.it</t>
         </is>
       </c>
-      <c r="E21" s="10" t="inlineStr">
+      <c r="E21" s="8" t="inlineStr">
         <is>
           <t>Residenziale, Commerciale</t>
         </is>
       </c>
-      <c r="F21" s="10" t="inlineStr">
+      <c r="F21" s="8" t="inlineStr">
         <is>
           <t>4959f</t>
         </is>
       </c>
-      <c r="G21" s="11" t="inlineStr">
+      <c r="G21" s="9" t="inlineStr">
         <is>
           <t>https://presentazione.rilievocontract.it/?ref=4959f</t>
         </is>
       </c>
     </row>
     <row r="22">
-      <c r="A22" s="8" t="inlineStr">
+      <c r="A22" s="6" t="inlineStr">
         <is>
           <t>38</t>
         </is>
       </c>
-      <c r="B22" s="8" t="inlineStr">
+      <c r="B22" s="6" t="inlineStr">
         <is>
           <t>Studio Cartamantiglia</t>
         </is>
       </c>
-      <c r="C22" s="8" t="inlineStr">
+      <c r="C22" s="6" t="inlineStr">
         <is>
           <t>Alghero</t>
         </is>
       </c>
-      <c r="D22" s="8" t="inlineStr">
+      <c r="D22" s="6" t="inlineStr">
         <is>
           <t>info@federicocartamantiglia.com</t>
         </is>
       </c>
-      <c r="E22" s="8" t="inlineStr">
+      <c r="E22" s="6" t="inlineStr">
         <is>
           <t>Hotel, Beach bar, Retail</t>
         </is>
       </c>
-      <c r="F22" s="8" t="inlineStr">
+      <c r="F22" s="6" t="inlineStr">
         <is>
           <t>80ed1</t>
         </is>
       </c>
-      <c r="G22" s="9" t="inlineStr">
+      <c r="G22" s="7" t="inlineStr">
         <is>
           <t>https://presentazione.rilievocontract.it/?ref=80ed1</t>
         </is>
       </c>
     </row>
     <row r="23">
-      <c r="A23" s="10" t="inlineStr">
+      <c r="A23" s="8" t="inlineStr">
         <is>
           <t>39</t>
         </is>
       </c>
-      <c r="B23" s="10" t="inlineStr">
+      <c r="B23" s="8" t="inlineStr">
         <is>
           <t>DESINNU Studio</t>
         </is>
       </c>
-      <c r="C23" s="10" t="inlineStr">
+      <c r="C23" s="8" t="inlineStr">
         <is>
           <t>Alghero</t>
         </is>
       </c>
-      <c r="D23" s="10" t="inlineStr">
+      <c r="D23" s="8" t="inlineStr">
         <is>
           <t>info@architettura-alghero.it</t>
         </is>
       </c>
-      <c r="E23" s="10" t="inlineStr">
+      <c r="E23" s="8" t="inlineStr">
         <is>
           <t>Commerciale, Residenziale</t>
         </is>
       </c>
-      <c r="F23" s="10" t="inlineStr">
+      <c r="F23" s="8" t="inlineStr">
         <is>
           <t>0b9cc</t>
         </is>
       </c>
-      <c r="G23" s="11" t="inlineStr">
+      <c r="G23" s="9" t="inlineStr">
         <is>
           <t>https://presentazione.rilievocontract.it/?ref=0b9cc</t>
         </is>
       </c>
     </row>
     <row r="24">
-      <c r="A24" s="8" t="inlineStr">
+      <c r="A24" s="6" t="inlineStr">
         <is>
           <t>40</t>
         </is>
       </c>
-      <c r="B24" s="8" t="inlineStr">
+      <c r="B24" s="6" t="inlineStr">
         <is>
           <t>Ark.e Studio</t>
         </is>
       </c>
-      <c r="C24" s="8" t="inlineStr">
+      <c r="C24" s="6" t="inlineStr">
         <is>
           <t>Alghero</t>
         </is>
       </c>
-      <c r="D24" s="8" t="inlineStr">
+      <c r="D24" s="6" t="inlineStr">
         <is>
           <t>info@arkestudio.eu</t>
         </is>
       </c>
-      <c r="E24" s="8" t="inlineStr">
+      <c r="E24" s="6" t="inlineStr">
         <is>
           <t>Residenziale, Ricettivo</t>
         </is>
       </c>
-      <c r="F24" s="8" t="inlineStr">
+      <c r="F24" s="6" t="inlineStr">
         <is>
           <t>e7f0f</t>
         </is>
       </c>
-      <c r="G24" s="9" t="inlineStr">
+      <c r="G24" s="7" t="inlineStr">
         <is>
           <t>https://presentazione.rilievocontract.it/?ref=e7f0f</t>
         </is>
       </c>
     </row>
     <row r="25">
-      <c r="A25" s="12" t="inlineStr">
+      <c r="A25" s="8" t="inlineStr">
         <is>
           <t>100</t>
         </is>
       </c>
-      <c r="B25" s="12" t="inlineStr">
+      <c r="B25" s="8" t="inlineStr">
         <is>
           <t>Studio Figus</t>
         </is>
       </c>
-      <c r="C25" s="12" t="inlineStr"/>
-      <c r="D25" s="12" t="inlineStr">
+      <c r="C25" s="8" t="inlineStr"/>
+      <c r="D25" s="8" t="inlineStr">
         <is>
           <t>gianluca@studiofigus.it</t>
         </is>
       </c>
-      <c r="E25" s="12" t="inlineStr">
+      <c r="E25" s="8" t="inlineStr">
         <is>
           <t>Architetto</t>
         </is>
       </c>
-      <c r="F25" s="13" t="inlineStr">
+      <c r="F25" s="8" t="inlineStr">
         <is>
           <t>4e268</t>
         </is>
       </c>
-      <c r="G25" s="14" t="inlineStr">
-        <is>
-          <t>https://collaboratori.rilievocontract.it/?ref=4e268</t>
+      <c r="G25" s="9" t="inlineStr">
+        <is>
+          <t>https://presentazione.rilievocontract.it/?ref=4e268</t>
         </is>
       </c>
     </row>
     <row r="26">
-      <c r="A26" s="8" t="inlineStr">
+      <c r="A26" s="6" t="inlineStr">
         <is>
           <t>101</t>
         </is>
       </c>
-      <c r="B26" s="8" t="inlineStr">
+      <c r="B26" s="6" t="inlineStr">
         <is>
           <t>Arch. Davide Fancello</t>
         </is>
       </c>
-      <c r="C26" s="8" t="inlineStr"/>
-      <c r="D26" s="8" t="inlineStr">
+      <c r="C26" s="6" t="inlineStr"/>
+      <c r="D26" s="6" t="inlineStr">
         <is>
           <t>info@davidefancello.it</t>
         </is>
       </c>
-      <c r="E26" s="8" t="inlineStr">
+      <c r="E26" s="6" t="inlineStr">
         <is>
           <t>Architetto</t>
         </is>
       </c>
-      <c r="F26" s="8" t="inlineStr">
+      <c r="F26" s="6" t="inlineStr">
         <is>
           <t>d59d8</t>
         </is>
       </c>
-      <c r="G26" s="9" t="inlineStr">
-        <is>
-          <t>https://collaboratori.rilievocontract.it/?ref=d59d8</t>
+      <c r="G26" s="7" t="inlineStr">
+        <is>
+          <t>https://presentazione.rilievocontract.it/?ref=d59d8</t>
         </is>
       </c>
     </row>
     <row r="27">
-      <c r="A27" s="10" t="inlineStr">
+      <c r="A27" s="8" t="inlineStr">
         <is>
           <t>102</t>
         </is>
       </c>
-      <c r="B27" s="10" t="inlineStr">
+      <c r="B27" s="8" t="inlineStr">
         <is>
           <t>Studio Arch. Colomo</t>
         </is>
       </c>
-      <c r="C27" s="10" t="inlineStr"/>
-      <c r="D27" s="10" t="inlineStr">
+      <c r="C27" s="8" t="inlineStr"/>
+      <c r="D27" s="8" t="inlineStr">
         <is>
           <t>virgilio.colomo@gmail.com</t>
         </is>
       </c>
-      <c r="E27" s="10" t="inlineStr">
+      <c r="E27" s="8" t="inlineStr">
         <is>
           <t>Architetto</t>
         </is>
       </c>
-      <c r="F27" s="10" t="inlineStr">
+      <c r="F27" s="8" t="inlineStr">
         <is>
           <t>c25f9</t>
         </is>
       </c>
-      <c r="G27" s="11" t="inlineStr">
-        <is>
-          <t>https://collaboratori.rilievocontract.it/?ref=c25f9</t>
+      <c r="G27" s="9" t="inlineStr">
+        <is>
+          <t>https://presentazione.rilievocontract.it/?ref=c25f9</t>
         </is>
       </c>
     </row>
     <row r="28">
-      <c r="A28" s="8" t="inlineStr">
+      <c r="A28" s="6" t="inlineStr">
         <is>
           <t>103</t>
         </is>
       </c>
-      <c r="B28" s="8" t="inlineStr">
+      <c r="B28" s="6" t="inlineStr">
         <is>
           <t>Studio Ing. Floridu Stefano</t>
         </is>
       </c>
-      <c r="C28" s="8" t="inlineStr"/>
-      <c r="D28" s="8" t="inlineStr">
+      <c r="C28" s="6" t="inlineStr"/>
+      <c r="D28" s="6" t="inlineStr">
         <is>
           <t>info@floridiastudio.com</t>
         </is>
       </c>
-      <c r="E28" s="8" t="inlineStr">
+      <c r="E28" s="6" t="inlineStr">
         <is>
           <t>Architetto</t>
         </is>
       </c>
-      <c r="F28" s="8" t="inlineStr">
+      <c r="F28" s="6" t="inlineStr">
         <is>
           <t>cd24d</t>
         </is>
       </c>
-      <c r="G28" s="9" t="inlineStr">
-        <is>
-          <t>https://collaboratori.rilievocontract.it/?ref=cd24d</t>
+      <c r="G28" s="7" t="inlineStr">
+        <is>
+          <t>https://presentazione.rilievocontract.it/?ref=cd24d</t>
         </is>
       </c>
     </row>
     <row r="29">
-      <c r="A29" s="10" t="inlineStr">
+      <c r="A29" s="8" t="inlineStr">
         <is>
           <t>104</t>
         </is>
       </c>
-      <c r="B29" s="10" t="inlineStr">
+      <c r="B29" s="8" t="inlineStr">
         <is>
           <t>Studio Arch. Soru Giovanni</t>
         </is>
       </c>
-      <c r="C29" s="10" t="inlineStr"/>
-      <c r="D29" s="10" t="inlineStr">
+      <c r="C29" s="8" t="inlineStr"/>
+      <c r="D29" s="8" t="inlineStr">
         <is>
           <t>archsoru@gmail.com</t>
         </is>
       </c>
-      <c r="E29" s="10" t="inlineStr">
+      <c r="E29" s="8" t="inlineStr">
         <is>
           <t>Architetto</t>
         </is>
       </c>
-      <c r="F29" s="10" t="inlineStr">
+      <c r="F29" s="8" t="inlineStr">
         <is>
           <t>62279</t>
         </is>
       </c>
-      <c r="G29" s="11" t="inlineStr">
-        <is>
-          <t>https://collaboratori.rilievocontract.it/?ref=62279</t>
+      <c r="G29" s="9" t="inlineStr">
+        <is>
+          <t>https://presentazione.rilievocontract.it/?ref=62279</t>
         </is>
       </c>
     </row>
     <row r="30">
-      <c r="A30" s="8" t="inlineStr">
+      <c r="A30" s="6" t="inlineStr">
         <is>
           <t>105</t>
         </is>
       </c>
-      <c r="B30" s="8" t="inlineStr">
+      <c r="B30" s="6" t="inlineStr">
         <is>
           <t>FASE Architettura</t>
         </is>
       </c>
-      <c r="C30" s="8" t="inlineStr"/>
-      <c r="D30" s="8" t="inlineStr">
+      <c r="C30" s="6" t="inlineStr"/>
+      <c r="D30" s="6" t="inlineStr">
         <is>
           <t>fasearchitettura@gmail.com</t>
         </is>
       </c>
-      <c r="E30" s="8" t="inlineStr">
+      <c r="E30" s="6" t="inlineStr">
         <is>
           <t>Architetto</t>
         </is>
       </c>
-      <c r="F30" s="8" t="inlineStr">
+      <c r="F30" s="6" t="inlineStr">
         <is>
           <t>4cde0</t>
         </is>
       </c>
-      <c r="G30" s="9" t="inlineStr">
-        <is>
-          <t>https://collaboratori.rilievocontract.it/?ref=4cde0</t>
+      <c r="G30" s="7" t="inlineStr">
+        <is>
+          <t>https://presentazione.rilievocontract.it/?ref=4cde0</t>
         </is>
       </c>
     </row>
     <row r="31">
-      <c r="A31" s="10" t="inlineStr">
+      <c r="A31" s="8" t="inlineStr">
         <is>
           <t>106</t>
         </is>
       </c>
-      <c r="B31" s="10" t="inlineStr">
+      <c r="B31" s="8" t="inlineStr">
         <is>
           <t>De signIS Studio</t>
         </is>
       </c>
-      <c r="C31" s="10" t="inlineStr"/>
-      <c r="D31" s="10" t="inlineStr">
+      <c r="C31" s="8" t="inlineStr"/>
+      <c r="D31" s="8" t="inlineStr">
         <is>
           <t>laura.designis@gmail.com</t>
         </is>
       </c>
-      <c r="E31" s="10" t="inlineStr">
+      <c r="E31" s="8" t="inlineStr">
         <is>
           <t>Architetto</t>
         </is>
       </c>
-      <c r="F31" s="10" t="inlineStr">
+      <c r="F31" s="8" t="inlineStr">
         <is>
           <t>0ccea</t>
         </is>
       </c>
-      <c r="G31" s="11" t="inlineStr">
-        <is>
-          <t>https://collaboratori.rilievocontract.it/?ref=0ccea</t>
+      <c r="G31" s="9" t="inlineStr">
+        <is>
+          <t>https://presentazione.rilievocontract.it/?ref=0ccea</t>
         </is>
       </c>
     </row>
     <row r="32">
-      <c r="A32" s="8" t="inlineStr">
+      <c r="A32" s="6" t="inlineStr">
         <is>
           <t>107</t>
         </is>
       </c>
-      <c r="B32" s="8" t="inlineStr">
+      <c r="B32" s="6" t="inlineStr">
         <is>
           <t>Studio Arch. Lubiani</t>
         </is>
       </c>
-      <c r="C32" s="8" t="inlineStr"/>
-      <c r="D32" s="8" t="inlineStr">
+      <c r="C32" s="6" t="inlineStr"/>
+      <c r="D32" s="6" t="inlineStr">
         <is>
           <t>marcello.lubiani@gmail.com</t>
         </is>
       </c>
-      <c r="E32" s="8" t="inlineStr">
+      <c r="E32" s="6" t="inlineStr">
         <is>
           <t>Architetto</t>
         </is>
       </c>
-      <c r="F32" s="8" t="inlineStr">
+      <c r="F32" s="6" t="inlineStr">
         <is>
           <t>59352</t>
         </is>
       </c>
-      <c r="G32" s="9" t="inlineStr">
-        <is>
-          <t>https://collaboratori.rilievocontract.it/?ref=59352</t>
+      <c r="G32" s="7" t="inlineStr">
+        <is>
+          <t>https://presentazione.rilievocontract.it/?ref=59352</t>
         </is>
       </c>
     </row>
     <row r="33">
-      <c r="A33" s="10" t="inlineStr">
+      <c r="A33" s="8" t="inlineStr">
         <is>
           <t>108</t>
         </is>
       </c>
-      <c r="B33" s="10" t="inlineStr">
+      <c r="B33" s="8" t="inlineStr">
         <is>
           <t>PIXEL Architecture Studio</t>
         </is>
       </c>
-      <c r="C33" s="10" t="inlineStr"/>
-      <c r="D33" s="10" t="inlineStr">
+      <c r="C33" s="8" t="inlineStr"/>
+      <c r="D33" s="8" t="inlineStr">
         <is>
           <t>archstefanogovoni@gmail.com</t>
         </is>
       </c>
-      <c r="E33" s="10" t="inlineStr">
+      <c r="E33" s="8" t="inlineStr">
         <is>
           <t>Architetto</t>
         </is>
       </c>
-      <c r="F33" s="10" t="inlineStr">
+      <c r="F33" s="8" t="inlineStr">
         <is>
           <t>1828a</t>
         </is>
       </c>
-      <c r="G33" s="11" t="inlineStr">
-        <is>
-          <t>https://collaboratori.rilievocontract.it/?ref=1828a</t>
+      <c r="G33" s="9" t="inlineStr">
+        <is>
+          <t>https://presentazione.rilievocontract.it/?ref=1828a</t>
         </is>
       </c>
     </row>
     <row r="34">
-      <c r="A34" s="8" t="inlineStr">
+      <c r="A34" s="6" t="inlineStr">
         <is>
           <t>109</t>
         </is>
       </c>
-      <c r="B34" s="8" t="inlineStr">
+      <c r="B34" s="6" t="inlineStr">
         <is>
           <t>Arch. Tedde</t>
         </is>
       </c>
-      <c r="C34" s="8" t="inlineStr"/>
-      <c r="D34" s="8" t="inlineStr">
+      <c r="C34" s="6" t="inlineStr"/>
+      <c r="D34" s="6" t="inlineStr">
         <is>
           <t>info@sandrotedde.com</t>
         </is>
       </c>
-      <c r="E34" s="8" t="inlineStr">
+      <c r="E34" s="6" t="inlineStr">
         <is>
           <t>Architetto</t>
         </is>
       </c>
-      <c r="F34" s="8" t="inlineStr">
+      <c r="F34" s="6" t="inlineStr">
         <is>
           <t>995bd</t>
         </is>
       </c>
-      <c r="G34" s="9" t="inlineStr">
-        <is>
-          <t>https://collaboratori.rilievocontract.it/?ref=995bd</t>
+      <c r="G34" s="7" t="inlineStr">
+        <is>
+          <t>https://presentazione.rilievocontract.it/?ref=995bd</t>
         </is>
       </c>
     </row>
     <row r="35">
-      <c r="A35" s="10" t="inlineStr">
+      <c r="A35" s="8" t="inlineStr">
         <is>
           <t>110</t>
         </is>
       </c>
-      <c r="B35" s="10" t="inlineStr">
+      <c r="B35" s="8" t="inlineStr">
         <is>
           <t>GAAP Studio</t>
         </is>
       </c>
-      <c r="C35" s="10" t="inlineStr"/>
-      <c r="D35" s="10" t="inlineStr">
+      <c r="C35" s="8" t="inlineStr"/>
+      <c r="D35" s="8" t="inlineStr">
         <is>
           <t>giorgio.asciutti@gmail.com</t>
         </is>
       </c>
-      <c r="E35" s="10" t="inlineStr">
+      <c r="E35" s="8" t="inlineStr">
         <is>
           <t>Architetto</t>
         </is>
       </c>
-      <c r="F35" s="10" t="inlineStr">
+      <c r="F35" s="8" t="inlineStr">
         <is>
           <t>929ef</t>
         </is>
       </c>
-      <c r="G35" s="11" t="inlineStr">
-        <is>
-          <t>https://collaboratori.rilievocontract.it/?ref=929ef</t>
+      <c r="G35" s="9" t="inlineStr">
+        <is>
+          <t>https://presentazione.rilievocontract.it/?ref=929ef</t>
         </is>
       </c>
     </row>
     <row r="36">
-      <c r="A36" s="8" t="inlineStr">
+      <c r="A36" s="6" t="inlineStr">
         <is>
           <t>111</t>
         </is>
       </c>
-      <c r="B36" s="8" t="inlineStr">
+      <c r="B36" s="6" t="inlineStr">
         <is>
           <t>Studio Lesuisse</t>
         </is>
       </c>
-      <c r="C36" s="8" t="inlineStr"/>
-      <c r="D36" s="8" t="inlineStr">
+      <c r="C36" s="6" t="inlineStr"/>
+      <c r="D36" s="6" t="inlineStr">
         <is>
           <t>studio@studiolesuisse.com</t>
         </is>
       </c>
-      <c r="E36" s="8" t="inlineStr">
+      <c r="E36" s="6" t="inlineStr">
         <is>
           <t>Architetto</t>
         </is>
       </c>
-      <c r="F36" s="8" t="inlineStr">
+      <c r="F36" s="6" t="inlineStr">
         <is>
           <t>d6f13</t>
         </is>
       </c>
-      <c r="G36" s="9" t="inlineStr">
-        <is>
-          <t>https://collaboratori.rilievocontract.it/?ref=d6f13</t>
+      <c r="G36" s="7" t="inlineStr">
+        <is>
+          <t>https://presentazione.rilievocontract.it/?ref=d6f13</t>
         </is>
       </c>
     </row>
     <row r="37">
-      <c r="A37" s="10" t="inlineStr">
+      <c r="A37" s="8" t="inlineStr">
         <is>
           <t>112</t>
         </is>
       </c>
-      <c r="B37" s="10" t="inlineStr">
+      <c r="B37" s="8" t="inlineStr">
         <is>
           <t>SP Interior Design</t>
         </is>
       </c>
-      <c r="C37" s="10" t="inlineStr"/>
-      <c r="D37" s="10" t="inlineStr">
+      <c r="C37" s="8" t="inlineStr"/>
+      <c r="D37" s="8" t="inlineStr">
         <is>
           <t>info@annalisazini.it</t>
         </is>
       </c>
-      <c r="E37" s="10" t="inlineStr">
+      <c r="E37" s="8" t="inlineStr">
         <is>
           <t>Architetto</t>
         </is>
       </c>
-      <c r="F37" s="10" t="inlineStr">
+      <c r="F37" s="8" t="inlineStr">
         <is>
           <t>8d0aa</t>
         </is>
       </c>
-      <c r="G37" s="11" t="inlineStr">
-        <is>
-          <t>https://collaboratori.rilievocontract.it/?ref=8d0aa</t>
+      <c r="G37" s="9" t="inlineStr">
+        <is>
+          <t>https://presentazione.rilievocontract.it/?ref=8d0aa</t>
         </is>
       </c>
     </row>
     <row r="38">
-      <c r="A38" s="8" t="inlineStr">
+      <c r="A38" s="6" t="inlineStr">
         <is>
           <t>113</t>
         </is>
       </c>
-      <c r="B38" s="8" t="inlineStr">
+      <c r="B38" s="6" t="inlineStr">
         <is>
           <t>Cozy Design</t>
         </is>
       </c>
-      <c r="C38" s="8" t="inlineStr"/>
-      <c r="D38" s="8" t="inlineStr">
+      <c r="C38" s="6" t="inlineStr"/>
+      <c r="D38" s="6" t="inlineStr">
         <is>
           <t>sonia@cozydesign.it</t>
         </is>
       </c>
-      <c r="E38" s="8" t="inlineStr">
+      <c r="E38" s="6" t="inlineStr">
         <is>
           <t>Architetto</t>
         </is>
       </c>
-      <c r="F38" s="8" t="inlineStr">
+      <c r="F38" s="6" t="inlineStr">
         <is>
           <t>56ef3</t>
         </is>
       </c>
-      <c r="G38" s="9" t="inlineStr">
-        <is>
-          <t>https://collaboratori.rilievocontract.it/?ref=56ef3</t>
+      <c r="G38" s="7" t="inlineStr">
+        <is>
+          <t>https://presentazione.rilievocontract.it/?ref=56ef3</t>
         </is>
       </c>
     </row>
     <row r="39">
-      <c r="A39" s="10" t="inlineStr">
+      <c r="A39" s="8" t="inlineStr">
         <is>
           <t>114</t>
         </is>
       </c>
-      <c r="B39" s="10" t="inlineStr">
+      <c r="B39" s="8" t="inlineStr">
         <is>
           <t>Studio LineArch</t>
         </is>
       </c>
-      <c r="C39" s="10" t="inlineStr"/>
-      <c r="D39" s="10" t="inlineStr">
+      <c r="C39" s="8" t="inlineStr"/>
+      <c r="D39" s="8" t="inlineStr">
         <is>
           <t>info@linearch.it</t>
         </is>
       </c>
-      <c r="E39" s="10" t="inlineStr">
+      <c r="E39" s="8" t="inlineStr">
         <is>
           <t>Architetto</t>
         </is>
       </c>
-      <c r="F39" s="10" t="inlineStr">
+      <c r="F39" s="8" t="inlineStr">
         <is>
           <t>bbd89</t>
         </is>
       </c>
-      <c r="G39" s="11" t="inlineStr">
-        <is>
-          <t>https://collaboratori.rilievocontract.it/?ref=bbd89</t>
+      <c r="G39" s="9" t="inlineStr">
+        <is>
+          <t>https://presentazione.rilievocontract.it/?ref=bbd89</t>
         </is>
       </c>
     </row>
     <row r="40">
-      <c r="A40" s="8" t="inlineStr">
+      <c r="A40" s="6" t="inlineStr">
         <is>
           <t>115</t>
         </is>
       </c>
-      <c r="B40" s="8" t="inlineStr">
+      <c r="B40" s="6" t="inlineStr">
         <is>
           <t>Arch. Danila Lampis</t>
         </is>
       </c>
-      <c r="C40" s="8" t="inlineStr"/>
-      <c r="D40" s="8" t="inlineStr">
+      <c r="C40" s="6" t="inlineStr"/>
+      <c r="D40" s="6" t="inlineStr">
         <is>
           <t>lampis.danila@gmail.com</t>
         </is>
       </c>
-      <c r="E40" s="8" t="inlineStr">
+      <c r="E40" s="6" t="inlineStr">
         <is>
           <t>Architetto</t>
         </is>
       </c>
-      <c r="F40" s="8" t="inlineStr">
+      <c r="F40" s="6" t="inlineStr">
         <is>
           <t>6897e</t>
         </is>
       </c>
-      <c r="G40" s="9" t="inlineStr">
-        <is>
-          <t>https://collaboratori.rilievocontract.it/?ref=6897e</t>
+      <c r="G40" s="7" t="inlineStr">
+        <is>
+          <t>https://presentazione.rilievocontract.it/?ref=6897e</t>
         </is>
       </c>
     </row>
     <row r="41">
-      <c r="A41" s="10" t="inlineStr">
+      <c r="A41" s="8" t="inlineStr">
         <is>
           <t>116</t>
         </is>
       </c>
-      <c r="B41" s="10" t="inlineStr">
+      <c r="B41" s="8" t="inlineStr">
         <is>
           <t>Arch. Alessandro Cardellini</t>
         </is>
       </c>
-      <c r="C41" s="10" t="inlineStr"/>
-      <c r="D41" s="10" t="inlineStr">
+      <c r="C41" s="8" t="inlineStr"/>
+      <c r="D41" s="8" t="inlineStr">
         <is>
           <t>alessandro@ac-architetto.com</t>
         </is>
       </c>
-      <c r="E41" s="10" t="inlineStr">
+      <c r="E41" s="8" t="inlineStr">
         <is>
           <t>Architetto</t>
         </is>
       </c>
-      <c r="F41" s="10" t="inlineStr">
+      <c r="F41" s="8" t="inlineStr">
         <is>
           <t>8d589</t>
         </is>
       </c>
-      <c r="G41" s="11" t="inlineStr">
-        <is>
-          <t>https://collaboratori.rilievocontract.it/?ref=8d589</t>
+      <c r="G41" s="9" t="inlineStr">
+        <is>
+          <t>https://presentazione.rilievocontract.it/?ref=8d589</t>
         </is>
       </c>
     </row>
     <row r="42">
-      <c r="A42" s="8" t="inlineStr">
+      <c r="A42" s="6" t="inlineStr">
         <is>
           <t>117</t>
         </is>
       </c>
-      <c r="B42" s="8" t="inlineStr">
+      <c r="B42" s="6" t="inlineStr">
         <is>
           <t>Arch. Stefania Negrini</t>
         </is>
       </c>
-      <c r="C42" s="8" t="inlineStr"/>
-      <c r="D42" s="8" t="inlineStr">
+      <c r="C42" s="6" t="inlineStr"/>
+      <c r="D42" s="6" t="inlineStr">
         <is>
           <t>info@negriniinteriors.com</t>
         </is>
       </c>
-      <c r="E42" s="8" t="inlineStr">
+      <c r="E42" s="6" t="inlineStr">
         <is>
           <t>Architetto</t>
         </is>
       </c>
-      <c r="F42" s="8" t="inlineStr">
+      <c r="F42" s="6" t="inlineStr">
         <is>
           <t>3322a</t>
         </is>
       </c>
-      <c r="G42" s="9" t="inlineStr">
-        <is>
-          <t>https://collaboratori.rilievocontract.it/?ref=3322a</t>
+      <c r="G42" s="7" t="inlineStr">
+        <is>
+          <t>https://presentazione.rilievocontract.it/?ref=3322a</t>
         </is>
       </c>
     </row>
     <row r="43">
-      <c r="A43" s="10" t="inlineStr">
+      <c r="A43" s="8" t="inlineStr">
         <is>
           <t>118</t>
         </is>
       </c>
-      <c r="B43" s="10" t="inlineStr">
+      <c r="B43" s="8" t="inlineStr">
         <is>
           <t>HZ Studio Architettura</t>
         </is>
       </c>
-      <c r="C43" s="10" t="inlineStr"/>
-      <c r="D43" s="10" t="inlineStr">
+      <c r="C43" s="8" t="inlineStr"/>
+      <c r="D43" s="8" t="inlineStr">
         <is>
           <t>studio@hzstudio.it</t>
         </is>
       </c>
-      <c r="E43" s="10" t="inlineStr">
+      <c r="E43" s="8" t="inlineStr">
         <is>
           <t>Architetto</t>
         </is>
       </c>
-      <c r="F43" s="10" t="inlineStr">
+      <c r="F43" s="8" t="inlineStr">
         <is>
           <t>f2d0e</t>
         </is>
       </c>
-      <c r="G43" s="11" t="inlineStr">
-        <is>
-          <t>https://collaboratori.rilievocontract.it/?ref=f2d0e</t>
+      <c r="G43" s="9" t="inlineStr">
+        <is>
+          <t>https://presentazione.rilievocontract.it/?ref=f2d0e</t>
         </is>
       </c>
     </row>
@@ -2204,7 +2148,6 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G43" r:id="rId42"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-  <legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="anysvml"/>
 </worksheet>
 </file>
 
@@ -2214,684 +2157,1165 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G20"/>
+  <dimension ref="A1:G33"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="8" customWidth="1" min="1" max="1"/>
-    <col width="34" customWidth="1" min="2" max="2"/>
-    <col width="24" customWidth="1" min="3" max="3"/>
-    <col width="32" customWidth="1" min="4" max="4"/>
-    <col width="26" customWidth="1" min="5" max="5"/>
-    <col width="10" customWidth="1" min="6" max="6"/>
+    <col width="30" customWidth="1" min="1" max="1"/>
+    <col width="30" customWidth="1" min="2" max="2"/>
+    <col width="30" customWidth="1" min="3" max="3"/>
+    <col width="30" customWidth="1" min="4" max="4"/>
+    <col width="30" customWidth="1" min="5" max="5"/>
+    <col width="30" customWidth="1" min="6" max="6"/>
     <col width="52" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
-    <row r="1" ht="20" customHeight="1">
-      <c r="A1" s="7" t="inlineStr">
-        <is>
-          <t>ID</t>
-        </is>
-      </c>
-      <c r="B1" s="7" t="inlineStr">
+    <row r="1">
+      <c r="A1" s="3" t="inlineStr">
+        <is>
+          <t>Id</t>
+        </is>
+      </c>
+      <c r="B1" s="3" t="inlineStr">
         <is>
           <t>Nome</t>
         </is>
       </c>
-      <c r="C1" s="7" t="inlineStr">
-        <is>
-          <t>Città</t>
-        </is>
-      </c>
-      <c r="D1" s="7" t="inlineStr">
+      <c r="C1" s="3" t="inlineStr">
+        <is>
+          <t>Citta</t>
+        </is>
+      </c>
+      <c r="D1" s="3" t="inlineStr">
         <is>
           <t>Email</t>
         </is>
       </c>
-      <c r="E1" s="7" t="inlineStr">
+      <c r="E1" s="3" t="inlineStr">
         <is>
           <t>Categoria</t>
         </is>
       </c>
-      <c r="F1" s="7" t="inlineStr">
+      <c r="F1" s="3" t="inlineStr">
         <is>
           <t>Ref</t>
         </is>
       </c>
-      <c r="G1" s="7" t="inlineStr">
-        <is>
-          <t>Link presentazione</t>
+      <c r="G1" s="3" t="inlineStr">
+        <is>
+          <t>Link</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="8" t="inlineStr">
+      <c r="A2" s="6" t="inlineStr">
         <is>
           <t>A1</t>
         </is>
       </c>
-      <c r="B2" s="8" t="inlineStr">
+      <c r="B2" s="6" t="inlineStr">
         <is>
           <t>Centocase Sardegna</t>
         </is>
       </c>
-      <c r="C2" s="8" t="inlineStr"/>
-      <c r="D2" s="8" t="inlineStr">
+      <c r="C2" s="6" t="inlineStr"/>
+      <c r="D2" s="6" t="inlineStr">
         <is>
           <t>info@centocasesardegna.it</t>
         </is>
       </c>
-      <c r="E2" s="8" t="inlineStr">
+      <c r="E2" s="6" t="inlineStr">
         <is>
           <t>Agenzia immobiliare</t>
         </is>
       </c>
-      <c r="F2" s="8" t="inlineStr">
+      <c r="F2" s="6" t="inlineStr">
         <is>
           <t>a1f1c</t>
         </is>
       </c>
-      <c r="G2" s="9" t="inlineStr">
+      <c r="G2" s="7" t="inlineStr">
         <is>
           <t>https://agenzie-immobiliari.rilievocontract.it/?ref=a1f1c</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="10" t="inlineStr">
+      <c r="A3" s="8" t="inlineStr">
         <is>
           <t>A2</t>
         </is>
       </c>
-      <c r="B3" s="10" t="inlineStr">
+      <c r="B3" s="8" t="inlineStr">
         <is>
           <t>Smeraldina Immobiliare</t>
         </is>
       </c>
-      <c r="C3" s="10" t="inlineStr"/>
-      <c r="D3" s="10" t="inlineStr">
+      <c r="C3" s="8" t="inlineStr"/>
+      <c r="D3" s="8" t="inlineStr">
         <is>
           <t>smeraldinaimmobiliare@gmail.com</t>
         </is>
       </c>
-      <c r="E3" s="10" t="inlineStr">
+      <c r="E3" s="8" t="inlineStr">
         <is>
           <t>Agenzia immobiliare</t>
         </is>
       </c>
-      <c r="F3" s="10" t="inlineStr">
+      <c r="F3" s="8" t="inlineStr">
         <is>
           <t>77a3d</t>
         </is>
       </c>
-      <c r="G3" s="11" t="inlineStr">
+      <c r="G3" s="9" t="inlineStr">
         <is>
           <t>https://agenzie-immobiliari.rilievocontract.it/?ref=77a3d</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="8" t="inlineStr">
+      <c r="A4" s="6" t="inlineStr">
         <is>
           <t>A3</t>
         </is>
       </c>
-      <c r="B4" s="8" t="inlineStr">
+      <c r="B4" s="6" t="inlineStr">
         <is>
           <t>Immobiliare La Maddalena</t>
         </is>
       </c>
-      <c r="C4" s="8" t="inlineStr"/>
-      <c r="D4" s="8" t="inlineStr">
+      <c r="C4" s="6" t="inlineStr"/>
+      <c r="D4" s="6" t="inlineStr">
         <is>
           <t>immlamaddalena@gmail.com</t>
         </is>
       </c>
-      <c r="E4" s="8" t="inlineStr">
+      <c r="E4" s="6" t="inlineStr">
         <is>
           <t>Agenzia immobiliare</t>
         </is>
       </c>
-      <c r="F4" s="8" t="inlineStr">
+      <c r="F4" s="6" t="inlineStr">
         <is>
           <t>18fd2</t>
         </is>
       </c>
-      <c r="G4" s="9" t="inlineStr">
+      <c r="G4" s="7" t="inlineStr">
         <is>
           <t>https://agenzie-immobiliari.rilievocontract.it/?ref=18fd2</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="10" t="inlineStr">
+      <c r="A5" s="8" t="inlineStr">
         <is>
           <t>A4</t>
         </is>
       </c>
-      <c r="B5" s="10" t="inlineStr">
+      <c r="B5" s="8" t="inlineStr">
         <is>
           <t>Realia Brokers</t>
         </is>
       </c>
-      <c r="C5" s="10" t="inlineStr"/>
-      <c r="D5" s="10" t="inlineStr">
+      <c r="C5" s="8" t="inlineStr"/>
+      <c r="D5" s="8" t="inlineStr">
         <is>
           <t>info@realiabrokers.com</t>
         </is>
       </c>
-      <c r="E5" s="10" t="inlineStr">
+      <c r="E5" s="8" t="inlineStr">
         <is>
           <t>Agenzia immobiliare</t>
         </is>
       </c>
-      <c r="F5" s="10" t="inlineStr">
+      <c r="F5" s="8" t="inlineStr">
         <is>
           <t>70df9</t>
         </is>
       </c>
-      <c r="G5" s="11" t="inlineStr">
+      <c r="G5" s="9" t="inlineStr">
         <is>
           <t>https://agenzie-immobiliari.rilievocontract.it/?ref=70df9</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="8" t="inlineStr">
+      <c r="A6" s="6" t="inlineStr">
         <is>
           <t>A5</t>
         </is>
       </c>
-      <c r="B6" s="8" t="inlineStr">
+      <c r="B6" s="6" t="inlineStr">
         <is>
           <t>Phoenix Real Estate</t>
         </is>
       </c>
-      <c r="C6" s="8" t="inlineStr"/>
-      <c r="D6" s="8" t="inlineStr">
+      <c r="C6" s="6" t="inlineStr"/>
+      <c r="D6" s="6" t="inlineStr">
         <is>
           <t>phoenixrealestatesrls@gmail.com</t>
         </is>
       </c>
-      <c r="E6" s="8" t="inlineStr">
+      <c r="E6" s="6" t="inlineStr">
         <is>
           <t>Agenzia immobiliare</t>
         </is>
       </c>
-      <c r="F6" s="8" t="inlineStr">
+      <c r="F6" s="6" t="inlineStr">
         <is>
           <t>67910</t>
         </is>
       </c>
-      <c r="G6" s="9" t="inlineStr">
+      <c r="G6" s="7" t="inlineStr">
         <is>
           <t>https://agenzie-immobiliari.rilievocontract.it/?ref=67910</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="10" t="inlineStr">
+      <c r="A7" s="8" t="inlineStr">
         <is>
           <t>A6</t>
         </is>
       </c>
-      <c r="B7" s="10" t="inlineStr">
+      <c r="B7" s="8" t="inlineStr">
         <is>
           <t>Maior Capital | Forbes Global Properties</t>
         </is>
       </c>
-      <c r="C7" s="10" t="inlineStr"/>
-      <c r="D7" s="10" t="inlineStr">
+      <c r="C7" s="8" t="inlineStr"/>
+      <c r="D7" s="8" t="inlineStr">
         <is>
           <t>sardinia@maiorcapital.com</t>
         </is>
       </c>
-      <c r="E7" s="10" t="inlineStr">
+      <c r="E7" s="8" t="inlineStr">
         <is>
           <t>Agenzia immobiliare</t>
         </is>
       </c>
-      <c r="F7" s="10" t="inlineStr">
+      <c r="F7" s="8" t="inlineStr">
         <is>
           <t>11f28</t>
         </is>
       </c>
-      <c r="G7" s="11" t="inlineStr">
+      <c r="G7" s="9" t="inlineStr">
         <is>
           <t>https://agenzie-immobiliari.rilievocontract.it/?ref=11f28</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="8" t="inlineStr">
+      <c r="A8" s="6" t="inlineStr">
         <is>
           <t>A7</t>
         </is>
       </c>
-      <c r="B8" s="8" t="inlineStr">
+      <c r="B8" s="6" t="inlineStr">
         <is>
           <t>Gallura Immobiliare</t>
         </is>
       </c>
-      <c r="C8" s="8" t="inlineStr"/>
-      <c r="D8" s="8" t="inlineStr">
+      <c r="C8" s="6" t="inlineStr"/>
+      <c r="D8" s="6" t="inlineStr">
         <is>
           <t>galluraimmobiliare@virgilio.it</t>
         </is>
       </c>
-      <c r="E8" s="8" t="inlineStr">
+      <c r="E8" s="6" t="inlineStr">
         <is>
           <t>Agenzia immobiliare</t>
         </is>
       </c>
-      <c r="F8" s="8" t="inlineStr">
+      <c r="F8" s="6" t="inlineStr">
         <is>
           <t>15eb0</t>
         </is>
       </c>
-      <c r="G8" s="9" t="inlineStr">
+      <c r="G8" s="7" t="inlineStr">
         <is>
           <t>https://agenzie-immobiliari.rilievocontract.it/?ref=15eb0</t>
         </is>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="10" t="inlineStr">
+      <c r="A9" s="8" t="inlineStr">
         <is>
           <t>A8</t>
         </is>
       </c>
-      <c r="B9" s="10" t="inlineStr">
+      <c r="B9" s="8" t="inlineStr">
         <is>
           <t>House &amp; Domos Immobiliare</t>
         </is>
       </c>
-      <c r="C9" s="10" t="inlineStr"/>
-      <c r="D9" s="10" t="inlineStr">
+      <c r="C9" s="8" t="inlineStr"/>
+      <c r="D9" s="8" t="inlineStr">
         <is>
           <t>info@housedomos.com</t>
         </is>
       </c>
-      <c r="E9" s="10" t="inlineStr">
+      <c r="E9" s="8" t="inlineStr">
         <is>
           <t>Agenzia immobiliare</t>
         </is>
       </c>
-      <c r="F9" s="10" t="inlineStr">
+      <c r="F9" s="8" t="inlineStr">
         <is>
           <t>61b12</t>
         </is>
       </c>
-      <c r="G9" s="11" t="inlineStr">
+      <c r="G9" s="9" t="inlineStr">
         <is>
           <t>https://agenzie-immobiliari.rilievocontract.it/?ref=61b12</t>
         </is>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="8" t="inlineStr">
+      <c r="A10" s="6" t="inlineStr">
         <is>
           <t>A9</t>
         </is>
       </c>
-      <c r="B10" s="8" t="inlineStr">
+      <c r="B10" s="6" t="inlineStr">
         <is>
           <t>Il Faro Immobiliare</t>
         </is>
       </c>
-      <c r="C10" s="8" t="inlineStr"/>
-      <c r="D10" s="8" t="inlineStr">
+      <c r="C10" s="6" t="inlineStr"/>
+      <c r="D10" s="6" t="inlineStr">
         <is>
           <t>info@agenziailfaro.it</t>
         </is>
       </c>
-      <c r="E10" s="8" t="inlineStr">
+      <c r="E10" s="6" t="inlineStr">
         <is>
           <t>Agenzia immobiliare</t>
         </is>
       </c>
-      <c r="F10" s="8" t="inlineStr">
+      <c r="F10" s="6" t="inlineStr">
         <is>
           <t>66476</t>
         </is>
       </c>
-      <c r="G10" s="9" t="inlineStr">
+      <c r="G10" s="7" t="inlineStr">
         <is>
           <t>https://agenzie-immobiliari.rilievocontract.it/?ref=66476</t>
         </is>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="10" t="inlineStr">
+      <c r="A11" s="8" t="inlineStr">
         <is>
           <t>A10</t>
         </is>
       </c>
-      <c r="B11" s="10" t="inlineStr">
+      <c r="B11" s="8" t="inlineStr">
         <is>
           <t>Simius Immobiliare</t>
         </is>
       </c>
-      <c r="C11" s="10" t="inlineStr"/>
-      <c r="D11" s="10" t="inlineStr">
+      <c r="C11" s="8" t="inlineStr"/>
+      <c r="D11" s="8" t="inlineStr">
         <is>
           <t>info@simiusimmobiliare.com</t>
         </is>
       </c>
-      <c r="E11" s="10" t="inlineStr">
+      <c r="E11" s="8" t="inlineStr">
         <is>
           <t>Agenzia immobiliare</t>
         </is>
       </c>
-      <c r="F11" s="10" t="inlineStr">
+      <c r="F11" s="8" t="inlineStr">
         <is>
           <t>2c1c5</t>
         </is>
       </c>
-      <c r="G11" s="11" t="inlineStr">
+      <c r="G11" s="9" t="inlineStr">
         <is>
           <t>https://agenzie-immobiliari.rilievocontract.it/?ref=2c1c5</t>
         </is>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="8" t="inlineStr">
+      <c r="A12" s="6" t="inlineStr">
         <is>
           <t>A11</t>
         </is>
       </c>
-      <c r="B12" s="8" t="inlineStr">
+      <c r="B12" s="6" t="inlineStr">
         <is>
           <t>FrauMare Immobiliare</t>
         </is>
       </c>
-      <c r="C12" s="8" t="inlineStr"/>
-      <c r="D12" s="8" t="inlineStr">
+      <c r="C12" s="6" t="inlineStr"/>
+      <c r="D12" s="6" t="inlineStr">
         <is>
           <t>agenzia@fraumare.com</t>
         </is>
       </c>
-      <c r="E12" s="8" t="inlineStr">
+      <c r="E12" s="6" t="inlineStr">
         <is>
           <t>Agenzia immobiliare</t>
         </is>
       </c>
-      <c r="F12" s="8" t="inlineStr">
+      <c r="F12" s="6" t="inlineStr">
         <is>
           <t>f0e2b</t>
         </is>
       </c>
-      <c r="G12" s="9" t="inlineStr">
+      <c r="G12" s="7" t="inlineStr">
         <is>
           <t>https://agenzie-immobiliari.rilievocontract.it/?ref=f0e2b</t>
         </is>
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="10" t="inlineStr">
+      <c r="A13" s="8" t="inlineStr">
         <is>
           <t>A12</t>
         </is>
       </c>
-      <c r="B13" s="10" t="inlineStr">
+      <c r="B13" s="8" t="inlineStr">
         <is>
           <t>Casula Immobiliare</t>
         </is>
       </c>
-      <c r="C13" s="10" t="inlineStr"/>
-      <c r="D13" s="10" t="inlineStr">
+      <c r="C13" s="8" t="inlineStr"/>
+      <c r="D13" s="8" t="inlineStr">
         <is>
           <t>info@casulaimmobiliare.com</t>
         </is>
       </c>
-      <c r="E13" s="10" t="inlineStr">
+      <c r="E13" s="8" t="inlineStr">
         <is>
           <t>Agenzia immobiliare</t>
         </is>
       </c>
-      <c r="F13" s="10" t="inlineStr">
+      <c r="F13" s="8" t="inlineStr">
         <is>
           <t>2d044</t>
         </is>
       </c>
-      <c r="G13" s="11" t="inlineStr">
+      <c r="G13" s="9" t="inlineStr">
         <is>
           <t>https://agenzie-immobiliari.rilievocontract.it/?ref=2d044</t>
         </is>
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="8" t="inlineStr">
+      <c r="A14" s="6" t="inlineStr">
         <is>
           <t>A13</t>
         </is>
       </c>
-      <c r="B14" s="8" t="inlineStr">
+      <c r="B14" s="6" t="inlineStr">
         <is>
           <t>Ital Home Costa Rei/Villasimius</t>
         </is>
       </c>
-      <c r="C14" s="8" t="inlineStr"/>
-      <c r="D14" s="8" t="inlineStr">
+      <c r="C14" s="6" t="inlineStr"/>
+      <c r="D14" s="6" t="inlineStr">
         <is>
           <t>villasimius@ital-home.it</t>
         </is>
       </c>
-      <c r="E14" s="8" t="inlineStr">
+      <c r="E14" s="6" t="inlineStr">
         <is>
           <t>Agenzia immobiliare</t>
         </is>
       </c>
-      <c r="F14" s="8" t="inlineStr">
+      <c r="F14" s="6" t="inlineStr">
         <is>
           <t>0d759</t>
         </is>
       </c>
-      <c r="G14" s="9" t="inlineStr">
+      <c r="G14" s="7" t="inlineStr">
         <is>
           <t>https://agenzie-immobiliari.rilievocontract.it/?ref=0d759</t>
         </is>
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="10" t="inlineStr">
+      <c r="A15" s="8" t="inlineStr">
         <is>
           <t>A14</t>
         </is>
       </c>
-      <c r="B15" s="10" t="inlineStr">
+      <c r="B15" s="8" t="inlineStr">
         <is>
           <t>IMMOVA</t>
         </is>
       </c>
-      <c r="C15" s="10" t="inlineStr"/>
-      <c r="D15" s="10" t="inlineStr">
+      <c r="C15" s="8" t="inlineStr"/>
+      <c r="D15" s="8" t="inlineStr">
         <is>
           <t>immova2021@gmail.com</t>
         </is>
       </c>
-      <c r="E15" s="10" t="inlineStr">
+      <c r="E15" s="8" t="inlineStr">
         <is>
           <t>Agenzia immobiliare</t>
         </is>
       </c>
-      <c r="F15" s="10" t="inlineStr">
+      <c r="F15" s="8" t="inlineStr">
         <is>
           <t>baa1e</t>
         </is>
       </c>
-      <c r="G15" s="11" t="inlineStr">
+      <c r="G15" s="9" t="inlineStr">
         <is>
           <t>https://agenzie-immobiliari.rilievocontract.it/?ref=baa1e</t>
         </is>
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="8" t="inlineStr">
+      <c r="A16" s="6" t="inlineStr">
         <is>
           <t>A15</t>
         </is>
       </c>
-      <c r="B16" s="8" t="inlineStr">
+      <c r="B16" s="6" t="inlineStr">
         <is>
           <t>Minvicase</t>
         </is>
       </c>
-      <c r="C16" s="8" t="inlineStr"/>
-      <c r="D16" s="8" t="inlineStr">
+      <c r="C16" s="6" t="inlineStr"/>
+      <c r="D16" s="6" t="inlineStr">
         <is>
           <t>info@minvicase.it</t>
         </is>
       </c>
-      <c r="E16" s="8" t="inlineStr">
+      <c r="E16" s="6" t="inlineStr">
         <is>
           <t>Agenzia immobiliare</t>
         </is>
       </c>
-      <c r="F16" s="8" t="inlineStr">
+      <c r="F16" s="6" t="inlineStr">
         <is>
           <t>24ebd</t>
         </is>
       </c>
-      <c r="G16" s="9" t="inlineStr">
+      <c r="G16" s="7" t="inlineStr">
         <is>
           <t>https://agenzie-immobiliari.rilievocontract.it/?ref=24ebd</t>
         </is>
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="10" t="inlineStr">
+      <c r="A17" s="8" t="inlineStr">
         <is>
           <t>A16</t>
         </is>
       </c>
-      <c r="B17" s="10" t="inlineStr">
+      <c r="B17" s="8" t="inlineStr">
         <is>
           <t>La Tua Casa al Mare</t>
         </is>
       </c>
-      <c r="C17" s="10" t="inlineStr"/>
-      <c r="D17" s="10" t="inlineStr">
+      <c r="C17" s="8" t="inlineStr"/>
+      <c r="D17" s="8" t="inlineStr">
         <is>
           <t>info@latuacasaalmare.it</t>
         </is>
       </c>
-      <c r="E17" s="10" t="inlineStr">
+      <c r="E17" s="8" t="inlineStr">
         <is>
           <t>Agenzia immobiliare</t>
         </is>
       </c>
-      <c r="F17" s="10" t="inlineStr">
+      <c r="F17" s="8" t="inlineStr">
         <is>
           <t>8583b</t>
         </is>
       </c>
-      <c r="G17" s="11" t="inlineStr">
+      <c r="G17" s="9" t="inlineStr">
         <is>
           <t>https://agenzie-immobiliari.rilievocontract.it/?ref=8583b</t>
         </is>
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="8" t="inlineStr">
+      <c r="A18" s="6" t="inlineStr">
         <is>
           <t>A17</t>
         </is>
       </c>
-      <c r="B18" s="8" t="inlineStr">
+      <c r="B18" s="6" t="inlineStr">
         <is>
           <t>Alghero Ital Home</t>
         </is>
       </c>
-      <c r="C18" s="8" t="inlineStr"/>
-      <c r="D18" s="8" t="inlineStr">
+      <c r="C18" s="6" t="inlineStr"/>
+      <c r="D18" s="6" t="inlineStr">
         <is>
           <t>alghero@ital-home.it</t>
         </is>
       </c>
-      <c r="E18" s="8" t="inlineStr">
+      <c r="E18" s="6" t="inlineStr">
         <is>
           <t>Agenzia immobiliare</t>
         </is>
       </c>
-      <c r="F18" s="8" t="inlineStr">
+      <c r="F18" s="6" t="inlineStr">
         <is>
           <t>3dfa7</t>
         </is>
       </c>
-      <c r="G18" s="9" t="inlineStr">
+      <c r="G18" s="7" t="inlineStr">
         <is>
           <t>https://agenzie-immobiliari.rilievocontract.it/?ref=3dfa7</t>
         </is>
       </c>
     </row>
     <row r="19">
-      <c r="A19" s="10" t="inlineStr">
+      <c r="A19" s="8" t="inlineStr">
         <is>
           <t>A18</t>
         </is>
       </c>
-      <c r="B19" s="10" t="inlineStr">
+      <c r="B19" s="8" t="inlineStr">
         <is>
           <t>Agenzia Capo Falcone</t>
         </is>
       </c>
-      <c r="C19" s="10" t="inlineStr"/>
-      <c r="D19" s="10" t="inlineStr">
+      <c r="C19" s="8" t="inlineStr"/>
+      <c r="D19" s="8" t="inlineStr">
         <is>
           <t>stintino@email.it</t>
         </is>
       </c>
-      <c r="E19" s="10" t="inlineStr">
+      <c r="E19" s="8" t="inlineStr">
         <is>
           <t>Agenzia immobiliare</t>
         </is>
       </c>
-      <c r="F19" s="10" t="inlineStr">
+      <c r="F19" s="8" t="inlineStr">
         <is>
           <t>4c4fd</t>
         </is>
       </c>
-      <c r="G19" s="11" t="inlineStr">
+      <c r="G19" s="9" t="inlineStr">
         <is>
           <t>https://agenzie-immobiliari.rilievocontract.it/?ref=4c4fd</t>
         </is>
       </c>
     </row>
     <row r="20">
-      <c r="A20" s="8" t="inlineStr">
+      <c r="A20" s="6" t="inlineStr">
         <is>
           <t>A19</t>
         </is>
       </c>
-      <c r="B20" s="8" t="inlineStr">
+      <c r="B20" s="6" t="inlineStr">
         <is>
           <t>Ajò Immobiliare</t>
         </is>
       </c>
-      <c r="C20" s="8" t="inlineStr"/>
-      <c r="D20" s="8" t="inlineStr">
+      <c r="C20" s="6" t="inlineStr"/>
+      <c r="D20" s="6" t="inlineStr">
         <is>
           <t>info@ajo.casa</t>
         </is>
       </c>
-      <c r="E20" s="8" t="inlineStr">
+      <c r="E20" s="6" t="inlineStr">
         <is>
           <t>Agenzia immobiliare</t>
         </is>
       </c>
-      <c r="F20" s="8" t="inlineStr">
+      <c r="F20" s="6" t="inlineStr">
         <is>
           <t>e3d9a</t>
         </is>
       </c>
-      <c r="G20" s="9" t="inlineStr">
+      <c r="G20" s="7" t="inlineStr">
         <is>
           <t>https://agenzie-immobiliari.rilievocontract.it/?ref=e3d9a</t>
         </is>
       </c>
     </row>
+    <row r="21">
+      <c r="A21" s="8" t="inlineStr">
+        <is>
+          <t>A20</t>
+        </is>
+      </c>
+      <c r="B21" s="8" t="inlineStr">
+        <is>
+          <t>Coldwell Banker Global Luxury</t>
+        </is>
+      </c>
+      <c r="C21" s="8" t="inlineStr">
+        <is>
+          <t>Porto Cervo — Arzachena (SS)</t>
+        </is>
+      </c>
+      <c r="D21" s="8" t="inlineStr">
+        <is>
+          <t>portocervo@cbitaly.it</t>
+        </is>
+      </c>
+      <c r="E21" s="8" t="inlineStr">
+        <is>
+          <t>Agenzia immobiliare</t>
+        </is>
+      </c>
+      <c r="F21" s="8" t="inlineStr">
+        <is>
+          <t>f169a</t>
+        </is>
+      </c>
+      <c r="G21" s="8" t="inlineStr">
+        <is>
+          <t>https://agenzie-immobiliari.rilievocontract.it/?ref=f169a</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="6" t="inlineStr">
+        <is>
+          <t>A21</t>
+        </is>
+      </c>
+      <c r="B22" s="6" t="inlineStr">
+        <is>
+          <t>Luxury Esmeralda (Savills)</t>
+        </is>
+      </c>
+      <c r="C22" s="6" t="inlineStr">
+        <is>
+          <t>Porto Rotondo — Olbia (SS)</t>
+        </is>
+      </c>
+      <c r="D22" s="6" t="inlineStr">
+        <is>
+          <t>info@luxuryesmeralda.com</t>
+        </is>
+      </c>
+      <c r="E22" s="6" t="inlineStr">
+        <is>
+          <t>Agenzia immobiliare</t>
+        </is>
+      </c>
+      <c r="F22" s="6" t="inlineStr">
+        <is>
+          <t>88560</t>
+        </is>
+      </c>
+      <c r="G22" s="6" t="inlineStr">
+        <is>
+          <t>https://agenzie-immobiliari.rilievocontract.it/?ref=88560</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="8" t="inlineStr">
+        <is>
+          <t>A22</t>
+        </is>
+      </c>
+      <c r="B23" s="8" t="inlineStr">
+        <is>
+          <t>BARNES Sardegna</t>
+        </is>
+      </c>
+      <c r="C23" s="8" t="inlineStr">
+        <is>
+          <t>Porto Cervo — Arzachena (SS)</t>
+        </is>
+      </c>
+      <c r="D23" s="8" t="inlineStr">
+        <is>
+          <t>portocervo@barnes-international.com</t>
+        </is>
+      </c>
+      <c r="E23" s="8" t="inlineStr">
+        <is>
+          <t>Agenzia immobiliare</t>
+        </is>
+      </c>
+      <c r="F23" s="8" t="inlineStr">
+        <is>
+          <t>90eca</t>
+        </is>
+      </c>
+      <c r="G23" s="8" t="inlineStr">
+        <is>
+          <t>https://agenzie-immobiliari.rilievocontract.it/?ref=90eca</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="6" t="inlineStr">
+        <is>
+          <t>A23</t>
+        </is>
+      </c>
+      <c r="B24" s="6" t="inlineStr">
+        <is>
+          <t>Engel &amp; Völkers Costa Smeralda</t>
+        </is>
+      </c>
+      <c r="C24" s="6" t="inlineStr">
+        <is>
+          <t>Porto Cervo — Arzachena (SS)</t>
+        </is>
+      </c>
+      <c r="D24" s="6" t="inlineStr">
+        <is>
+          <t>portocervo@engelvoelkers.com</t>
+        </is>
+      </c>
+      <c r="E24" s="6" t="inlineStr">
+        <is>
+          <t>Agenzia immobiliare</t>
+        </is>
+      </c>
+      <c r="F24" s="6" t="inlineStr">
+        <is>
+          <t>d73db</t>
+        </is>
+      </c>
+      <c r="G24" s="6" t="inlineStr">
+        <is>
+          <t>https://agenzie-immobiliari.rilievocontract.it/?ref=d73db</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="8" t="inlineStr">
+        <is>
+          <t>A24</t>
+        </is>
+      </c>
+      <c r="B25" s="8" t="inlineStr">
+        <is>
+          <t>Italy Sotheby's International Realty</t>
+        </is>
+      </c>
+      <c r="C25" s="8" t="inlineStr">
+        <is>
+          <t>Porto Cervo (SS)</t>
+        </is>
+      </c>
+      <c r="D25" s="8" t="inlineStr">
+        <is>
+          <t>portocervo@sothebysrealty.it</t>
+        </is>
+      </c>
+      <c r="E25" s="8" t="inlineStr">
+        <is>
+          <t>Agenzia immobiliare</t>
+        </is>
+      </c>
+      <c r="F25" s="8" t="inlineStr">
+        <is>
+          <t>e6e4d</t>
+        </is>
+      </c>
+      <c r="G25" s="8" t="inlineStr">
+        <is>
+          <t>https://agenzie-immobiliari.rilievocontract.it/?ref=e6e4d</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="6" t="inlineStr">
+        <is>
+          <t>A25</t>
+        </is>
+      </c>
+      <c r="B26" s="6" t="inlineStr">
+        <is>
+          <t>ImmobilSarda Christie's International Real Estate</t>
+        </is>
+      </c>
+      <c r="C26" s="6" t="inlineStr">
+        <is>
+          <t>Porto Cervo (SS)</t>
+        </is>
+      </c>
+      <c r="D26" s="6" t="inlineStr">
+        <is>
+          <t>portocervo@immobilsarda.com</t>
+        </is>
+      </c>
+      <c r="E26" s="6" t="inlineStr">
+        <is>
+          <t>Agenzia immobiliare</t>
+        </is>
+      </c>
+      <c r="F26" s="6" t="inlineStr">
+        <is>
+          <t>f36e7</t>
+        </is>
+      </c>
+      <c r="G26" s="6" t="inlineStr">
+        <is>
+          <t>https://agenzie-immobiliari.rilievocontract.it/?ref=f36e7</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="8" t="inlineStr">
+        <is>
+          <t>A26</t>
+        </is>
+      </c>
+      <c r="B27" s="8" t="inlineStr">
+        <is>
+          <t>Capitta &amp; Partners</t>
+        </is>
+      </c>
+      <c r="C27" s="8" t="inlineStr">
+        <is>
+          <t>Cagliari</t>
+        </is>
+      </c>
+      <c r="D27" s="8" t="inlineStr">
+        <is>
+          <t>info@capittaepartners.it</t>
+        </is>
+      </c>
+      <c r="E27" s="8" t="inlineStr">
+        <is>
+          <t>Agenzia immobiliare</t>
+        </is>
+      </c>
+      <c r="F27" s="8" t="inlineStr">
+        <is>
+          <t>65a2a</t>
+        </is>
+      </c>
+      <c r="G27" s="8" t="inlineStr">
+        <is>
+          <t>https://agenzie-immobiliari.rilievocontract.it/?ref=65a2a</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="6" t="inlineStr">
+        <is>
+          <t>A27</t>
+        </is>
+      </c>
+      <c r="B28" s="6" t="inlineStr">
+        <is>
+          <t>Ladiri Immobiliare</t>
+        </is>
+      </c>
+      <c r="C28" s="6" t="inlineStr">
+        <is>
+          <t>Cagliari</t>
+        </is>
+      </c>
+      <c r="D28" s="6" t="inlineStr">
+        <is>
+          <t>info@ladiri.it</t>
+        </is>
+      </c>
+      <c r="E28" s="6" t="inlineStr">
+        <is>
+          <t>Agenzia immobiliare</t>
+        </is>
+      </c>
+      <c r="F28" s="6" t="inlineStr">
+        <is>
+          <t>00fb9</t>
+        </is>
+      </c>
+      <c r="G28" s="6" t="inlineStr">
+        <is>
+          <t>https://agenzie-immobiliari.rilievocontract.it/?ref=00fb9</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="8" t="inlineStr">
+        <is>
+          <t>A28</t>
+        </is>
+      </c>
+      <c r="B29" s="8" t="inlineStr">
+        <is>
+          <t>P&amp;S Property &amp; Sales</t>
+        </is>
+      </c>
+      <c r="C29" s="8" t="inlineStr">
+        <is>
+          <t>Cagliari</t>
+        </is>
+      </c>
+      <c r="D29" s="8" t="inlineStr">
+        <is>
+          <t>pes.intermediazioni@gmail.com</t>
+        </is>
+      </c>
+      <c r="E29" s="8" t="inlineStr">
+        <is>
+          <t>Agenzia immobiliare</t>
+        </is>
+      </c>
+      <c r="F29" s="8" t="inlineStr">
+        <is>
+          <t>06282</t>
+        </is>
+      </c>
+      <c r="G29" s="8" t="inlineStr">
+        <is>
+          <t>https://agenzie-immobiliari.rilievocontract.it/?ref=06282</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="6" t="inlineStr">
+        <is>
+          <t>A29</t>
+        </is>
+      </c>
+      <c r="B30" s="6" t="inlineStr">
+        <is>
+          <t>Sardinia Real Estate</t>
+        </is>
+      </c>
+      <c r="C30" s="6" t="inlineStr">
+        <is>
+          <t>Quartucciu (CA)</t>
+        </is>
+      </c>
+      <c r="D30" s="6" t="inlineStr">
+        <is>
+          <t>info.sardiniare@gmail.com</t>
+        </is>
+      </c>
+      <c r="E30" s="6" t="inlineStr">
+        <is>
+          <t>Agenzia immobiliare</t>
+        </is>
+      </c>
+      <c r="F30" s="6" t="inlineStr">
+        <is>
+          <t>b5bfb</t>
+        </is>
+      </c>
+      <c r="G30" s="6" t="inlineStr">
+        <is>
+          <t>https://agenzie-immobiliari.rilievocontract.it/?ref=b5bfb</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="8" t="inlineStr">
+        <is>
+          <t>A30</t>
+        </is>
+      </c>
+      <c r="B31" s="8" t="inlineStr">
+        <is>
+          <t>Galleria d'Autore Immobili di Lusso</t>
+        </is>
+      </c>
+      <c r="C31" s="8" t="inlineStr">
+        <is>
+          <t>Sassari</t>
+        </is>
+      </c>
+      <c r="D31" s="8" t="inlineStr">
+        <is>
+          <t>info@galleriadautore.it</t>
+        </is>
+      </c>
+      <c r="E31" s="8" t="inlineStr">
+        <is>
+          <t>Agenzia immobiliare</t>
+        </is>
+      </c>
+      <c r="F31" s="8" t="inlineStr">
+        <is>
+          <t>3d65f</t>
+        </is>
+      </c>
+      <c r="G31" s="8" t="inlineStr">
+        <is>
+          <t>https://agenzie-immobiliari.rilievocontract.it/?ref=3d65f</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="6" t="inlineStr">
+        <is>
+          <t>A31</t>
+        </is>
+      </c>
+      <c r="B32" s="6" t="inlineStr">
+        <is>
+          <t>Vallebona Immobiliare</t>
+        </is>
+      </c>
+      <c r="C32" s="6" t="inlineStr">
+        <is>
+          <t>Cagliari / Chia / Villasimius</t>
+        </is>
+      </c>
+      <c r="D32" s="6" t="inlineStr">
+        <is>
+          <t>info@vallebonarealestate.it</t>
+        </is>
+      </c>
+      <c r="E32" s="6" t="inlineStr">
+        <is>
+          <t>Agenzia immobiliare</t>
+        </is>
+      </c>
+      <c r="F32" s="6" t="inlineStr">
+        <is>
+          <t>6c731</t>
+        </is>
+      </c>
+      <c r="G32" s="6" t="inlineStr">
+        <is>
+          <t>https://agenzie-immobiliari.rilievocontract.it/?ref=6c731</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="8" t="inlineStr">
+        <is>
+          <t>A32</t>
+        </is>
+      </c>
+      <c r="B33" s="8" t="inlineStr">
+        <is>
+          <t>L'Immobiliare Sardegna</t>
+        </is>
+      </c>
+      <c r="C33" s="8" t="inlineStr">
+        <is>
+          <t>Alghero (SS)</t>
+        </is>
+      </c>
+      <c r="D33" s="8" t="inlineStr">
+        <is>
+          <t>info@immobiliaresardegna.eu</t>
+        </is>
+      </c>
+      <c r="E33" s="8" t="inlineStr">
+        <is>
+          <t>Agenzia immobiliare</t>
+        </is>
+      </c>
+      <c r="F33" s="8" t="inlineStr">
+        <is>
+          <t>95611</t>
+        </is>
+      </c>
+      <c r="G33" s="8" t="inlineStr">
+        <is>
+          <t>https://agenzie-immobiliari.rilievocontract.it/?ref=95611</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:G20"/>
+  <autoFilter ref="A1:G33"/>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G2" r:id="rId1"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G3" r:id="rId2"/>

</xml_diff>

<commit_message>
Rimuove Galleria d'Autore Immobili di Lusso dalla lista agenzie (competitor di Rilievo, non partner)
- Lista_Contatti_Rilievo_Contract.xlsx: 42 architetti + 31 agenzie (73 totali)
- generatore_email.html: rigenerato senza Galleria d'Autore, aggiunti i campi Oggetto/Destinatario email con relativi bottoni copia
</commit_message>
<xml_diff>
--- a/Lista_Contatti_Rilievo_Contract.xlsx
+++ b/Lista_Contatti_Rilievo_Contract.xlsx
@@ -517,6 +517,7 @@
         </is>
       </c>
     </row>
+    <row r="3"/>
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
         <is>
@@ -546,7 +547,7 @@
         </is>
       </c>
       <c r="B6" s="4" t="n">
-        <v>32</v>
+        <v>31</v>
       </c>
     </row>
     <row r="7">
@@ -556,7 +557,7 @@
         </is>
       </c>
       <c r="B7" s="5" t="n">
-        <v>74</v>
+        <v>73</v>
       </c>
     </row>
   </sheetData>
@@ -2157,7 +2158,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G33"/>
+  <dimension ref="A1:G32"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -3204,111 +3205,74 @@
       </c>
     </row>
     <row r="31">
-      <c r="A31" s="8" t="inlineStr">
-        <is>
-          <t>A30</t>
-        </is>
-      </c>
-      <c r="B31" s="8" t="inlineStr">
-        <is>
-          <t>Galleria d'Autore Immobili di Lusso</t>
-        </is>
-      </c>
-      <c r="C31" s="8" t="inlineStr">
-        <is>
-          <t>Sassari</t>
-        </is>
-      </c>
-      <c r="D31" s="8" t="inlineStr">
-        <is>
-          <t>info@galleriadautore.it</t>
-        </is>
-      </c>
-      <c r="E31" s="8" t="inlineStr">
+      <c r="A31" s="6" t="inlineStr">
+        <is>
+          <t>A31</t>
+        </is>
+      </c>
+      <c r="B31" s="6" t="inlineStr">
+        <is>
+          <t>Vallebona Immobiliare</t>
+        </is>
+      </c>
+      <c r="C31" s="6" t="inlineStr">
+        <is>
+          <t>Cagliari / Chia / Villasimius</t>
+        </is>
+      </c>
+      <c r="D31" s="6" t="inlineStr">
+        <is>
+          <t>info@vallebonarealestate.it</t>
+        </is>
+      </c>
+      <c r="E31" s="6" t="inlineStr">
         <is>
           <t>Agenzia immobiliare</t>
         </is>
       </c>
-      <c r="F31" s="8" t="inlineStr">
-        <is>
-          <t>3d65f</t>
-        </is>
-      </c>
-      <c r="G31" s="8" t="inlineStr">
-        <is>
-          <t>https://agenzie-immobiliari.rilievocontract.it/?ref=3d65f</t>
+      <c r="F31" s="6" t="inlineStr">
+        <is>
+          <t>6c731</t>
+        </is>
+      </c>
+      <c r="G31" s="6" t="inlineStr">
+        <is>
+          <t>https://agenzie-immobiliari.rilievocontract.it/?ref=6c731</t>
         </is>
       </c>
     </row>
     <row r="32">
-      <c r="A32" s="6" t="inlineStr">
-        <is>
-          <t>A31</t>
-        </is>
-      </c>
-      <c r="B32" s="6" t="inlineStr">
-        <is>
-          <t>Vallebona Immobiliare</t>
-        </is>
-      </c>
-      <c r="C32" s="6" t="inlineStr">
-        <is>
-          <t>Cagliari / Chia / Villasimius</t>
-        </is>
-      </c>
-      <c r="D32" s="6" t="inlineStr">
-        <is>
-          <t>info@vallebonarealestate.it</t>
-        </is>
-      </c>
-      <c r="E32" s="6" t="inlineStr">
+      <c r="A32" s="8" t="inlineStr">
+        <is>
+          <t>A32</t>
+        </is>
+      </c>
+      <c r="B32" s="8" t="inlineStr">
+        <is>
+          <t>L'Immobiliare Sardegna</t>
+        </is>
+      </c>
+      <c r="C32" s="8" t="inlineStr">
+        <is>
+          <t>Alghero (SS)</t>
+        </is>
+      </c>
+      <c r="D32" s="8" t="inlineStr">
+        <is>
+          <t>info@immobiliaresardegna.eu</t>
+        </is>
+      </c>
+      <c r="E32" s="8" t="inlineStr">
         <is>
           <t>Agenzia immobiliare</t>
         </is>
       </c>
-      <c r="F32" s="6" t="inlineStr">
-        <is>
-          <t>6c731</t>
-        </is>
-      </c>
-      <c r="G32" s="6" t="inlineStr">
-        <is>
-          <t>https://agenzie-immobiliari.rilievocontract.it/?ref=6c731</t>
-        </is>
-      </c>
-    </row>
-    <row r="33">
-      <c r="A33" s="8" t="inlineStr">
-        <is>
-          <t>A32</t>
-        </is>
-      </c>
-      <c r="B33" s="8" t="inlineStr">
-        <is>
-          <t>L'Immobiliare Sardegna</t>
-        </is>
-      </c>
-      <c r="C33" s="8" t="inlineStr">
-        <is>
-          <t>Alghero (SS)</t>
-        </is>
-      </c>
-      <c r="D33" s="8" t="inlineStr">
-        <is>
-          <t>info@immobiliaresardegna.eu</t>
-        </is>
-      </c>
-      <c r="E33" s="8" t="inlineStr">
-        <is>
-          <t>Agenzia immobiliare</t>
-        </is>
-      </c>
-      <c r="F33" s="8" t="inlineStr">
+      <c r="F32" s="8" t="inlineStr">
         <is>
           <t>95611</t>
         </is>
       </c>
-      <c r="G33" s="8" t="inlineStr">
+      <c r="G32" s="8" t="inlineStr">
         <is>
           <t>https://agenzie-immobiliari.rilievocontract.it/?ref=95611</t>
         </is>

</xml_diff>